<commit_message>
add version  of the sum_select_12 with input reg in bitonic_merge
</commit_message>
<xml_diff>
--- a/module_library/comp_sum_select.xlsx
+++ b/module_library/comp_sum_select.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\LRMLD\module_library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD9F1144-4C91-42A7-8BC4-0A82590EB4B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C5596CF-D0F5-433F-839E-31C6EE54006A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="19">
   <si>
     <t>Замена метрик на индексы, добавлено насыщение</t>
   </si>
@@ -115,6 +115,9 @@
   </si>
   <si>
     <t>Задержка, такты: 9</t>
+  </si>
+  <si>
+    <t>sum_select_12, + входная регистрация в bitonic_merge</t>
   </si>
 </sst>
 </file>
@@ -474,15 +477,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="D1:V10"/>
+  <dimension ref="D1:Y10"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="7" width="8.88671875" style="1"/>
-    <col min="8" max="22" width="10.77734375" style="1" customWidth="1"/>
-    <col min="23" max="16384" width="8.88671875" style="1"/>
+    <col min="8" max="25" width="10.77734375" style="1" customWidth="1"/>
+    <col min="26" max="27" width="8.88671875" style="1"/>
+    <col min="28" max="28" width="10.77734375" style="1" customWidth="1"/>
+    <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="4:22" x14ac:dyDescent="0.3">
+    <row r="1" spans="4:25" x14ac:dyDescent="0.3">
       <c r="D1" s="3" t="s">
         <v>8</v>
       </c>
@@ -494,7 +499,7 @@
       <c r="H1" s="3"/>
       <c r="I1" s="3"/>
     </row>
-    <row r="3" spans="4:22" x14ac:dyDescent="0.3">
+    <row r="3" spans="4:25" x14ac:dyDescent="0.3">
       <c r="H3" s="3" t="s">
         <v>14</v>
       </c>
@@ -520,8 +525,13 @@
       </c>
       <c r="U3" s="3"/>
       <c r="V3" s="3"/>
+      <c r="W3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="X3" s="3"/>
+      <c r="Y3" s="3"/>
     </row>
-    <row r="4" spans="4:22" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="4:25" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D4" s="3" t="s">
         <v>4</v>
       </c>
@@ -553,8 +563,13 @@
       </c>
       <c r="U4" s="3"/>
       <c r="V4" s="3"/>
+      <c r="W4" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="X4" s="4"/>
+      <c r="Y4" s="4"/>
     </row>
-    <row r="5" spans="4:22" x14ac:dyDescent="0.3">
+    <row r="5" spans="4:25" x14ac:dyDescent="0.3">
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
@@ -574,8 +589,11 @@
       <c r="T5" s="3"/>
       <c r="U5" s="3"/>
       <c r="V5" s="3"/>
+      <c r="W5" s="4"/>
+      <c r="X5" s="4"/>
+      <c r="Y5" s="4"/>
     </row>
-    <row r="6" spans="4:22" x14ac:dyDescent="0.3">
+    <row r="6" spans="4:25" x14ac:dyDescent="0.3">
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
@@ -595,8 +613,11 @@
       <c r="T6" s="3"/>
       <c r="U6" s="3"/>
       <c r="V6" s="3"/>
+      <c r="W6" s="4"/>
+      <c r="X6" s="4"/>
+      <c r="Y6" s="4"/>
     </row>
-    <row r="7" spans="4:22" ht="20.399999999999999" x14ac:dyDescent="0.3">
+    <row r="7" spans="4:25" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="D7" s="3" t="s">
         <v>5</v>
       </c>
@@ -650,8 +671,17 @@
       <c r="V7" s="2" t="s">
         <v>7</v>
       </c>
+      <c r="W7" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="X7" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="Y7" s="2" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="8" spans="4:22" x14ac:dyDescent="0.3">
+    <row r="8" spans="4:25" x14ac:dyDescent="0.3">
       <c r="D8" s="3">
         <v>8</v>
       </c>
@@ -705,8 +735,17 @@
       <c r="V8" s="2">
         <v>246</v>
       </c>
+      <c r="W8" s="2">
+        <v>3968</v>
+      </c>
+      <c r="X8" s="2">
+        <v>3734</v>
+      </c>
+      <c r="Y8" s="2">
+        <v>297</v>
+      </c>
     </row>
-    <row r="9" spans="4:22" x14ac:dyDescent="0.3">
+    <row r="9" spans="4:25" x14ac:dyDescent="0.3">
       <c r="D9" s="3">
         <v>10</v>
       </c>
@@ -752,16 +791,25 @@
         <v>301</v>
       </c>
       <c r="T9" s="2">
-        <v>8531</v>
+        <v>5511</v>
       </c>
       <c r="U9" s="2">
-        <v>6519</v>
+        <v>5209</v>
       </c>
       <c r="V9" s="2">
-        <v>301</v>
+        <v>242</v>
+      </c>
+      <c r="W9" s="2">
+        <v>5807</v>
+      </c>
+      <c r="X9" s="2">
+        <v>5764</v>
+      </c>
+      <c r="Y9" s="2">
+        <v>291</v>
       </c>
     </row>
-    <row r="10" spans="4:22" x14ac:dyDescent="0.3">
+    <row r="10" spans="4:25" x14ac:dyDescent="0.3">
       <c r="D10" s="3">
         <v>10</v>
       </c>
@@ -807,17 +855,28 @@
         <v>276</v>
       </c>
       <c r="T10" s="2">
-        <v>12897</v>
+        <v>8367</v>
       </c>
       <c r="U10" s="2">
-        <v>10161</v>
+        <v>8997</v>
       </c>
       <c r="V10" s="2">
-        <v>276</v>
+        <v>231</v>
+      </c>
+      <c r="W10" s="2">
+        <v>9107</v>
+      </c>
+      <c r="X10" s="2">
+        <v>8871</v>
+      </c>
+      <c r="Y10" s="2">
+        <v>296</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="21">
+  <mergeCells count="23">
+    <mergeCell ref="W3:Y3"/>
+    <mergeCell ref="W4:Y6"/>
     <mergeCell ref="T4:V6"/>
     <mergeCell ref="Q3:S3"/>
     <mergeCell ref="T3:V3"/>

</xml_diff>

<commit_message>
add sum_select8 (input list's size = 8, opposite to sum_select_8, mistake in labeling)
</commit_message>
<xml_diff>
--- a/module_library/comp_sum_select.xlsx
+++ b/module_library/comp_sum_select.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\LRMLD\module_library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B6FC0C4-14C2-4782-8C21-611AF9D0D6BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4214EA95-264A-4986-8654-9E1452393D94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="26">
   <si>
     <t>LUT</t>
   </si>
@@ -128,12 +128,24 @@
   <si>
     <t>sum_select_4 - замена метрик на индексы, добавлено насыщение</t>
   </si>
+  <si>
+    <t>Задержка, такты: 7</t>
+  </si>
+  <si>
+    <t>sum_select8</t>
+  </si>
+  <si>
+    <t>Базовые блоки</t>
+  </si>
+  <si>
+    <t>↑</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -156,6 +168,13 @@
       <family val="1"/>
       <charset val="204"/>
     </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -165,7 +184,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="38">
+  <borders count="39">
     <border>
       <left/>
       <right/>
@@ -668,11 +687,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FFC00000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -680,151 +708,148 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1107,212 +1132,216 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="D1:AE17"/>
+  <dimension ref="D1:AE15"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="7" width="8.88671875" style="1"/>
     <col min="8" max="25" width="10.77734375" style="1" customWidth="1"/>
     <col min="26" max="27" width="8.88671875" style="1"/>
-    <col min="28" max="28" width="10.77734375" style="1" customWidth="1"/>
-    <col min="29" max="16384" width="8.88671875" style="1"/>
+    <col min="28" max="31" width="10.77734375" style="1" customWidth="1"/>
+    <col min="32" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3" t="s">
+      <c r="E1" s="31"/>
+      <c r="F1" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="3"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
     </row>
     <row r="2" spans="4:31" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="3" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="H3" s="38" t="s">
+      <c r="H3" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="I3" s="39"/>
-      <c r="J3" s="39"/>
-      <c r="K3" s="39" t="s">
+      <c r="I3" s="38"/>
+      <c r="J3" s="38"/>
+      <c r="K3" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="L3" s="39"/>
-      <c r="M3" s="39"/>
-      <c r="N3" s="40" t="s">
+      <c r="L3" s="38"/>
+      <c r="M3" s="38"/>
+      <c r="N3" s="35" t="s">
         <v>14</v>
       </c>
-      <c r="O3" s="41"/>
-      <c r="P3" s="42"/>
-      <c r="Q3" s="36" t="s">
+      <c r="O3" s="36"/>
+      <c r="P3" s="37"/>
+      <c r="Q3" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="R3" s="17"/>
-      <c r="S3" s="17"/>
-      <c r="T3" s="17" t="s">
+      <c r="R3" s="33"/>
+      <c r="S3" s="33"/>
+      <c r="T3" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="U3" s="17"/>
-      <c r="V3" s="30"/>
-      <c r="W3" s="16" t="s">
+      <c r="U3" s="33"/>
+      <c r="V3" s="39"/>
+      <c r="W3" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="X3" s="17"/>
-      <c r="Y3" s="17"/>
-      <c r="Z3" s="18" t="s">
+      <c r="X3" s="33"/>
+      <c r="Y3" s="33"/>
+      <c r="Z3" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="AA3" s="19"/>
-      <c r="AB3" s="20"/>
-      <c r="AC3" s="5"/>
-      <c r="AD3" s="5"/>
-      <c r="AE3" s="5"/>
+      <c r="AA3" s="20"/>
+      <c r="AB3" s="21"/>
+      <c r="AC3" s="19" t="s">
+        <v>22</v>
+      </c>
+      <c r="AD3" s="20"/>
+      <c r="AE3" s="21"/>
     </row>
     <row r="4" spans="4:31" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="12"/>
-      <c r="H4" s="43" t="s">
+      <c r="E4" s="31"/>
+      <c r="F4" s="31"/>
+      <c r="G4" s="43"/>
+      <c r="H4" s="47" t="s">
         <v>20</v>
       </c>
-      <c r="I4" s="34"/>
-      <c r="J4" s="34"/>
-      <c r="K4" s="34" t="s">
+      <c r="I4" s="44"/>
+      <c r="J4" s="44"/>
+      <c r="K4" s="44" t="s">
         <v>21</v>
       </c>
-      <c r="L4" s="34"/>
-      <c r="M4" s="34"/>
-      <c r="N4" s="32" t="s">
+      <c r="L4" s="44"/>
+      <c r="M4" s="44"/>
+      <c r="N4" s="45" t="s">
         <v>9</v>
       </c>
-      <c r="O4" s="4"/>
-      <c r="P4" s="44"/>
-      <c r="Q4" s="13" t="s">
+      <c r="O4" s="40"/>
+      <c r="P4" s="46"/>
+      <c r="Q4" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="R4" s="3"/>
-      <c r="S4" s="3"/>
-      <c r="T4" s="4" t="s">
+      <c r="R4" s="31"/>
+      <c r="S4" s="31"/>
+      <c r="T4" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="U4" s="4"/>
-      <c r="V4" s="31"/>
-      <c r="W4" s="21" t="s">
+      <c r="U4" s="40"/>
+      <c r="V4" s="41"/>
+      <c r="W4" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="X4" s="3"/>
-      <c r="Y4" s="3"/>
-      <c r="Z4" s="6" t="s">
+      <c r="X4" s="31"/>
+      <c r="Y4" s="31"/>
+      <c r="Z4" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="AA4" s="7"/>
-      <c r="AB4" s="22"/>
-      <c r="AC4" s="5"/>
-      <c r="AD4" s="5"/>
-      <c r="AE4" s="5"/>
+      <c r="AA4" s="23"/>
+      <c r="AB4" s="24"/>
+      <c r="AC4" s="22" t="s">
+        <v>23</v>
+      </c>
+      <c r="AD4" s="23"/>
+      <c r="AE4" s="24"/>
     </row>
     <row r="5" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="12"/>
-      <c r="H5" s="43"/>
-      <c r="I5" s="34"/>
-      <c r="J5" s="34"/>
-      <c r="K5" s="34"/>
-      <c r="L5" s="34"/>
-      <c r="M5" s="34"/>
-      <c r="N5" s="32"/>
-      <c r="O5" s="4"/>
-      <c r="P5" s="44"/>
-      <c r="Q5" s="13"/>
-      <c r="R5" s="3"/>
-      <c r="S5" s="3"/>
-      <c r="T5" s="4"/>
-      <c r="U5" s="4"/>
-      <c r="V5" s="31"/>
-      <c r="W5" s="21"/>
-      <c r="X5" s="3"/>
-      <c r="Y5" s="3"/>
-      <c r="Z5" s="8"/>
-      <c r="AA5" s="9"/>
-      <c r="AB5" s="23"/>
-      <c r="AC5" s="5"/>
-      <c r="AD5" s="5"/>
-      <c r="AE5" s="5"/>
+      <c r="D5" s="31"/>
+      <c r="E5" s="31"/>
+      <c r="F5" s="31"/>
+      <c r="G5" s="43"/>
+      <c r="H5" s="47"/>
+      <c r="I5" s="44"/>
+      <c r="J5" s="44"/>
+      <c r="K5" s="44"/>
+      <c r="L5" s="44"/>
+      <c r="M5" s="44"/>
+      <c r="N5" s="45"/>
+      <c r="O5" s="40"/>
+      <c r="P5" s="46"/>
+      <c r="Q5" s="42"/>
+      <c r="R5" s="31"/>
+      <c r="S5" s="31"/>
+      <c r="T5" s="40"/>
+      <c r="U5" s="40"/>
+      <c r="V5" s="41"/>
+      <c r="W5" s="30"/>
+      <c r="X5" s="31"/>
+      <c r="Y5" s="31"/>
+      <c r="Z5" s="25"/>
+      <c r="AA5" s="18"/>
+      <c r="AB5" s="26"/>
+      <c r="AC5" s="25"/>
+      <c r="AD5" s="18"/>
+      <c r="AE5" s="26"/>
     </row>
     <row r="6" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="12"/>
-      <c r="H6" s="43"/>
-      <c r="I6" s="34"/>
-      <c r="J6" s="34"/>
-      <c r="K6" s="34"/>
-      <c r="L6" s="34"/>
-      <c r="M6" s="34"/>
-      <c r="N6" s="32"/>
-      <c r="O6" s="4"/>
-      <c r="P6" s="44"/>
-      <c r="Q6" s="13"/>
-      <c r="R6" s="3"/>
-      <c r="S6" s="3"/>
-      <c r="T6" s="4"/>
-      <c r="U6" s="4"/>
-      <c r="V6" s="31"/>
-      <c r="W6" s="21"/>
-      <c r="X6" s="3"/>
-      <c r="Y6" s="3"/>
-      <c r="Z6" s="10"/>
-      <c r="AA6" s="11"/>
-      <c r="AB6" s="24"/>
-      <c r="AC6" s="5"/>
-      <c r="AD6" s="5"/>
-      <c r="AE6" s="5"/>
+      <c r="D6" s="31"/>
+      <c r="E6" s="31"/>
+      <c r="F6" s="31"/>
+      <c r="G6" s="43"/>
+      <c r="H6" s="47"/>
+      <c r="I6" s="44"/>
+      <c r="J6" s="44"/>
+      <c r="K6" s="44"/>
+      <c r="L6" s="44"/>
+      <c r="M6" s="44"/>
+      <c r="N6" s="45"/>
+      <c r="O6" s="40"/>
+      <c r="P6" s="46"/>
+      <c r="Q6" s="42"/>
+      <c r="R6" s="31"/>
+      <c r="S6" s="31"/>
+      <c r="T6" s="40"/>
+      <c r="U6" s="40"/>
+      <c r="V6" s="41"/>
+      <c r="W6" s="30"/>
+      <c r="X6" s="31"/>
+      <c r="Y6" s="31"/>
+      <c r="Z6" s="27"/>
+      <c r="AA6" s="28"/>
+      <c r="AB6" s="29"/>
+      <c r="AC6" s="27"/>
+      <c r="AD6" s="28"/>
+      <c r="AE6" s="29"/>
     </row>
     <row r="7" spans="4:31" ht="20.399999999999999" x14ac:dyDescent="0.3">
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3" t="s">
+      <c r="E7" s="31"/>
+      <c r="F7" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="G7" s="12"/>
-      <c r="H7" s="45" t="s">
+      <c r="G7" s="43"/>
+      <c r="H7" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="I7" s="35" t="s">
+      <c r="I7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="J7" s="35" t="s">
+      <c r="J7" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="K7" s="35" t="s">
+      <c r="K7" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="L7" s="35" t="s">
+      <c r="L7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="M7" s="35" t="s">
+      <c r="M7" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="N7" s="14" t="s">
+      <c r="N7" s="3" t="s">
         <v>0</v>
       </c>
       <c r="O7" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="P7" s="46" t="s">
+      <c r="P7" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="Q7" s="14" t="s">
+      <c r="Q7" s="3" t="s">
         <v>0</v>
       </c>
       <c r="R7" s="2" t="s">
@@ -1327,10 +1356,10 @@
       <c r="U7" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="V7" s="26" t="s">
+      <c r="V7" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="W7" s="25" t="s">
+      <c r="W7" s="4" t="s">
         <v>0</v>
       </c>
       <c r="X7" s="2" t="s">
@@ -1345,47 +1374,56 @@
       <c r="AA7" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="AB7" s="26" t="s">
+      <c r="AB7" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="AC7" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AD7" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AE7" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="8" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="D8" s="3">
+      <c r="D8" s="31">
         <v>8</v>
       </c>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3">
+      <c r="E8" s="31"/>
+      <c r="F8" s="31">
         <v>8</v>
       </c>
-      <c r="G8" s="12"/>
-      <c r="H8" s="45">
+      <c r="G8" s="43"/>
+      <c r="H8" s="11">
         <v>331</v>
       </c>
-      <c r="I8" s="35">
+      <c r="I8" s="9">
         <v>306</v>
       </c>
-      <c r="J8" s="35">
+      <c r="J8" s="9">
         <v>321</v>
       </c>
-      <c r="K8" s="35">
+      <c r="K8" s="9">
         <v>374</v>
       </c>
-      <c r="L8" s="35">
+      <c r="L8" s="9">
         <v>254</v>
       </c>
-      <c r="M8" s="35">
+      <c r="M8" s="9">
         <v>332</v>
       </c>
-      <c r="N8" s="14">
+      <c r="N8" s="3">
         <v>868</v>
       </c>
       <c r="O8" s="2">
         <v>541</v>
       </c>
-      <c r="P8" s="46">
+      <c r="P8" s="12">
         <v>382</v>
       </c>
-      <c r="Q8" s="14">
+      <c r="Q8" s="3">
         <v>6641</v>
       </c>
       <c r="R8" s="2">
@@ -1400,10 +1438,10 @@
       <c r="U8" s="2">
         <v>5523</v>
       </c>
-      <c r="V8" s="26">
+      <c r="V8" s="5">
         <v>294</v>
       </c>
-      <c r="W8" s="25">
+      <c r="W8" s="4">
         <v>3800</v>
       </c>
       <c r="X8" s="2">
@@ -1418,47 +1456,56 @@
       <c r="AA8" s="2">
         <v>3734</v>
       </c>
-      <c r="AB8" s="26">
+      <c r="AB8" s="5">
         <v>297</v>
+      </c>
+      <c r="AC8" s="2">
+        <v>763</v>
+      </c>
+      <c r="AD8" s="2">
+        <v>624</v>
+      </c>
+      <c r="AE8" s="5">
+        <v>368</v>
       </c>
     </row>
     <row r="9" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="D9" s="3">
+      <c r="D9" s="31">
         <v>10</v>
       </c>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3">
+      <c r="E9" s="31"/>
+      <c r="F9" s="31">
         <v>16</v>
       </c>
-      <c r="G9" s="12"/>
-      <c r="H9" s="45">
+      <c r="G9" s="43"/>
+      <c r="H9" s="11">
         <v>504</v>
       </c>
-      <c r="I9" s="35">
+      <c r="I9" s="9">
         <v>507</v>
       </c>
-      <c r="J9" s="35">
+      <c r="J9" s="9">
         <v>305</v>
       </c>
-      <c r="K9" s="35">
+      <c r="K9" s="9">
         <v>522</v>
       </c>
-      <c r="L9" s="35">
+      <c r="L9" s="9">
         <v>395</v>
       </c>
-      <c r="M9" s="35">
+      <c r="M9" s="9">
         <v>326</v>
       </c>
-      <c r="N9" s="14">
+      <c r="N9" s="3">
         <v>1052</v>
       </c>
       <c r="O9" s="2">
         <v>702</v>
       </c>
-      <c r="P9" s="46">
+      <c r="P9" s="12">
         <v>372</v>
       </c>
-      <c r="Q9" s="14">
+      <c r="Q9" s="3">
         <v>10250</v>
       </c>
       <c r="R9" s="2">
@@ -1473,10 +1520,10 @@
       <c r="U9" s="2">
         <v>8570</v>
       </c>
-      <c r="V9" s="26">
+      <c r="V9" s="5">
         <v>271</v>
       </c>
-      <c r="W9" s="25">
+      <c r="W9" s="4">
         <v>5511</v>
       </c>
       <c r="X9" s="2">
@@ -1491,117 +1538,144 @@
       <c r="AA9" s="2">
         <v>5764</v>
       </c>
-      <c r="AB9" s="26">
+      <c r="AB9" s="5">
         <v>291</v>
+      </c>
+      <c r="AC9" s="2">
+        <v>1231</v>
+      </c>
+      <c r="AD9" s="2">
+        <v>1023</v>
+      </c>
+      <c r="AE9" s="5">
+        <v>356</v>
       </c>
     </row>
     <row r="10" spans="4:31" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D10" s="3">
+      <c r="D10" s="31">
         <v>10</v>
       </c>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3">
+      <c r="E10" s="31"/>
+      <c r="F10" s="31">
         <v>32</v>
       </c>
-      <c r="G10" s="12"/>
-      <c r="H10" s="47">
+      <c r="G10" s="43"/>
+      <c r="H10" s="13">
         <v>761</v>
       </c>
-      <c r="I10" s="48">
+      <c r="I10" s="14">
         <v>864</v>
       </c>
-      <c r="J10" s="48">
+      <c r="J10" s="14">
         <v>300</v>
       </c>
-      <c r="K10" s="48">
+      <c r="K10" s="14">
         <v>776</v>
       </c>
-      <c r="L10" s="48">
+      <c r="L10" s="14">
         <v>616</v>
       </c>
-      <c r="M10" s="48">
+      <c r="M10" s="14">
         <v>308</v>
       </c>
-      <c r="N10" s="49">
+      <c r="N10" s="15">
         <v>1709</v>
       </c>
-      <c r="O10" s="50">
+      <c r="O10" s="16">
         <v>830</v>
       </c>
-      <c r="P10" s="51">
+      <c r="P10" s="17">
         <v>363</v>
       </c>
-      <c r="Q10" s="37">
+      <c r="Q10" s="10">
         <v>15069</v>
       </c>
-      <c r="R10" s="28">
+      <c r="R10" s="7">
         <v>14526</v>
       </c>
-      <c r="S10" s="28">
+      <c r="S10" s="7">
         <v>278</v>
       </c>
-      <c r="T10" s="28">
+      <c r="T10" s="7">
         <v>15837</v>
       </c>
-      <c r="U10" s="28">
+      <c r="U10" s="7">
         <v>14265</v>
       </c>
-      <c r="V10" s="29">
+      <c r="V10" s="8">
         <v>276</v>
       </c>
-      <c r="W10" s="27">
+      <c r="W10" s="6">
         <v>8367</v>
       </c>
-      <c r="X10" s="28">
+      <c r="X10" s="7">
         <v>8997</v>
       </c>
-      <c r="Y10" s="28">
+      <c r="Y10" s="7">
         <v>231</v>
       </c>
-      <c r="Z10" s="28">
+      <c r="Z10" s="7">
         <v>9107</v>
       </c>
-      <c r="AA10" s="28">
+      <c r="AA10" s="7">
         <v>8871</v>
       </c>
-      <c r="AB10" s="29">
+      <c r="AB10" s="8">
         <v>296</v>
+      </c>
+      <c r="AC10" s="7">
+        <v>1857</v>
+      </c>
+      <c r="AD10" s="7">
+        <v>8871</v>
+      </c>
+      <c r="AE10" s="8">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="11" spans="4:31" x14ac:dyDescent="0.3">
+      <c r="H11" s="49" t="s">
+        <v>24</v>
+      </c>
+      <c r="I11" s="49"/>
+      <c r="J11" s="49"/>
+      <c r="K11" s="49"/>
+      <c r="L11" s="49"/>
+      <c r="M11" s="49"/>
+      <c r="N11" s="49"/>
+      <c r="O11" s="49"/>
+      <c r="P11" s="49"/>
+    </row>
+    <row r="12" spans="4:31" ht="23.4" x14ac:dyDescent="0.3">
+      <c r="O12" s="50" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="13" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="N13" s="33" t="s">
+      <c r="N13" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="O13" s="33"/>
-      <c r="P13" s="33"/>
+      <c r="O13" s="18"/>
+      <c r="P13" s="18"/>
     </row>
     <row r="14" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="N14" s="33"/>
-      <c r="O14" s="33"/>
-      <c r="P14" s="33"/>
+      <c r="N14" s="18"/>
+      <c r="O14" s="18"/>
+      <c r="P14" s="18"/>
     </row>
     <row r="15" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="N15" s="33"/>
-      <c r="O15" s="33"/>
-      <c r="P15" s="33"/>
-    </row>
-    <row r="16" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="I16" s="15"/>
-    </row>
-    <row r="17" spans="9:9" x14ac:dyDescent="0.3">
-      <c r="I17" s="15"/>
+      <c r="N15" s="18"/>
+      <c r="O15" s="18"/>
+      <c r="P15" s="18"/>
     </row>
   </sheetData>
-  <mergeCells count="28">
-    <mergeCell ref="N13:P15"/>
-    <mergeCell ref="AC3:AE3"/>
-    <mergeCell ref="AC4:AE6"/>
-    <mergeCell ref="Z3:AB3"/>
-    <mergeCell ref="Z4:AB6"/>
-    <mergeCell ref="W4:Y6"/>
-    <mergeCell ref="Q3:S3"/>
-    <mergeCell ref="W3:Y3"/>
-    <mergeCell ref="N3:P3"/>
+  <mergeCells count="29">
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="F1:I1"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="H4:J6"/>
+    <mergeCell ref="H3:J3"/>
     <mergeCell ref="K3:M3"/>
     <mergeCell ref="T3:V3"/>
     <mergeCell ref="T4:V6"/>
@@ -1615,12 +1689,16 @@
     <mergeCell ref="D8:E8"/>
     <mergeCell ref="K4:M6"/>
     <mergeCell ref="N4:P6"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="F1:I1"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="H4:J6"/>
-    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="N13:P15"/>
+    <mergeCell ref="AC3:AE3"/>
+    <mergeCell ref="AC4:AE6"/>
+    <mergeCell ref="Z3:AB3"/>
+    <mergeCell ref="Z4:AB6"/>
+    <mergeCell ref="W4:Y6"/>
+    <mergeCell ref="Q3:S3"/>
+    <mergeCell ref="W3:Y3"/>
+    <mergeCell ref="N3:P3"/>
+    <mergeCell ref="H11:P11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
done top_comb and modify table of comparasions
</commit_message>
<xml_diff>
--- a/module_library/comp_sum_select.xlsx
+++ b/module_library/comp_sum_select.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\LRMLD\module_library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DED6FCC-3D99-401D-ADBC-B1D13755D4CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06C9BDA5-2C13-4385-A252-985703916597}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="51">
   <si>
     <t>LUT</t>
   </si>
@@ -226,6 +226,17 @@
  L_W = 16
 IS_FSM = 1
 Latency + N_U cycles</t>
+  </si>
+  <si>
+    <t>Reduce resources</t>
+  </si>
+  <si>
+    <t>top_comb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M_W = 10
+ L_W = 32
+</t>
   </si>
 </sst>
 </file>
@@ -279,7 +290,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="47">
+  <borders count="58">
     <border>
       <left/>
       <right/>
@@ -883,11 +894,160 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -958,149 +1118,200 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1382,188 +1593,188 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="D1:AJ45"/>
+  <dimension ref="D1:AJ64"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="7" width="8.88671875" style="1"/>
     <col min="8" max="25" width="10.77734375" style="1" customWidth="1"/>
-    <col min="26" max="27" width="8.88671875" style="1"/>
+    <col min="26" max="27" width="12.5546875" style="1" bestFit="1" customWidth="1"/>
     <col min="28" max="35" width="10.77734375" style="1" customWidth="1"/>
     <col min="36" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="D1" s="25" t="s">
+      <c r="D1" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25" t="s">
-        <v>8</v>
-      </c>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="25"/>
+      <c r="E1" s="53"/>
+      <c r="F1" s="53" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" s="53"/>
+      <c r="H1" s="53"/>
+      <c r="I1" s="53"/>
     </row>
     <row r="2" spans="4:31" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="3" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="H3" s="29" t="s">
+      <c r="H3" s="71" t="s">
         <v>12</v>
       </c>
-      <c r="I3" s="30"/>
-      <c r="J3" s="30"/>
-      <c r="K3" s="30" t="s">
+      <c r="I3" s="48"/>
+      <c r="J3" s="48"/>
+      <c r="K3" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="L3" s="30"/>
-      <c r="M3" s="30"/>
-      <c r="N3" s="47" t="s">
+      <c r="L3" s="48"/>
+      <c r="M3" s="48"/>
+      <c r="N3" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="O3" s="48"/>
-      <c r="P3" s="49"/>
-      <c r="Q3" s="44" t="s">
+      <c r="O3" s="45"/>
+      <c r="P3" s="46"/>
+      <c r="Q3" s="41" t="s">
         <v>13</v>
       </c>
-      <c r="R3" s="45"/>
-      <c r="S3" s="45"/>
-      <c r="T3" s="45" t="s">
+      <c r="R3" s="42"/>
+      <c r="S3" s="42"/>
+      <c r="T3" s="42" t="s">
         <v>17</v>
       </c>
-      <c r="U3" s="45"/>
-      <c r="V3" s="51"/>
-      <c r="W3" s="46" t="s">
+      <c r="U3" s="42"/>
+      <c r="V3" s="49"/>
+      <c r="W3" s="43" t="s">
         <v>15</v>
       </c>
-      <c r="X3" s="45"/>
-      <c r="Y3" s="45"/>
-      <c r="Z3" s="32" t="s">
+      <c r="X3" s="42"/>
+      <c r="Y3" s="42"/>
+      <c r="Z3" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="AA3" s="33"/>
-      <c r="AB3" s="34"/>
-      <c r="AC3" s="32" t="s">
+      <c r="AA3" s="58"/>
+      <c r="AB3" s="59"/>
+      <c r="AC3" s="57" t="s">
         <v>22</v>
       </c>
-      <c r="AD3" s="33"/>
-      <c r="AE3" s="34"/>
+      <c r="AD3" s="58"/>
+      <c r="AE3" s="59"/>
     </row>
     <row r="4" spans="4:31" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D4" s="25" t="s">
+      <c r="D4" s="53" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="25"/>
-      <c r="F4" s="25"/>
-      <c r="G4" s="26"/>
-      <c r="H4" s="27" t="s">
+      <c r="E4" s="53"/>
+      <c r="F4" s="53"/>
+      <c r="G4" s="69"/>
+      <c r="H4" s="70" t="s">
         <v>20</v>
       </c>
-      <c r="I4" s="28"/>
-      <c r="J4" s="28"/>
-      <c r="K4" s="28" t="s">
+      <c r="I4" s="54"/>
+      <c r="J4" s="54"/>
+      <c r="K4" s="54" t="s">
         <v>21</v>
       </c>
-      <c r="L4" s="28"/>
-      <c r="M4" s="28"/>
-      <c r="N4" s="54" t="s">
+      <c r="L4" s="54"/>
+      <c r="M4" s="54"/>
+      <c r="N4" s="55" t="s">
         <v>9</v>
       </c>
-      <c r="O4" s="24"/>
-      <c r="P4" s="55"/>
-      <c r="Q4" s="53" t="s">
+      <c r="O4" s="50"/>
+      <c r="P4" s="56"/>
+      <c r="Q4" s="52" t="s">
         <v>10</v>
       </c>
-      <c r="R4" s="25"/>
-      <c r="S4" s="25"/>
-      <c r="T4" s="24" t="s">
+      <c r="R4" s="53"/>
+      <c r="S4" s="53"/>
+      <c r="T4" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="U4" s="24"/>
-      <c r="V4" s="52"/>
-      <c r="W4" s="43" t="s">
+      <c r="U4" s="50"/>
+      <c r="V4" s="51"/>
+      <c r="W4" s="68" t="s">
         <v>11</v>
       </c>
-      <c r="X4" s="25"/>
-      <c r="Y4" s="25"/>
-      <c r="Z4" s="35" t="s">
+      <c r="X4" s="53"/>
+      <c r="Y4" s="53"/>
+      <c r="Z4" s="60" t="s">
         <v>16</v>
       </c>
-      <c r="AA4" s="36"/>
-      <c r="AB4" s="37"/>
-      <c r="AC4" s="35" t="s">
+      <c r="AA4" s="61"/>
+      <c r="AB4" s="62"/>
+      <c r="AC4" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="AD4" s="36"/>
-      <c r="AE4" s="37"/>
+      <c r="AD4" s="61"/>
+      <c r="AE4" s="62"/>
     </row>
     <row r="5" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="D5" s="25"/>
-      <c r="E5" s="25"/>
-      <c r="F5" s="25"/>
-      <c r="G5" s="26"/>
-      <c r="H5" s="27"/>
-      <c r="I5" s="28"/>
-      <c r="J5" s="28"/>
-      <c r="K5" s="28"/>
-      <c r="L5" s="28"/>
-      <c r="M5" s="28"/>
-      <c r="N5" s="54"/>
-      <c r="O5" s="24"/>
-      <c r="P5" s="55"/>
-      <c r="Q5" s="53"/>
-      <c r="R5" s="25"/>
-      <c r="S5" s="25"/>
-      <c r="T5" s="24"/>
-      <c r="U5" s="24"/>
-      <c r="V5" s="52"/>
-      <c r="W5" s="43"/>
-      <c r="X5" s="25"/>
-      <c r="Y5" s="25"/>
-      <c r="Z5" s="38"/>
-      <c r="AA5" s="31"/>
-      <c r="AB5" s="39"/>
-      <c r="AC5" s="38"/>
-      <c r="AD5" s="31"/>
-      <c r="AE5" s="39"/>
+      <c r="D5" s="53"/>
+      <c r="E5" s="53"/>
+      <c r="F5" s="53"/>
+      <c r="G5" s="69"/>
+      <c r="H5" s="70"/>
+      <c r="I5" s="54"/>
+      <c r="J5" s="54"/>
+      <c r="K5" s="54"/>
+      <c r="L5" s="54"/>
+      <c r="M5" s="54"/>
+      <c r="N5" s="55"/>
+      <c r="O5" s="50"/>
+      <c r="P5" s="56"/>
+      <c r="Q5" s="52"/>
+      <c r="R5" s="53"/>
+      <c r="S5" s="53"/>
+      <c r="T5" s="50"/>
+      <c r="U5" s="50"/>
+      <c r="V5" s="51"/>
+      <c r="W5" s="68"/>
+      <c r="X5" s="53"/>
+      <c r="Y5" s="53"/>
+      <c r="Z5" s="63"/>
+      <c r="AA5" s="64"/>
+      <c r="AB5" s="27"/>
+      <c r="AC5" s="63"/>
+      <c r="AD5" s="64"/>
+      <c r="AE5" s="27"/>
     </row>
     <row r="6" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="D6" s="25"/>
-      <c r="E6" s="25"/>
-      <c r="F6" s="25"/>
-      <c r="G6" s="26"/>
-      <c r="H6" s="27"/>
-      <c r="I6" s="28"/>
-      <c r="J6" s="28"/>
-      <c r="K6" s="28"/>
-      <c r="L6" s="28"/>
-      <c r="M6" s="28"/>
-      <c r="N6" s="54"/>
-      <c r="O6" s="24"/>
-      <c r="P6" s="55"/>
-      <c r="Q6" s="53"/>
-      <c r="R6" s="25"/>
-      <c r="S6" s="25"/>
-      <c r="T6" s="24"/>
-      <c r="U6" s="24"/>
-      <c r="V6" s="52"/>
-      <c r="W6" s="43"/>
-      <c r="X6" s="25"/>
-      <c r="Y6" s="25"/>
-      <c r="Z6" s="40"/>
-      <c r="AA6" s="41"/>
-      <c r="AB6" s="42"/>
-      <c r="AC6" s="40"/>
-      <c r="AD6" s="41"/>
-      <c r="AE6" s="42"/>
+      <c r="D6" s="53"/>
+      <c r="E6" s="53"/>
+      <c r="F6" s="53"/>
+      <c r="G6" s="69"/>
+      <c r="H6" s="70"/>
+      <c r="I6" s="54"/>
+      <c r="J6" s="54"/>
+      <c r="K6" s="54"/>
+      <c r="L6" s="54"/>
+      <c r="M6" s="54"/>
+      <c r="N6" s="55"/>
+      <c r="O6" s="50"/>
+      <c r="P6" s="56"/>
+      <c r="Q6" s="52"/>
+      <c r="R6" s="53"/>
+      <c r="S6" s="53"/>
+      <c r="T6" s="50"/>
+      <c r="U6" s="50"/>
+      <c r="V6" s="51"/>
+      <c r="W6" s="68"/>
+      <c r="X6" s="53"/>
+      <c r="Y6" s="53"/>
+      <c r="Z6" s="65"/>
+      <c r="AA6" s="66"/>
+      <c r="AB6" s="67"/>
+      <c r="AC6" s="65"/>
+      <c r="AD6" s="66"/>
+      <c r="AE6" s="67"/>
     </row>
     <row r="7" spans="4:31" ht="20.399999999999999" x14ac:dyDescent="0.3">
-      <c r="D7" s="25" t="s">
-        <v>4</v>
-      </c>
-      <c r="E7" s="25"/>
-      <c r="F7" s="25" t="s">
+      <c r="D7" s="53" t="s">
+        <v>4</v>
+      </c>
+      <c r="E7" s="53"/>
+      <c r="F7" s="53" t="s">
         <v>5</v>
       </c>
-      <c r="G7" s="26"/>
+      <c r="G7" s="69"/>
       <c r="H7" s="11" t="s">
         <v>0</v>
       </c>
@@ -1638,14 +1849,14 @@
       </c>
     </row>
     <row r="8" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="D8" s="25">
-        <v>8</v>
-      </c>
-      <c r="E8" s="25"/>
-      <c r="F8" s="25">
-        <v>8</v>
-      </c>
-      <c r="G8" s="26"/>
+      <c r="D8" s="53">
+        <v>8</v>
+      </c>
+      <c r="E8" s="53"/>
+      <c r="F8" s="53">
+        <v>8</v>
+      </c>
+      <c r="G8" s="69"/>
       <c r="H8" s="11">
         <v>331</v>
       </c>
@@ -1720,14 +1931,14 @@
       </c>
     </row>
     <row r="9" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="D9" s="25">
+      <c r="D9" s="53">
         <v>10</v>
       </c>
-      <c r="E9" s="25"/>
-      <c r="F9" s="25">
+      <c r="E9" s="53"/>
+      <c r="F9" s="53">
         <v>16</v>
       </c>
-      <c r="G9" s="26"/>
+      <c r="G9" s="69"/>
       <c r="H9" s="11">
         <v>504</v>
       </c>
@@ -1802,14 +2013,14 @@
       </c>
     </row>
     <row r="10" spans="4:31" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D10" s="25">
+      <c r="D10" s="53">
         <v>10</v>
       </c>
-      <c r="E10" s="25"/>
-      <c r="F10" s="25">
+      <c r="E10" s="53"/>
+      <c r="F10" s="53">
         <v>32</v>
       </c>
-      <c r="G10" s="26"/>
+      <c r="G10" s="69"/>
       <c r="H10" s="13">
         <v>761</v>
       </c>
@@ -1884,17 +2095,17 @@
       </c>
     </row>
     <row r="11" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="H11" s="50" t="s">
+      <c r="H11" s="47" t="s">
         <v>24</v>
       </c>
-      <c r="I11" s="50"/>
-      <c r="J11" s="50"/>
-      <c r="K11" s="50"/>
-      <c r="L11" s="50"/>
-      <c r="M11" s="50"/>
-      <c r="N11" s="50"/>
-      <c r="O11" s="50"/>
-      <c r="P11" s="50"/>
+      <c r="I11" s="47"/>
+      <c r="J11" s="47"/>
+      <c r="K11" s="47"/>
+      <c r="L11" s="47"/>
+      <c r="M11" s="47"/>
+      <c r="N11" s="47"/>
+      <c r="O11" s="47"/>
+      <c r="P11" s="47"/>
     </row>
     <row r="12" spans="4:31" ht="23.4" x14ac:dyDescent="0.3">
       <c r="O12" s="19" t="s">
@@ -1902,103 +2113,103 @@
       </c>
     </row>
     <row r="13" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="N13" s="31" t="s">
+      <c r="N13" s="64" t="s">
         <v>19</v>
       </c>
-      <c r="O13" s="31"/>
-      <c r="P13" s="31"/>
+      <c r="O13" s="64"/>
+      <c r="P13" s="64"/>
     </row>
     <row r="14" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="N14" s="31"/>
-      <c r="O14" s="31"/>
-      <c r="P14" s="31"/>
+      <c r="N14" s="64"/>
+      <c r="O14" s="64"/>
+      <c r="P14" s="64"/>
     </row>
     <row r="15" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="N15" s="31"/>
-      <c r="O15" s="31"/>
-      <c r="P15" s="31"/>
+      <c r="N15" s="64"/>
+      <c r="O15" s="64"/>
+      <c r="P15" s="64"/>
     </row>
     <row r="17" spans="5:36" x14ac:dyDescent="0.3">
-      <c r="H17" s="25" t="s">
+      <c r="H17" s="53" t="s">
         <v>26</v>
       </c>
-      <c r="I17" s="25"/>
-      <c r="J17" s="25"/>
-      <c r="K17" s="25" t="s">
+      <c r="I17" s="53"/>
+      <c r="J17" s="53"/>
+      <c r="K17" s="53" t="s">
         <v>26</v>
       </c>
-      <c r="L17" s="25"/>
-      <c r="M17" s="25"/>
+      <c r="L17" s="53"/>
+      <c r="M17" s="53"/>
       <c r="S17"/>
       <c r="T17"/>
       <c r="U17"/>
     </row>
     <row r="18" spans="5:36" x14ac:dyDescent="0.3">
-      <c r="H18" s="24" t="s">
+      <c r="H18" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="I18" s="24"/>
-      <c r="J18" s="24"/>
-      <c r="K18" s="24" t="s">
+      <c r="I18" s="50"/>
+      <c r="J18" s="50"/>
+      <c r="K18" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="L18" s="24"/>
-      <c r="M18" s="24"/>
-      <c r="S18" s="24" t="s">
+      <c r="L18" s="50"/>
+      <c r="M18" s="50"/>
+      <c r="S18" s="50" t="s">
         <v>32</v>
       </c>
-      <c r="T18" s="24"/>
-      <c r="U18" s="24"/>
-      <c r="AA18" s="24" t="s">
+      <c r="T18" s="50"/>
+      <c r="U18" s="50"/>
+      <c r="AA18" s="50" t="s">
         <v>35</v>
       </c>
-      <c r="AB18" s="24"/>
-      <c r="AC18" s="24"/>
-      <c r="AH18" s="24" t="s">
+      <c r="AB18" s="50"/>
+      <c r="AC18" s="50"/>
+      <c r="AH18" s="50" t="s">
         <v>36</v>
       </c>
-      <c r="AI18" s="24"/>
-      <c r="AJ18" s="24"/>
+      <c r="AI18" s="50"/>
+      <c r="AJ18" s="50"/>
     </row>
     <row r="19" spans="5:36" x14ac:dyDescent="0.3">
-      <c r="H19" s="24"/>
-      <c r="I19" s="24"/>
-      <c r="J19" s="24"/>
-      <c r="K19" s="24"/>
-      <c r="L19" s="24"/>
-      <c r="M19" s="24"/>
-      <c r="S19" s="24"/>
-      <c r="T19" s="24"/>
-      <c r="U19" s="24"/>
-      <c r="AA19" s="24"/>
-      <c r="AB19" s="24"/>
-      <c r="AC19" s="24"/>
-      <c r="AH19" s="24"/>
-      <c r="AI19" s="24"/>
-      <c r="AJ19" s="24"/>
+      <c r="H19" s="50"/>
+      <c r="I19" s="50"/>
+      <c r="J19" s="50"/>
+      <c r="K19" s="50"/>
+      <c r="L19" s="50"/>
+      <c r="M19" s="50"/>
+      <c r="S19" s="50"/>
+      <c r="T19" s="50"/>
+      <c r="U19" s="50"/>
+      <c r="AA19" s="50"/>
+      <c r="AB19" s="50"/>
+      <c r="AC19" s="50"/>
+      <c r="AH19" s="50"/>
+      <c r="AI19" s="50"/>
+      <c r="AJ19" s="50"/>
     </row>
     <row r="20" spans="5:36" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H20" s="24"/>
-      <c r="I20" s="24"/>
-      <c r="J20" s="24"/>
-      <c r="K20" s="24"/>
-      <c r="L20" s="24"/>
-      <c r="M20" s="24"/>
-      <c r="S20" s="24"/>
-      <c r="T20" s="24"/>
-      <c r="U20" s="24"/>
-      <c r="AA20" s="24"/>
-      <c r="AB20" s="24"/>
-      <c r="AC20" s="24"/>
-      <c r="AH20" s="24"/>
-      <c r="AI20" s="24"/>
-      <c r="AJ20" s="24"/>
+      <c r="H20" s="50"/>
+      <c r="I20" s="50"/>
+      <c r="J20" s="50"/>
+      <c r="K20" s="50"/>
+      <c r="L20" s="50"/>
+      <c r="M20" s="50"/>
+      <c r="S20" s="50"/>
+      <c r="T20" s="50"/>
+      <c r="U20" s="50"/>
+      <c r="AA20" s="50"/>
+      <c r="AB20" s="50"/>
+      <c r="AC20" s="50"/>
+      <c r="AH20" s="50"/>
+      <c r="AI20" s="50"/>
+      <c r="AJ20" s="50"/>
     </row>
     <row r="21" spans="5:36" ht="20.399999999999999" x14ac:dyDescent="0.3">
-      <c r="E21" s="24" t="s">
+      <c r="E21" s="50" t="s">
         <v>30</v>
       </c>
-      <c r="F21" s="24"/>
+      <c r="F21" s="50"/>
       <c r="G21" s="2" t="s">
         <v>27</v>
       </c>
@@ -2020,10 +2231,10 @@
       <c r="M21" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="O21" s="24" t="s">
+      <c r="O21" s="50" t="s">
         <v>34</v>
       </c>
-      <c r="P21" s="24"/>
+      <c r="P21" s="50"/>
       <c r="Q21" s="18" t="s">
         <v>33</v>
       </c>
@@ -2040,10 +2251,10 @@
         <v>2</v>
       </c>
       <c r="W21"/>
-      <c r="X21" s="24" t="s">
+      <c r="X21" s="50" t="s">
         <v>34</v>
       </c>
-      <c r="Y21" s="24"/>
+      <c r="Y21" s="50"/>
       <c r="Z21" s="2" t="s">
         <v>31</v>
       </c>
@@ -2056,10 +2267,10 @@
       <c r="AC21" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="AE21" s="24" t="s">
+      <c r="AE21" s="50" t="s">
         <v>37</v>
       </c>
-      <c r="AF21" s="24"/>
+      <c r="AF21" s="50"/>
       <c r="AG21" s="18" t="s">
         <v>38</v>
       </c>
@@ -2074,8 +2285,8 @@
       </c>
     </row>
     <row r="22" spans="5:36" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E22" s="24"/>
-      <c r="F22" s="24"/>
+      <c r="E22" s="50"/>
+      <c r="F22" s="50"/>
       <c r="G22" s="2">
         <v>4</v>
       </c>
@@ -2097,8 +2308,8 @@
       <c r="M22" s="2">
         <v>578</v>
       </c>
-      <c r="O22" s="24"/>
-      <c r="P22" s="24"/>
+      <c r="O22" s="50"/>
+      <c r="P22" s="50"/>
       <c r="Q22" s="18">
         <v>8</v>
       </c>
@@ -2115,8 +2326,8 @@
         <v>455</v>
       </c>
       <c r="W22"/>
-      <c r="X22" s="24"/>
-      <c r="Y22" s="24"/>
+      <c r="X22" s="50"/>
+      <c r="Y22" s="50"/>
       <c r="Z22" s="2">
         <v>4</v>
       </c>
@@ -2129,8 +2340,8 @@
       <c r="AC22" s="2">
         <v>555</v>
       </c>
-      <c r="AE22" s="24"/>
-      <c r="AF22" s="24"/>
+      <c r="AE22" s="50"/>
+      <c r="AF22" s="50"/>
       <c r="AG22" s="2">
         <v>2</v>
       </c>
@@ -2145,8 +2356,8 @@
       </c>
     </row>
     <row r="23" spans="5:36" x14ac:dyDescent="0.3">
-      <c r="E23" s="24"/>
-      <c r="F23" s="24"/>
+      <c r="E23" s="50"/>
+      <c r="F23" s="50"/>
       <c r="G23" s="2">
         <v>8</v>
       </c>
@@ -2168,8 +2379,8 @@
       <c r="M23" s="2">
         <v>476</v>
       </c>
-      <c r="O23" s="24"/>
-      <c r="P23" s="24"/>
+      <c r="O23" s="50"/>
+      <c r="P23" s="50"/>
       <c r="Q23" s="18">
         <v>12</v>
       </c>
@@ -2186,8 +2397,8 @@
         <v>462</v>
       </c>
       <c r="W23"/>
-      <c r="X23" s="24"/>
-      <c r="Y23" s="24"/>
+      <c r="X23" s="50"/>
+      <c r="Y23" s="50"/>
       <c r="Z23" s="2">
         <v>8</v>
       </c>
@@ -2200,8 +2411,8 @@
       <c r="AC23" s="2">
         <v>542</v>
       </c>
-      <c r="AE23" s="24"/>
-      <c r="AF23" s="24"/>
+      <c r="AE23" s="50"/>
+      <c r="AF23" s="50"/>
       <c r="AG23" s="2">
         <v>4</v>
       </c>
@@ -2216,8 +2427,8 @@
       </c>
     </row>
     <row r="24" spans="5:36" x14ac:dyDescent="0.3">
-      <c r="E24" s="24"/>
-      <c r="F24" s="24"/>
+      <c r="E24" s="50"/>
+      <c r="F24" s="50"/>
       <c r="G24" s="2">
         <v>16</v>
       </c>
@@ -2239,8 +2450,8 @@
       <c r="M24" s="2">
         <v>387</v>
       </c>
-      <c r="O24" s="24"/>
-      <c r="P24" s="24"/>
+      <c r="O24" s="50"/>
+      <c r="P24" s="50"/>
       <c r="Q24" s="18">
         <v>16</v>
       </c>
@@ -2257,8 +2468,8 @@
         <v>390</v>
       </c>
       <c r="W24"/>
-      <c r="X24" s="24"/>
-      <c r="Y24" s="24"/>
+      <c r="X24" s="50"/>
+      <c r="Y24" s="50"/>
       <c r="Z24" s="2">
         <v>16</v>
       </c>
@@ -2271,8 +2482,8 @@
       <c r="AC24" s="2">
         <v>493</v>
       </c>
-      <c r="AE24" s="24"/>
-      <c r="AF24" s="24"/>
+      <c r="AE24" s="50"/>
+      <c r="AF24" s="50"/>
       <c r="AG24" s="2">
         <v>8</v>
       </c>
@@ -2288,49 +2499,81 @@
     </row>
     <row r="26" spans="5:36" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="27" spans="5:36" x14ac:dyDescent="0.3">
-      <c r="E27" s="58" t="s">
+      <c r="E27" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="F27" s="59"/>
-      <c r="G27" s="59"/>
-      <c r="H27" s="59"/>
-      <c r="I27" s="59"/>
-      <c r="J27" s="59"/>
-      <c r="K27" s="59"/>
-      <c r="L27" s="59"/>
-      <c r="M27" s="59"/>
-      <c r="N27" s="60"/>
+      <c r="F27" s="33"/>
+      <c r="G27" s="33"/>
+      <c r="H27" s="33"/>
+      <c r="I27" s="33"/>
+      <c r="J27" s="33"/>
+      <c r="K27" s="33"/>
+      <c r="L27" s="33"/>
+      <c r="M27" s="33"/>
+      <c r="N27" s="34"/>
+      <c r="S27" s="32" t="s">
+        <v>39</v>
+      </c>
+      <c r="T27" s="33"/>
+      <c r="U27" s="33"/>
+      <c r="V27" s="33"/>
+      <c r="W27" s="33"/>
+      <c r="X27" s="33"/>
+      <c r="Y27" s="33"/>
+      <c r="Z27" s="33"/>
+      <c r="AA27" s="33"/>
+      <c r="AB27" s="34"/>
     </row>
     <row r="28" spans="5:36" x14ac:dyDescent="0.3">
-      <c r="E28" s="61"/>
-      <c r="F28" s="56"/>
-      <c r="G28" s="56"/>
-      <c r="H28" s="56"/>
-      <c r="I28" s="56"/>
-      <c r="J28" s="56"/>
-      <c r="K28" s="56"/>
-      <c r="L28" s="56"/>
-      <c r="M28" s="56"/>
-      <c r="N28" s="62"/>
+      <c r="E28" s="35"/>
+      <c r="F28" s="36"/>
+      <c r="G28" s="36"/>
+      <c r="H28" s="36"/>
+      <c r="I28" s="36"/>
+      <c r="J28" s="36"/>
+      <c r="K28" s="36"/>
+      <c r="L28" s="36"/>
+      <c r="M28" s="36"/>
+      <c r="N28" s="37"/>
+      <c r="S28" s="35"/>
+      <c r="T28" s="36"/>
+      <c r="U28" s="36"/>
+      <c r="V28" s="36"/>
+      <c r="W28" s="36"/>
+      <c r="X28" s="36"/>
+      <c r="Y28" s="36"/>
+      <c r="Z28" s="36"/>
+      <c r="AA28" s="36"/>
+      <c r="AB28" s="37"/>
     </row>
     <row r="29" spans="5:36" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E29" s="70"/>
-      <c r="F29" s="57"/>
-      <c r="G29" s="57"/>
-      <c r="H29" s="57"/>
-      <c r="I29" s="57"/>
-      <c r="J29" s="57"/>
-      <c r="K29" s="57"/>
-      <c r="L29" s="57"/>
-      <c r="M29" s="57"/>
-      <c r="N29" s="71"/>
+      <c r="E29" s="38"/>
+      <c r="F29" s="39"/>
+      <c r="G29" s="39"/>
+      <c r="H29" s="39"/>
+      <c r="I29" s="39"/>
+      <c r="J29" s="39"/>
+      <c r="K29" s="39"/>
+      <c r="L29" s="39"/>
+      <c r="M29" s="39"/>
+      <c r="N29" s="40"/>
+      <c r="S29" s="38"/>
+      <c r="T29" s="39"/>
+      <c r="U29" s="39"/>
+      <c r="V29" s="39"/>
+      <c r="W29" s="39"/>
+      <c r="X29" s="39"/>
+      <c r="Y29" s="39"/>
+      <c r="Z29" s="39"/>
+      <c r="AA29" s="39"/>
+      <c r="AB29" s="40"/>
     </row>
     <row r="30" spans="5:36" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E30" s="63" t="s">
+      <c r="E30" s="30" t="s">
         <v>44</v>
       </c>
-      <c r="F30" s="67"/>
-      <c r="G30" s="66" t="s">
+      <c r="F30" s="31"/>
+      <c r="G30" s="24" t="s">
         <v>33</v>
       </c>
       <c r="H30" s="20" t="s">
@@ -2354,10 +2597,38 @@
       <c r="N30" s="22" t="s">
         <v>2</v>
       </c>
+      <c r="S30" s="30" t="s">
+        <v>44</v>
+      </c>
+      <c r="T30" s="31"/>
+      <c r="U30" s="24" t="s">
+        <v>33</v>
+      </c>
+      <c r="V30" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="W30" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="X30" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y30" s="20" t="s">
+        <v>43</v>
+      </c>
+      <c r="Z30" s="20" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA30" s="20" t="s">
+        <v>1</v>
+      </c>
+      <c r="AB30" s="22" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="31" spans="5:36" x14ac:dyDescent="0.3">
-      <c r="E31" s="64"/>
-      <c r="F31" s="39"/>
+      <c r="E31" s="26"/>
+      <c r="F31" s="27"/>
       <c r="G31" s="23">
         <v>4</v>
       </c>
@@ -2382,10 +2653,36 @@
       <c r="N31" s="5">
         <v>479</v>
       </c>
+      <c r="S31" s="26"/>
+      <c r="T31" s="27"/>
+      <c r="U31" s="23">
+        <v>4</v>
+      </c>
+      <c r="V31" s="2">
+        <v>2</v>
+      </c>
+      <c r="W31" s="2">
+        <v>2</v>
+      </c>
+      <c r="X31" s="2">
+        <v>2</v>
+      </c>
+      <c r="Y31" s="2">
+        <v>2</v>
+      </c>
+      <c r="Z31" s="2">
+        <v>2175</v>
+      </c>
+      <c r="AA31" s="2">
+        <v>2480</v>
+      </c>
+      <c r="AB31" s="5">
+        <v>479</v>
+      </c>
     </row>
     <row r="32" spans="5:36" x14ac:dyDescent="0.3">
-      <c r="E32" s="64"/>
-      <c r="F32" s="39"/>
+      <c r="E32" s="26"/>
+      <c r="F32" s="27"/>
       <c r="G32" s="23">
         <v>4</v>
       </c>
@@ -2410,10 +2707,36 @@
       <c r="N32" s="5">
         <v>300</v>
       </c>
-    </row>
-    <row r="33" spans="5:17" x14ac:dyDescent="0.3">
-      <c r="E33" s="64"/>
-      <c r="F33" s="39"/>
+      <c r="S32" s="26"/>
+      <c r="T32" s="27"/>
+      <c r="U32" s="23">
+        <v>4</v>
+      </c>
+      <c r="V32" s="2">
+        <v>4</v>
+      </c>
+      <c r="W32" s="2">
+        <v>4</v>
+      </c>
+      <c r="X32" s="2">
+        <v>4</v>
+      </c>
+      <c r="Y32" s="2">
+        <v>2</v>
+      </c>
+      <c r="Z32" s="2">
+        <v>6171</v>
+      </c>
+      <c r="AA32" s="2">
+        <v>6193</v>
+      </c>
+      <c r="AB32" s="5">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="33" spans="5:30" x14ac:dyDescent="0.3">
+      <c r="E33" s="26"/>
+      <c r="F33" s="27"/>
       <c r="G33" s="23">
         <v>4</v>
       </c>
@@ -2438,10 +2761,36 @@
       <c r="N33" s="5">
         <v>276</v>
       </c>
-    </row>
-    <row r="34" spans="5:17" x14ac:dyDescent="0.3">
-      <c r="E34" s="64"/>
-      <c r="F34" s="39"/>
+      <c r="S33" s="26"/>
+      <c r="T33" s="27"/>
+      <c r="U33" s="23">
+        <v>4</v>
+      </c>
+      <c r="V33" s="2">
+        <v>4</v>
+      </c>
+      <c r="W33" s="2">
+        <v>4</v>
+      </c>
+      <c r="X33" s="2">
+        <v>8</v>
+      </c>
+      <c r="Y33" s="2">
+        <v>2</v>
+      </c>
+      <c r="Z33" s="2">
+        <v>12422</v>
+      </c>
+      <c r="AA33" s="2">
+        <v>12448</v>
+      </c>
+      <c r="AB33" s="5">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="34" spans="5:30" x14ac:dyDescent="0.3">
+      <c r="E34" s="26"/>
+      <c r="F34" s="27"/>
       <c r="G34" s="23">
         <v>4</v>
       </c>
@@ -2466,10 +2815,36 @@
       <c r="N34" s="5">
         <v>290</v>
       </c>
-    </row>
-    <row r="35" spans="5:17" x14ac:dyDescent="0.3">
-      <c r="E35" s="64"/>
-      <c r="F35" s="39"/>
+      <c r="S34" s="26"/>
+      <c r="T34" s="27"/>
+      <c r="U34" s="23">
+        <v>4</v>
+      </c>
+      <c r="V34" s="2">
+        <v>4</v>
+      </c>
+      <c r="W34" s="2">
+        <v>4</v>
+      </c>
+      <c r="X34" s="2">
+        <v>8</v>
+      </c>
+      <c r="Y34" s="2">
+        <v>4</v>
+      </c>
+      <c r="Z34" s="2">
+        <v>28834</v>
+      </c>
+      <c r="AA34" s="2">
+        <v>27684</v>
+      </c>
+      <c r="AB34" s="5">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="35" spans="5:30" x14ac:dyDescent="0.3">
+      <c r="E35" s="26"/>
+      <c r="F35" s="27"/>
       <c r="G35" s="23">
         <v>8</v>
       </c>
@@ -2494,10 +2869,36 @@
       <c r="N35" s="5">
         <v>320</v>
       </c>
-    </row>
-    <row r="36" spans="5:17" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E36" s="64"/>
-      <c r="F36" s="39"/>
+      <c r="S35" s="26"/>
+      <c r="T35" s="27"/>
+      <c r="U35" s="23">
+        <v>8</v>
+      </c>
+      <c r="V35" s="2">
+        <v>8</v>
+      </c>
+      <c r="W35" s="2">
+        <v>8</v>
+      </c>
+      <c r="X35" s="2">
+        <v>8</v>
+      </c>
+      <c r="Y35" s="2">
+        <v>2</v>
+      </c>
+      <c r="Z35" s="2">
+        <v>31853</v>
+      </c>
+      <c r="AA35" s="2">
+        <v>27935</v>
+      </c>
+      <c r="AB35" s="5">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="36" spans="5:30" ht="20.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E36" s="26"/>
+      <c r="F36" s="27"/>
       <c r="G36" s="23">
         <v>8</v>
       </c>
@@ -2522,11 +2923,37 @@
       <c r="N36" s="5">
         <v>291</v>
       </c>
-    </row>
-    <row r="37" spans="5:17" ht="20.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E37" s="65"/>
-      <c r="F37" s="68"/>
-      <c r="G37" s="69">
+      <c r="S36" s="26"/>
+      <c r="T36" s="27"/>
+      <c r="U36" s="23">
+        <v>8</v>
+      </c>
+      <c r="V36" s="2">
+        <v>8</v>
+      </c>
+      <c r="W36" s="2">
+        <v>8</v>
+      </c>
+      <c r="X36" s="2">
+        <v>8</v>
+      </c>
+      <c r="Y36" s="2">
+        <v>4</v>
+      </c>
+      <c r="Z36" s="2">
+        <v>75076</v>
+      </c>
+      <c r="AA36" s="2">
+        <v>65148</v>
+      </c>
+      <c r="AB36" s="5">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="37" spans="5:30" ht="20.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E37" s="28"/>
+      <c r="F37" s="29"/>
+      <c r="G37" s="25">
         <v>12</v>
       </c>
       <c r="H37" s="7">
@@ -2551,13 +2978,43 @@
         <v>304</v>
       </c>
       <c r="Q37"/>
-    </row>
-    <row r="38" spans="5:17" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E38" s="64" t="s">
+      <c r="S37" s="28"/>
+      <c r="T37" s="29"/>
+      <c r="U37" s="25">
+        <v>12</v>
+      </c>
+      <c r="V37" s="7">
+        <v>12</v>
+      </c>
+      <c r="W37" s="7">
+        <v>12</v>
+      </c>
+      <c r="X37" s="7">
+        <v>8</v>
+      </c>
+      <c r="Y37" s="7">
+        <v>4</v>
+      </c>
+      <c r="Z37" s="72">
+        <v>242691</v>
+      </c>
+      <c r="AA37" s="72">
+        <v>242553</v>
+      </c>
+      <c r="AB37" s="8">
+        <v>304</v>
+      </c>
+      <c r="AC37" s="73" t="s">
+        <v>48</v>
+      </c>
+      <c r="AD37" s="74"/>
+    </row>
+    <row r="38" spans="5:30" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E38" s="26" t="s">
         <v>47</v>
       </c>
-      <c r="F38" s="39"/>
-      <c r="G38" s="66" t="s">
+      <c r="F38" s="27"/>
+      <c r="G38" s="24" t="s">
         <v>33</v>
       </c>
       <c r="H38" s="20" t="s">
@@ -2588,10 +3045,44 @@
         <v>46</v>
       </c>
       <c r="Q38"/>
-    </row>
-    <row r="39" spans="5:17" x14ac:dyDescent="0.3">
-      <c r="E39" s="64"/>
-      <c r="F39" s="39"/>
+      <c r="S38" s="26" t="s">
+        <v>47</v>
+      </c>
+      <c r="T38" s="27"/>
+      <c r="U38" s="24" t="s">
+        <v>33</v>
+      </c>
+      <c r="V38" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="W38" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="X38" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y38" s="20" t="s">
+        <v>43</v>
+      </c>
+      <c r="Z38" s="20" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA38" s="20" t="s">
+        <v>1</v>
+      </c>
+      <c r="AB38" s="22" t="s">
+        <v>2</v>
+      </c>
+      <c r="AC38" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="AD38" s="22" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="39" spans="5:30" x14ac:dyDescent="0.3">
+      <c r="E39" s="26"/>
+      <c r="F39" s="27"/>
       <c r="G39" s="23">
         <v>4</v>
       </c>
@@ -2617,18 +3108,52 @@
         <v>518</v>
       </c>
       <c r="O39" s="4">
-        <f>-(L31-L39)/L31*100</f>
+        <f t="shared" ref="O39:O45" si="0">-(L31-L39)/L31*100</f>
         <v>-11.03448275862069</v>
       </c>
       <c r="P39" s="5">
-        <f>-(M31-M39)/M39*100</f>
+        <f t="shared" ref="P39:P45" si="1">-(M31-M39)/M39*100</f>
         <v>17.056856187290968</v>
       </c>
       <c r="Q39"/>
-    </row>
-    <row r="40" spans="5:17" x14ac:dyDescent="0.3">
-      <c r="E40" s="64"/>
-      <c r="F40" s="39"/>
+      <c r="S39" s="26"/>
+      <c r="T39" s="27"/>
+      <c r="U39" s="23">
+        <v>4</v>
+      </c>
+      <c r="V39" s="2">
+        <v>2</v>
+      </c>
+      <c r="W39" s="2">
+        <v>2</v>
+      </c>
+      <c r="X39" s="2">
+        <v>2</v>
+      </c>
+      <c r="Y39" s="2">
+        <v>2</v>
+      </c>
+      <c r="Z39" s="2">
+        <v>1935</v>
+      </c>
+      <c r="AA39" s="2">
+        <v>2990</v>
+      </c>
+      <c r="AB39" s="5">
+        <v>518</v>
+      </c>
+      <c r="AC39" s="4">
+        <f t="shared" ref="AC39:AC45" si="2">-(Z31-Z39)/Z31*100</f>
+        <v>-11.03448275862069</v>
+      </c>
+      <c r="AD39" s="5">
+        <f t="shared" ref="AD39:AD45" si="3">-(AA31-AA39)/AA39*100</f>
+        <v>17.056856187290968</v>
+      </c>
+    </row>
+    <row r="40" spans="5:30" x14ac:dyDescent="0.3">
+      <c r="E40" s="26"/>
+      <c r="F40" s="27"/>
       <c r="G40" s="23">
         <v>4</v>
       </c>
@@ -2654,18 +3179,52 @@
         <v>295</v>
       </c>
       <c r="O40" s="4">
-        <f>-(L32-L40)/L32*100</f>
+        <f t="shared" si="0"/>
         <v>-15.84832280019446</v>
       </c>
       <c r="P40" s="5">
-        <f>-(M32-M40)/M40*100</f>
+        <f t="shared" si="1"/>
         <v>9.6440035016049013</v>
       </c>
       <c r="Q40"/>
-    </row>
-    <row r="41" spans="5:17" x14ac:dyDescent="0.3">
-      <c r="E41" s="64"/>
-      <c r="F41" s="39"/>
+      <c r="S40" s="26"/>
+      <c r="T40" s="27"/>
+      <c r="U40" s="23">
+        <v>4</v>
+      </c>
+      <c r="V40" s="2">
+        <v>4</v>
+      </c>
+      <c r="W40" s="2">
+        <v>4</v>
+      </c>
+      <c r="X40" s="2">
+        <v>4</v>
+      </c>
+      <c r="Y40" s="2">
+        <v>2</v>
+      </c>
+      <c r="Z40" s="2">
+        <v>5193</v>
+      </c>
+      <c r="AA40" s="2">
+        <v>6854</v>
+      </c>
+      <c r="AB40" s="5">
+        <v>309</v>
+      </c>
+      <c r="AC40" s="4">
+        <f t="shared" si="2"/>
+        <v>-15.84832280019446</v>
+      </c>
+      <c r="AD40" s="5">
+        <f t="shared" si="3"/>
+        <v>9.6440035016049013</v>
+      </c>
+    </row>
+    <row r="41" spans="5:30" x14ac:dyDescent="0.3">
+      <c r="E41" s="26"/>
+      <c r="F41" s="27"/>
       <c r="G41" s="23">
         <v>4</v>
       </c>
@@ -2691,18 +3250,52 @@
         <v>284</v>
       </c>
       <c r="O41" s="4">
-        <f>-(L33-L41)/L33*100</f>
+        <f t="shared" si="0"/>
         <v>-16.140718080824342</v>
       </c>
       <c r="P41" s="5">
-        <f>-(M33-M41)/M41*100</f>
+        <f t="shared" si="1"/>
         <v>9.1386861313868604</v>
       </c>
       <c r="Q41"/>
-    </row>
-    <row r="42" spans="5:17" x14ac:dyDescent="0.3">
-      <c r="E42" s="64"/>
-      <c r="F42" s="39"/>
+      <c r="S41" s="26"/>
+      <c r="T41" s="27"/>
+      <c r="U41" s="23">
+        <v>4</v>
+      </c>
+      <c r="V41" s="2">
+        <v>4</v>
+      </c>
+      <c r="W41" s="2">
+        <v>4</v>
+      </c>
+      <c r="X41" s="2">
+        <v>8</v>
+      </c>
+      <c r="Y41" s="2">
+        <v>2</v>
+      </c>
+      <c r="Z41" s="2">
+        <v>10417</v>
+      </c>
+      <c r="AA41" s="2">
+        <v>13700</v>
+      </c>
+      <c r="AB41" s="5">
+        <v>303</v>
+      </c>
+      <c r="AC41" s="4">
+        <f t="shared" si="2"/>
+        <v>-16.140718080824342</v>
+      </c>
+      <c r="AD41" s="5">
+        <f t="shared" si="3"/>
+        <v>9.1386861313868604</v>
+      </c>
+    </row>
+    <row r="42" spans="5:30" x14ac:dyDescent="0.3">
+      <c r="E42" s="26"/>
+      <c r="F42" s="27"/>
       <c r="G42" s="23">
         <v>4</v>
       </c>
@@ -2728,17 +3321,51 @@
         <v>290</v>
       </c>
       <c r="O42" s="4">
-        <f>-(L34-L42)/L34*100</f>
+        <f t="shared" si="0"/>
         <v>-31.670944024415622</v>
       </c>
       <c r="P42" s="5">
-        <f>-(M34-M42)/M42*100</f>
+        <f t="shared" si="1"/>
         <v>0.54248248607867799</v>
       </c>
-    </row>
-    <row r="43" spans="5:17" x14ac:dyDescent="0.3">
-      <c r="E43" s="64"/>
-      <c r="F43" s="39"/>
+      <c r="S42" s="26"/>
+      <c r="T42" s="27"/>
+      <c r="U42" s="23">
+        <v>4</v>
+      </c>
+      <c r="V42" s="2">
+        <v>4</v>
+      </c>
+      <c r="W42" s="2">
+        <v>4</v>
+      </c>
+      <c r="X42" s="2">
+        <v>8</v>
+      </c>
+      <c r="Y42" s="2">
+        <v>4</v>
+      </c>
+      <c r="Z42" s="2">
+        <v>19702</v>
+      </c>
+      <c r="AA42" s="2">
+        <v>27835</v>
+      </c>
+      <c r="AB42" s="5">
+        <v>303</v>
+      </c>
+      <c r="AC42" s="4">
+        <f t="shared" si="2"/>
+        <v>-31.670944024415622</v>
+      </c>
+      <c r="AD42" s="5">
+        <f t="shared" si="3"/>
+        <v>0.54248248607867799</v>
+      </c>
+    </row>
+    <row r="43" spans="5:30" x14ac:dyDescent="0.3">
+      <c r="E43" s="26"/>
+      <c r="F43" s="27"/>
       <c r="G43" s="23">
         <v>8</v>
       </c>
@@ -2764,17 +3391,51 @@
         <v>332</v>
       </c>
       <c r="O43" s="4">
-        <f>-(L35-L43)/L35*100</f>
+        <f t="shared" si="0"/>
         <v>-25.93162339497065</v>
       </c>
       <c r="P43" s="5">
-        <f>-(M35-M43)/M43*100</f>
+        <f t="shared" si="1"/>
         <v>0.28200185621474977</v>
       </c>
-    </row>
-    <row r="44" spans="5:17" x14ac:dyDescent="0.3">
-      <c r="E44" s="64"/>
-      <c r="F44" s="39"/>
+      <c r="S43" s="26"/>
+      <c r="T43" s="27"/>
+      <c r="U43" s="23">
+        <v>8</v>
+      </c>
+      <c r="V43" s="2">
+        <v>8</v>
+      </c>
+      <c r="W43" s="2">
+        <v>8</v>
+      </c>
+      <c r="X43" s="2">
+        <v>8</v>
+      </c>
+      <c r="Y43" s="2">
+        <v>2</v>
+      </c>
+      <c r="Z43" s="2">
+        <v>23593</v>
+      </c>
+      <c r="AA43" s="2">
+        <v>28014</v>
+      </c>
+      <c r="AB43" s="5">
+        <v>332</v>
+      </c>
+      <c r="AC43" s="4">
+        <f t="shared" si="2"/>
+        <v>-25.93162339497065</v>
+      </c>
+      <c r="AD43" s="5">
+        <f t="shared" si="3"/>
+        <v>0.28200185621474977</v>
+      </c>
+    </row>
+    <row r="44" spans="5:30" x14ac:dyDescent="0.3">
+      <c r="E44" s="26"/>
+      <c r="F44" s="27"/>
       <c r="G44" s="23">
         <v>8</v>
       </c>
@@ -2800,18 +3461,52 @@
         <v>320</v>
       </c>
       <c r="O44" s="4">
-        <f>-(L36-L44)/L36*100</f>
+        <f t="shared" si="0"/>
         <v>-36.688156001918053</v>
       </c>
       <c r="P44" s="5">
-        <f>-(M36-M44)/M44*100</f>
+        <f t="shared" si="1"/>
         <v>-5.6277056277056277</v>
       </c>
-    </row>
-    <row r="45" spans="5:17" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E45" s="65"/>
-      <c r="F45" s="68"/>
-      <c r="G45" s="69">
+      <c r="S44" s="26"/>
+      <c r="T44" s="27"/>
+      <c r="U44" s="23">
+        <v>8</v>
+      </c>
+      <c r="V44" s="2">
+        <v>8</v>
+      </c>
+      <c r="W44" s="2">
+        <v>8</v>
+      </c>
+      <c r="X44" s="2">
+        <v>8</v>
+      </c>
+      <c r="Y44" s="2">
+        <v>4</v>
+      </c>
+      <c r="Z44" s="2">
+        <v>47532</v>
+      </c>
+      <c r="AA44" s="2">
+        <v>61677</v>
+      </c>
+      <c r="AB44" s="5">
+        <v>320</v>
+      </c>
+      <c r="AC44" s="4">
+        <f t="shared" si="2"/>
+        <v>-36.688156001918053</v>
+      </c>
+      <c r="AD44" s="5">
+        <f t="shared" si="3"/>
+        <v>-5.6277056277056277</v>
+      </c>
+    </row>
+    <row r="45" spans="5:30" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E45" s="28"/>
+      <c r="F45" s="29"/>
+      <c r="G45" s="25">
         <v>12</v>
       </c>
       <c r="H45" s="7">
@@ -2836,16 +3531,393 @@
         <v>290</v>
       </c>
       <c r="O45" s="6">
-        <f>-(L37-L45)/L37*100</f>
+        <f t="shared" si="0"/>
         <v>-48.854716491340838</v>
       </c>
       <c r="P45" s="8">
-        <f>-(M37-M45)/M45*100</f>
+        <f t="shared" si="1"/>
         <v>-61.256930870796602</v>
       </c>
+      <c r="S45" s="28"/>
+      <c r="T45" s="29"/>
+      <c r="U45" s="25">
+        <v>12</v>
+      </c>
+      <c r="V45" s="7">
+        <v>12</v>
+      </c>
+      <c r="W45" s="7">
+        <v>12</v>
+      </c>
+      <c r="X45" s="7">
+        <v>8</v>
+      </c>
+      <c r="Y45" s="7">
+        <v>4</v>
+      </c>
+      <c r="Z45" s="7">
+        <v>124125</v>
+      </c>
+      <c r="AA45" s="7">
+        <v>150414</v>
+      </c>
+      <c r="AB45" s="8">
+        <v>290</v>
+      </c>
+      <c r="AC45" s="6">
+        <f t="shared" si="2"/>
+        <v>-48.854716491340838</v>
+      </c>
+      <c r="AD45" s="8">
+        <f t="shared" si="3"/>
+        <v>-61.256930870796602</v>
+      </c>
+    </row>
+    <row r="47" spans="5:30" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="48" spans="5:30" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E48" s="32" t="s">
+        <v>49</v>
+      </c>
+      <c r="F48" s="33"/>
+      <c r="G48" s="33"/>
+      <c r="H48" s="33"/>
+      <c r="I48" s="33"/>
+      <c r="J48" s="33"/>
+      <c r="K48" s="34"/>
+      <c r="L48"/>
+      <c r="M48"/>
+      <c r="N48"/>
+    </row>
+    <row r="49" spans="5:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E49" s="35"/>
+      <c r="F49" s="36"/>
+      <c r="G49" s="36"/>
+      <c r="H49" s="36"/>
+      <c r="I49" s="36"/>
+      <c r="J49" s="36"/>
+      <c r="K49" s="37"/>
+      <c r="L49"/>
+      <c r="M49"/>
+      <c r="N49"/>
+    </row>
+    <row r="50" spans="5:14" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E50" s="77"/>
+      <c r="F50" s="78"/>
+      <c r="G50" s="78"/>
+      <c r="H50" s="78"/>
+      <c r="I50" s="78"/>
+      <c r="J50" s="78"/>
+      <c r="K50" s="79"/>
+      <c r="L50"/>
+      <c r="M50"/>
+      <c r="N50"/>
+    </row>
+    <row r="51" spans="5:14" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E51" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="F51" s="31"/>
+      <c r="G51" s="86" t="s">
+        <v>33</v>
+      </c>
+      <c r="H51" s="87" t="s">
+        <v>42</v>
+      </c>
+      <c r="I51" s="87" t="s">
+        <v>0</v>
+      </c>
+      <c r="J51" s="87" t="s">
+        <v>1</v>
+      </c>
+      <c r="K51" s="88" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="52" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="E52" s="26"/>
+      <c r="F52" s="27"/>
+      <c r="G52" s="4">
+        <v>2</v>
+      </c>
+      <c r="H52" s="2">
+        <v>4</v>
+      </c>
+      <c r="I52" s="2">
+        <v>1616</v>
+      </c>
+      <c r="J52" s="2">
+        <v>2121</v>
+      </c>
+      <c r="K52" s="5">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="53" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="E53" s="26"/>
+      <c r="F53" s="27"/>
+      <c r="G53" s="4">
+        <v>2</v>
+      </c>
+      <c r="H53" s="2">
+        <v>8</v>
+      </c>
+      <c r="I53" s="2">
+        <v>3441</v>
+      </c>
+      <c r="J53" s="2">
+        <v>4449</v>
+      </c>
+      <c r="K53" s="5">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="54" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="E54" s="26"/>
+      <c r="F54" s="27"/>
+      <c r="G54" s="80">
+        <v>4</v>
+      </c>
+      <c r="H54" s="2">
+        <v>4</v>
+      </c>
+      <c r="I54" s="2">
+        <v>3767</v>
+      </c>
+      <c r="J54" s="2">
+        <v>4161</v>
+      </c>
+      <c r="K54" s="5">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="55" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="E55" s="26"/>
+      <c r="F55" s="27"/>
+      <c r="G55" s="80">
+        <v>4</v>
+      </c>
+      <c r="H55" s="2">
+        <v>8</v>
+      </c>
+      <c r="I55" s="2">
+        <v>8139</v>
+      </c>
+      <c r="J55" s="2">
+        <v>8917</v>
+      </c>
+      <c r="K55" s="5">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="56" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="E56" s="26"/>
+      <c r="F56" s="27"/>
+      <c r="G56" s="80">
+        <v>8</v>
+      </c>
+      <c r="H56" s="2">
+        <v>4</v>
+      </c>
+      <c r="I56" s="2">
+        <v>9244</v>
+      </c>
+      <c r="J56" s="2">
+        <v>9133</v>
+      </c>
+      <c r="K56" s="5">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="57" spans="5:14" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E57" s="28"/>
+      <c r="F57" s="29"/>
+      <c r="G57" s="81">
+        <v>8</v>
+      </c>
+      <c r="H57" s="7">
+        <v>8</v>
+      </c>
+      <c r="I57" s="7">
+        <v>20588</v>
+      </c>
+      <c r="J57" s="7">
+        <v>19846</v>
+      </c>
+      <c r="K57" s="8">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="58" spans="5:14" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E58" s="30" t="s">
+        <v>50</v>
+      </c>
+      <c r="F58" s="31"/>
+      <c r="G58" s="83" t="s">
+        <v>33</v>
+      </c>
+      <c r="H58" s="84" t="s">
+        <v>42</v>
+      </c>
+      <c r="I58" s="84" t="s">
+        <v>0</v>
+      </c>
+      <c r="J58" s="84" t="s">
+        <v>1</v>
+      </c>
+      <c r="K58" s="85" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="59" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="E59" s="26"/>
+      <c r="F59" s="27"/>
+      <c r="G59" s="21">
+        <v>2</v>
+      </c>
+      <c r="H59" s="20">
+        <v>4</v>
+      </c>
+      <c r="I59" s="20">
+        <v>2251</v>
+      </c>
+      <c r="J59" s="20">
+        <v>3242</v>
+      </c>
+      <c r="K59" s="22">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="60" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="E60" s="26"/>
+      <c r="F60" s="27"/>
+      <c r="G60" s="4">
+        <v>2</v>
+      </c>
+      <c r="H60" s="2">
+        <v>8</v>
+      </c>
+      <c r="I60" s="2">
+        <v>4844</v>
+      </c>
+      <c r="J60" s="2">
+        <v>6858</v>
+      </c>
+      <c r="K60" s="5">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="61" spans="5:14" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E61" s="26"/>
+      <c r="F61" s="27"/>
+      <c r="G61" s="82">
+        <v>4</v>
+      </c>
+      <c r="H61" s="75">
+        <v>4</v>
+      </c>
+      <c r="I61" s="75">
+        <v>5986</v>
+      </c>
+      <c r="J61" s="75">
+        <v>6798</v>
+      </c>
+      <c r="K61" s="76">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="62" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="E62" s="26"/>
+      <c r="F62" s="27"/>
+      <c r="G62" s="80">
+        <v>4</v>
+      </c>
+      <c r="H62" s="2">
+        <v>8</v>
+      </c>
+      <c r="I62" s="2">
+        <v>12977</v>
+      </c>
+      <c r="J62" s="2">
+        <v>14628</v>
+      </c>
+      <c r="K62" s="5">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="63" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="E63" s="26"/>
+      <c r="F63" s="27"/>
+      <c r="G63" s="80">
+        <v>8</v>
+      </c>
+      <c r="H63" s="2">
+        <v>4</v>
+      </c>
+      <c r="I63" s="2">
+        <v>14749</v>
+      </c>
+      <c r="J63" s="2">
+        <v>14033</v>
+      </c>
+      <c r="K63" s="5">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="64" spans="5:14" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E64" s="28"/>
+      <c r="F64" s="29"/>
+      <c r="G64" s="81">
+        <v>8</v>
+      </c>
+      <c r="H64" s="7">
+        <v>8</v>
+      </c>
+      <c r="I64" s="7">
+        <v>32081</v>
+      </c>
+      <c r="J64" s="7">
+        <v>30525</v>
+      </c>
+      <c r="K64" s="8">
+        <v>341</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="43">
+  <mergeCells count="50">
+    <mergeCell ref="E48:K50"/>
+    <mergeCell ref="E51:F57"/>
+    <mergeCell ref="E58:F64"/>
+    <mergeCell ref="S27:AB29"/>
+    <mergeCell ref="S30:T37"/>
+    <mergeCell ref="S38:T45"/>
+    <mergeCell ref="AC37:AD37"/>
+    <mergeCell ref="AA18:AC20"/>
+    <mergeCell ref="X21:Y24"/>
+    <mergeCell ref="AH18:AJ20"/>
+    <mergeCell ref="AE21:AF24"/>
+    <mergeCell ref="S18:U20"/>
+    <mergeCell ref="N13:P15"/>
+    <mergeCell ref="H17:J17"/>
+    <mergeCell ref="H18:J20"/>
+    <mergeCell ref="E21:F24"/>
+    <mergeCell ref="K17:M17"/>
+    <mergeCell ref="K18:M20"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="F1:I1"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="H4:J6"/>
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="D4:G6"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="AC3:AE3"/>
+    <mergeCell ref="AC4:AE6"/>
+    <mergeCell ref="Z3:AB3"/>
+    <mergeCell ref="Z4:AB6"/>
+    <mergeCell ref="W4:Y6"/>
     <mergeCell ref="E38:F45"/>
     <mergeCell ref="E30:F37"/>
     <mergeCell ref="E27:N29"/>
@@ -2859,36 +3931,9 @@
     <mergeCell ref="Q4:S6"/>
     <mergeCell ref="K4:M6"/>
     <mergeCell ref="N4:P6"/>
-    <mergeCell ref="AC3:AE3"/>
-    <mergeCell ref="AC4:AE6"/>
-    <mergeCell ref="Z3:AB3"/>
-    <mergeCell ref="Z4:AB6"/>
-    <mergeCell ref="W4:Y6"/>
     <mergeCell ref="O21:P24"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="F1:I1"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="H4:J6"/>
-    <mergeCell ref="H3:J3"/>
     <mergeCell ref="D10:E10"/>
     <mergeCell ref="F10:G10"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="D4:G6"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="N13:P15"/>
-    <mergeCell ref="H17:J17"/>
-    <mergeCell ref="H18:J20"/>
-    <mergeCell ref="E21:F24"/>
-    <mergeCell ref="K17:M17"/>
-    <mergeCell ref="K18:M20"/>
-    <mergeCell ref="AA18:AC20"/>
-    <mergeCell ref="X21:Y24"/>
-    <mergeCell ref="AH18:AJ20"/>
-    <mergeCell ref="AE21:AF24"/>
-    <mergeCell ref="S18:U20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
modify table_sort and add make CBT module
</commit_message>
<xml_diff>
--- a/module_library/comp_sum_select.xlsx
+++ b/module_library/comp_sum_select.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\LRMLD\module_library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06C9BDA5-2C13-4385-A252-985703916597}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA8207AC-ED92-43BA-ABC7-D60F99CCF1B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="54">
   <si>
     <t>LUT</t>
   </si>
@@ -236,6 +236,19 @@
   <si>
     <t xml:space="preserve">M_W = 10
  L_W = 32
+</t>
+  </si>
+  <si>
+    <t>table_sort</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M_W = 10
+ L_W = 4
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M_W = 10
+ L_W = 8
 </t>
   </si>
 </sst>
@@ -290,7 +303,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="58">
+  <borders count="55">
     <border>
       <left/>
       <right/>
@@ -1004,50 +1017,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="89">
+  <cellXfs count="87">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1124,6 +1098,66 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1136,30 +1170,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1169,148 +1179,106 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1604,177 +1572,177 @@
   </cols>
   <sheetData>
     <row r="1" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="D1" s="53" t="s">
+      <c r="D1" s="57" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="53"/>
-      <c r="F1" s="53" t="s">
-        <v>8</v>
-      </c>
-      <c r="G1" s="53"/>
-      <c r="H1" s="53"/>
-      <c r="I1" s="53"/>
+      <c r="E1" s="57"/>
+      <c r="F1" s="57" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" s="57"/>
+      <c r="H1" s="57"/>
+      <c r="I1" s="57"/>
     </row>
     <row r="2" spans="4:31" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="3" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="H3" s="71" t="s">
+      <c r="H3" s="61" t="s">
         <v>12</v>
       </c>
-      <c r="I3" s="48"/>
-      <c r="J3" s="48"/>
-      <c r="K3" s="48" t="s">
+      <c r="I3" s="62"/>
+      <c r="J3" s="62"/>
+      <c r="K3" s="62" t="s">
         <v>12</v>
       </c>
-      <c r="L3" s="48"/>
-      <c r="M3" s="48"/>
-      <c r="N3" s="44" t="s">
+      <c r="L3" s="62"/>
+      <c r="M3" s="62"/>
+      <c r="N3" s="77" t="s">
         <v>14</v>
       </c>
-      <c r="O3" s="45"/>
-      <c r="P3" s="46"/>
-      <c r="Q3" s="41" t="s">
+      <c r="O3" s="78"/>
+      <c r="P3" s="79"/>
+      <c r="Q3" s="74" t="s">
         <v>13</v>
       </c>
-      <c r="R3" s="42"/>
-      <c r="S3" s="42"/>
-      <c r="T3" s="42" t="s">
+      <c r="R3" s="75"/>
+      <c r="S3" s="75"/>
+      <c r="T3" s="75" t="s">
         <v>17</v>
       </c>
-      <c r="U3" s="42"/>
-      <c r="V3" s="49"/>
-      <c r="W3" s="43" t="s">
+      <c r="U3" s="75"/>
+      <c r="V3" s="81"/>
+      <c r="W3" s="76" t="s">
         <v>15</v>
       </c>
-      <c r="X3" s="42"/>
-      <c r="Y3" s="42"/>
-      <c r="Z3" s="57" t="s">
+      <c r="X3" s="75"/>
+      <c r="Y3" s="75"/>
+      <c r="Z3" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="AA3" s="58"/>
-      <c r="AB3" s="59"/>
-      <c r="AC3" s="57" t="s">
+      <c r="AA3" s="64"/>
+      <c r="AB3" s="65"/>
+      <c r="AC3" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="AD3" s="58"/>
-      <c r="AE3" s="59"/>
+      <c r="AD3" s="64"/>
+      <c r="AE3" s="65"/>
     </row>
     <row r="4" spans="4:31" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D4" s="53" t="s">
+      <c r="D4" s="57" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="53"/>
-      <c r="F4" s="53"/>
-      <c r="G4" s="69"/>
-      <c r="H4" s="70" t="s">
+      <c r="E4" s="57"/>
+      <c r="F4" s="57"/>
+      <c r="G4" s="58"/>
+      <c r="H4" s="59" t="s">
         <v>20</v>
       </c>
-      <c r="I4" s="54"/>
-      <c r="J4" s="54"/>
-      <c r="K4" s="54" t="s">
+      <c r="I4" s="60"/>
+      <c r="J4" s="60"/>
+      <c r="K4" s="60" t="s">
         <v>21</v>
       </c>
-      <c r="L4" s="54"/>
-      <c r="M4" s="54"/>
-      <c r="N4" s="55" t="s">
+      <c r="L4" s="60"/>
+      <c r="M4" s="60"/>
+      <c r="N4" s="84" t="s">
         <v>9</v>
       </c>
-      <c r="O4" s="50"/>
-      <c r="P4" s="56"/>
-      <c r="Q4" s="52" t="s">
+      <c r="O4" s="55"/>
+      <c r="P4" s="85"/>
+      <c r="Q4" s="83" t="s">
         <v>10</v>
       </c>
-      <c r="R4" s="53"/>
-      <c r="S4" s="53"/>
-      <c r="T4" s="50" t="s">
+      <c r="R4" s="57"/>
+      <c r="S4" s="57"/>
+      <c r="T4" s="55" t="s">
         <v>18</v>
       </c>
-      <c r="U4" s="50"/>
-      <c r="V4" s="51"/>
-      <c r="W4" s="68" t="s">
+      <c r="U4" s="55"/>
+      <c r="V4" s="82"/>
+      <c r="W4" s="73" t="s">
         <v>11</v>
       </c>
-      <c r="X4" s="53"/>
-      <c r="Y4" s="53"/>
-      <c r="Z4" s="60" t="s">
+      <c r="X4" s="57"/>
+      <c r="Y4" s="57"/>
+      <c r="Z4" s="66" t="s">
         <v>16</v>
       </c>
-      <c r="AA4" s="61"/>
-      <c r="AB4" s="62"/>
-      <c r="AC4" s="60" t="s">
+      <c r="AA4" s="67"/>
+      <c r="AB4" s="68"/>
+      <c r="AC4" s="66" t="s">
         <v>23</v>
       </c>
-      <c r="AD4" s="61"/>
-      <c r="AE4" s="62"/>
+      <c r="AD4" s="67"/>
+      <c r="AE4" s="68"/>
     </row>
     <row r="5" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="D5" s="53"/>
-      <c r="E5" s="53"/>
-      <c r="F5" s="53"/>
-      <c r="G5" s="69"/>
-      <c r="H5" s="70"/>
-      <c r="I5" s="54"/>
-      <c r="J5" s="54"/>
-      <c r="K5" s="54"/>
-      <c r="L5" s="54"/>
-      <c r="M5" s="54"/>
-      <c r="N5" s="55"/>
-      <c r="O5" s="50"/>
-      <c r="P5" s="56"/>
-      <c r="Q5" s="52"/>
-      <c r="R5" s="53"/>
-      <c r="S5" s="53"/>
-      <c r="T5" s="50"/>
-      <c r="U5" s="50"/>
-      <c r="V5" s="51"/>
-      <c r="W5" s="68"/>
-      <c r="X5" s="53"/>
-      <c r="Y5" s="53"/>
-      <c r="Z5" s="63"/>
-      <c r="AA5" s="64"/>
-      <c r="AB5" s="27"/>
-      <c r="AC5" s="63"/>
-      <c r="AD5" s="64"/>
-      <c r="AE5" s="27"/>
+      <c r="D5" s="57"/>
+      <c r="E5" s="57"/>
+      <c r="F5" s="57"/>
+      <c r="G5" s="58"/>
+      <c r="H5" s="59"/>
+      <c r="I5" s="60"/>
+      <c r="J5" s="60"/>
+      <c r="K5" s="60"/>
+      <c r="L5" s="60"/>
+      <c r="M5" s="60"/>
+      <c r="N5" s="84"/>
+      <c r="O5" s="55"/>
+      <c r="P5" s="85"/>
+      <c r="Q5" s="83"/>
+      <c r="R5" s="57"/>
+      <c r="S5" s="57"/>
+      <c r="T5" s="55"/>
+      <c r="U5" s="55"/>
+      <c r="V5" s="82"/>
+      <c r="W5" s="73"/>
+      <c r="X5" s="57"/>
+      <c r="Y5" s="57"/>
+      <c r="Z5" s="69"/>
+      <c r="AA5" s="56"/>
+      <c r="AB5" s="47"/>
+      <c r="AC5" s="69"/>
+      <c r="AD5" s="56"/>
+      <c r="AE5" s="47"/>
     </row>
     <row r="6" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="D6" s="53"/>
-      <c r="E6" s="53"/>
-      <c r="F6" s="53"/>
-      <c r="G6" s="69"/>
-      <c r="H6" s="70"/>
-      <c r="I6" s="54"/>
-      <c r="J6" s="54"/>
-      <c r="K6" s="54"/>
-      <c r="L6" s="54"/>
-      <c r="M6" s="54"/>
-      <c r="N6" s="55"/>
-      <c r="O6" s="50"/>
-      <c r="P6" s="56"/>
-      <c r="Q6" s="52"/>
-      <c r="R6" s="53"/>
-      <c r="S6" s="53"/>
-      <c r="T6" s="50"/>
-      <c r="U6" s="50"/>
-      <c r="V6" s="51"/>
-      <c r="W6" s="68"/>
-      <c r="X6" s="53"/>
-      <c r="Y6" s="53"/>
-      <c r="Z6" s="65"/>
-      <c r="AA6" s="66"/>
-      <c r="AB6" s="67"/>
-      <c r="AC6" s="65"/>
-      <c r="AD6" s="66"/>
-      <c r="AE6" s="67"/>
+      <c r="D6" s="57"/>
+      <c r="E6" s="57"/>
+      <c r="F6" s="57"/>
+      <c r="G6" s="58"/>
+      <c r="H6" s="59"/>
+      <c r="I6" s="60"/>
+      <c r="J6" s="60"/>
+      <c r="K6" s="60"/>
+      <c r="L6" s="60"/>
+      <c r="M6" s="60"/>
+      <c r="N6" s="84"/>
+      <c r="O6" s="55"/>
+      <c r="P6" s="85"/>
+      <c r="Q6" s="83"/>
+      <c r="R6" s="57"/>
+      <c r="S6" s="57"/>
+      <c r="T6" s="55"/>
+      <c r="U6" s="55"/>
+      <c r="V6" s="82"/>
+      <c r="W6" s="73"/>
+      <c r="X6" s="57"/>
+      <c r="Y6" s="57"/>
+      <c r="Z6" s="70"/>
+      <c r="AA6" s="71"/>
+      <c r="AB6" s="72"/>
+      <c r="AC6" s="70"/>
+      <c r="AD6" s="71"/>
+      <c r="AE6" s="72"/>
     </row>
     <row r="7" spans="4:31" ht="20.399999999999999" x14ac:dyDescent="0.3">
-      <c r="D7" s="53" t="s">
-        <v>4</v>
-      </c>
-      <c r="E7" s="53"/>
-      <c r="F7" s="53" t="s">
+      <c r="D7" s="57" t="s">
+        <v>4</v>
+      </c>
+      <c r="E7" s="57"/>
+      <c r="F7" s="57" t="s">
         <v>5</v>
       </c>
-      <c r="G7" s="69"/>
+      <c r="G7" s="58"/>
       <c r="H7" s="11" t="s">
         <v>0</v>
       </c>
@@ -1849,14 +1817,14 @@
       </c>
     </row>
     <row r="8" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="D8" s="53">
-        <v>8</v>
-      </c>
-      <c r="E8" s="53"/>
-      <c r="F8" s="53">
-        <v>8</v>
-      </c>
-      <c r="G8" s="69"/>
+      <c r="D8" s="57">
+        <v>8</v>
+      </c>
+      <c r="E8" s="57"/>
+      <c r="F8" s="57">
+        <v>8</v>
+      </c>
+      <c r="G8" s="58"/>
       <c r="H8" s="11">
         <v>331</v>
       </c>
@@ -1931,14 +1899,14 @@
       </c>
     </row>
     <row r="9" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="D9" s="53">
+      <c r="D9" s="57">
         <v>10</v>
       </c>
-      <c r="E9" s="53"/>
-      <c r="F9" s="53">
+      <c r="E9" s="57"/>
+      <c r="F9" s="57">
         <v>16</v>
       </c>
-      <c r="G9" s="69"/>
+      <c r="G9" s="58"/>
       <c r="H9" s="11">
         <v>504</v>
       </c>
@@ -2013,14 +1981,14 @@
       </c>
     </row>
     <row r="10" spans="4:31" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D10" s="53">
+      <c r="D10" s="57">
         <v>10</v>
       </c>
-      <c r="E10" s="53"/>
-      <c r="F10" s="53">
+      <c r="E10" s="57"/>
+      <c r="F10" s="57">
         <v>32</v>
       </c>
-      <c r="G10" s="69"/>
+      <c r="G10" s="58"/>
       <c r="H10" s="13">
         <v>761</v>
       </c>
@@ -2095,17 +2063,17 @@
       </c>
     </row>
     <row r="11" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="H11" s="47" t="s">
+      <c r="H11" s="80" t="s">
         <v>24</v>
       </c>
-      <c r="I11" s="47"/>
-      <c r="J11" s="47"/>
-      <c r="K11" s="47"/>
-      <c r="L11" s="47"/>
-      <c r="M11" s="47"/>
-      <c r="N11" s="47"/>
-      <c r="O11" s="47"/>
-      <c r="P11" s="47"/>
+      <c r="I11" s="80"/>
+      <c r="J11" s="80"/>
+      <c r="K11" s="80"/>
+      <c r="L11" s="80"/>
+      <c r="M11" s="80"/>
+      <c r="N11" s="80"/>
+      <c r="O11" s="80"/>
+      <c r="P11" s="80"/>
     </row>
     <row r="12" spans="4:31" ht="23.4" x14ac:dyDescent="0.3">
       <c r="O12" s="19" t="s">
@@ -2113,103 +2081,103 @@
       </c>
     </row>
     <row r="13" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="N13" s="64" t="s">
+      <c r="N13" s="56" t="s">
         <v>19</v>
       </c>
-      <c r="O13" s="64"/>
-      <c r="P13" s="64"/>
+      <c r="O13" s="56"/>
+      <c r="P13" s="56"/>
     </row>
     <row r="14" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="N14" s="64"/>
-      <c r="O14" s="64"/>
-      <c r="P14" s="64"/>
+      <c r="N14" s="56"/>
+      <c r="O14" s="56"/>
+      <c r="P14" s="56"/>
     </row>
     <row r="15" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="N15" s="64"/>
-      <c r="O15" s="64"/>
-      <c r="P15" s="64"/>
+      <c r="N15" s="56"/>
+      <c r="O15" s="56"/>
+      <c r="P15" s="56"/>
     </row>
     <row r="17" spans="5:36" x14ac:dyDescent="0.3">
-      <c r="H17" s="53" t="s">
+      <c r="H17" s="57" t="s">
         <v>26</v>
       </c>
-      <c r="I17" s="53"/>
-      <c r="J17" s="53"/>
-      <c r="K17" s="53" t="s">
+      <c r="I17" s="57"/>
+      <c r="J17" s="57"/>
+      <c r="K17" s="57" t="s">
         <v>26</v>
       </c>
-      <c r="L17" s="53"/>
-      <c r="M17" s="53"/>
+      <c r="L17" s="57"/>
+      <c r="M17" s="57"/>
       <c r="S17"/>
       <c r="T17"/>
       <c r="U17"/>
     </row>
     <row r="18" spans="5:36" x14ac:dyDescent="0.3">
-      <c r="H18" s="50" t="s">
+      <c r="H18" s="55" t="s">
         <v>28</v>
       </c>
-      <c r="I18" s="50"/>
-      <c r="J18" s="50"/>
-      <c r="K18" s="50" t="s">
+      <c r="I18" s="55"/>
+      <c r="J18" s="55"/>
+      <c r="K18" s="55" t="s">
         <v>29</v>
       </c>
-      <c r="L18" s="50"/>
-      <c r="M18" s="50"/>
-      <c r="S18" s="50" t="s">
+      <c r="L18" s="55"/>
+      <c r="M18" s="55"/>
+      <c r="S18" s="55" t="s">
         <v>32</v>
       </c>
-      <c r="T18" s="50"/>
-      <c r="U18" s="50"/>
-      <c r="AA18" s="50" t="s">
+      <c r="T18" s="55"/>
+      <c r="U18" s="55"/>
+      <c r="AA18" s="55" t="s">
         <v>35</v>
       </c>
-      <c r="AB18" s="50"/>
-      <c r="AC18" s="50"/>
-      <c r="AH18" s="50" t="s">
+      <c r="AB18" s="55"/>
+      <c r="AC18" s="55"/>
+      <c r="AH18" s="55" t="s">
         <v>36</v>
       </c>
-      <c r="AI18" s="50"/>
-      <c r="AJ18" s="50"/>
+      <c r="AI18" s="55"/>
+      <c r="AJ18" s="55"/>
     </row>
     <row r="19" spans="5:36" x14ac:dyDescent="0.3">
-      <c r="H19" s="50"/>
-      <c r="I19" s="50"/>
-      <c r="J19" s="50"/>
-      <c r="K19" s="50"/>
-      <c r="L19" s="50"/>
-      <c r="M19" s="50"/>
-      <c r="S19" s="50"/>
-      <c r="T19" s="50"/>
-      <c r="U19" s="50"/>
-      <c r="AA19" s="50"/>
-      <c r="AB19" s="50"/>
-      <c r="AC19" s="50"/>
-      <c r="AH19" s="50"/>
-      <c r="AI19" s="50"/>
-      <c r="AJ19" s="50"/>
+      <c r="H19" s="55"/>
+      <c r="I19" s="55"/>
+      <c r="J19" s="55"/>
+      <c r="K19" s="55"/>
+      <c r="L19" s="55"/>
+      <c r="M19" s="55"/>
+      <c r="S19" s="55"/>
+      <c r="T19" s="55"/>
+      <c r="U19" s="55"/>
+      <c r="AA19" s="55"/>
+      <c r="AB19" s="55"/>
+      <c r="AC19" s="55"/>
+      <c r="AH19" s="55"/>
+      <c r="AI19" s="55"/>
+      <c r="AJ19" s="55"/>
     </row>
     <row r="20" spans="5:36" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H20" s="50"/>
-      <c r="I20" s="50"/>
-      <c r="J20" s="50"/>
-      <c r="K20" s="50"/>
-      <c r="L20" s="50"/>
-      <c r="M20" s="50"/>
-      <c r="S20" s="50"/>
-      <c r="T20" s="50"/>
-      <c r="U20" s="50"/>
-      <c r="AA20" s="50"/>
-      <c r="AB20" s="50"/>
-      <c r="AC20" s="50"/>
-      <c r="AH20" s="50"/>
-      <c r="AI20" s="50"/>
-      <c r="AJ20" s="50"/>
+      <c r="H20" s="55"/>
+      <c r="I20" s="55"/>
+      <c r="J20" s="55"/>
+      <c r="K20" s="55"/>
+      <c r="L20" s="55"/>
+      <c r="M20" s="55"/>
+      <c r="S20" s="55"/>
+      <c r="T20" s="55"/>
+      <c r="U20" s="55"/>
+      <c r="AA20" s="55"/>
+      <c r="AB20" s="55"/>
+      <c r="AC20" s="55"/>
+      <c r="AH20" s="55"/>
+      <c r="AI20" s="55"/>
+      <c r="AJ20" s="55"/>
     </row>
     <row r="21" spans="5:36" ht="20.399999999999999" x14ac:dyDescent="0.3">
-      <c r="E21" s="50" t="s">
+      <c r="E21" s="55" t="s">
         <v>30</v>
       </c>
-      <c r="F21" s="50"/>
+      <c r="F21" s="55"/>
       <c r="G21" s="2" t="s">
         <v>27</v>
       </c>
@@ -2231,10 +2199,10 @@
       <c r="M21" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="O21" s="50" t="s">
+      <c r="O21" s="55" t="s">
         <v>34</v>
       </c>
-      <c r="P21" s="50"/>
+      <c r="P21" s="55"/>
       <c r="Q21" s="18" t="s">
         <v>33</v>
       </c>
@@ -2251,10 +2219,10 @@
         <v>2</v>
       </c>
       <c r="W21"/>
-      <c r="X21" s="50" t="s">
+      <c r="X21" s="55" t="s">
         <v>34</v>
       </c>
-      <c r="Y21" s="50"/>
+      <c r="Y21" s="55"/>
       <c r="Z21" s="2" t="s">
         <v>31</v>
       </c>
@@ -2267,10 +2235,10 @@
       <c r="AC21" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="AE21" s="50" t="s">
+      <c r="AE21" s="55" t="s">
         <v>37</v>
       </c>
-      <c r="AF21" s="50"/>
+      <c r="AF21" s="55"/>
       <c r="AG21" s="18" t="s">
         <v>38</v>
       </c>
@@ -2285,8 +2253,8 @@
       </c>
     </row>
     <row r="22" spans="5:36" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E22" s="50"/>
-      <c r="F22" s="50"/>
+      <c r="E22" s="55"/>
+      <c r="F22" s="55"/>
       <c r="G22" s="2">
         <v>4</v>
       </c>
@@ -2308,8 +2276,8 @@
       <c r="M22" s="2">
         <v>578</v>
       </c>
-      <c r="O22" s="50"/>
-      <c r="P22" s="50"/>
+      <c r="O22" s="55"/>
+      <c r="P22" s="55"/>
       <c r="Q22" s="18">
         <v>8</v>
       </c>
@@ -2326,8 +2294,8 @@
         <v>455</v>
       </c>
       <c r="W22"/>
-      <c r="X22" s="50"/>
-      <c r="Y22" s="50"/>
+      <c r="X22" s="55"/>
+      <c r="Y22" s="55"/>
       <c r="Z22" s="2">
         <v>4</v>
       </c>
@@ -2340,8 +2308,8 @@
       <c r="AC22" s="2">
         <v>555</v>
       </c>
-      <c r="AE22" s="50"/>
-      <c r="AF22" s="50"/>
+      <c r="AE22" s="55"/>
+      <c r="AF22" s="55"/>
       <c r="AG22" s="2">
         <v>2</v>
       </c>
@@ -2356,8 +2324,8 @@
       </c>
     </row>
     <row r="23" spans="5:36" x14ac:dyDescent="0.3">
-      <c r="E23" s="50"/>
-      <c r="F23" s="50"/>
+      <c r="E23" s="55"/>
+      <c r="F23" s="55"/>
       <c r="G23" s="2">
         <v>8</v>
       </c>
@@ -2379,8 +2347,8 @@
       <c r="M23" s="2">
         <v>476</v>
       </c>
-      <c r="O23" s="50"/>
-      <c r="P23" s="50"/>
+      <c r="O23" s="55"/>
+      <c r="P23" s="55"/>
       <c r="Q23" s="18">
         <v>12</v>
       </c>
@@ -2397,8 +2365,8 @@
         <v>462</v>
       </c>
       <c r="W23"/>
-      <c r="X23" s="50"/>
-      <c r="Y23" s="50"/>
+      <c r="X23" s="55"/>
+      <c r="Y23" s="55"/>
       <c r="Z23" s="2">
         <v>8</v>
       </c>
@@ -2411,8 +2379,8 @@
       <c r="AC23" s="2">
         <v>542</v>
       </c>
-      <c r="AE23" s="50"/>
-      <c r="AF23" s="50"/>
+      <c r="AE23" s="55"/>
+      <c r="AF23" s="55"/>
       <c r="AG23" s="2">
         <v>4</v>
       </c>
@@ -2427,8 +2395,8 @@
       </c>
     </row>
     <row r="24" spans="5:36" x14ac:dyDescent="0.3">
-      <c r="E24" s="50"/>
-      <c r="F24" s="50"/>
+      <c r="E24" s="55"/>
+      <c r="F24" s="55"/>
       <c r="G24" s="2">
         <v>16</v>
       </c>
@@ -2450,8 +2418,8 @@
       <c r="M24" s="2">
         <v>387</v>
       </c>
-      <c r="O24" s="50"/>
-      <c r="P24" s="50"/>
+      <c r="O24" s="55"/>
+      <c r="P24" s="55"/>
       <c r="Q24" s="18">
         <v>16</v>
       </c>
@@ -2468,8 +2436,8 @@
         <v>390</v>
       </c>
       <c r="W24"/>
-      <c r="X24" s="50"/>
-      <c r="Y24" s="50"/>
+      <c r="X24" s="55"/>
+      <c r="Y24" s="55"/>
       <c r="Z24" s="2">
         <v>16</v>
       </c>
@@ -2482,8 +2450,8 @@
       <c r="AC24" s="2">
         <v>493</v>
       </c>
-      <c r="AE24" s="50"/>
-      <c r="AF24" s="50"/>
+      <c r="AE24" s="55"/>
+      <c r="AF24" s="55"/>
       <c r="AG24" s="2">
         <v>8</v>
       </c>
@@ -2499,80 +2467,80 @@
     </row>
     <row r="26" spans="5:36" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="27" spans="5:36" x14ac:dyDescent="0.3">
-      <c r="E27" s="32" t="s">
+      <c r="E27" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="F27" s="33"/>
-      <c r="G27" s="33"/>
-      <c r="H27" s="33"/>
-      <c r="I27" s="33"/>
-      <c r="J27" s="33"/>
-      <c r="K27" s="33"/>
-      <c r="L27" s="33"/>
-      <c r="M27" s="33"/>
-      <c r="N27" s="34"/>
-      <c r="S27" s="32" t="s">
+      <c r="F27" s="36"/>
+      <c r="G27" s="36"/>
+      <c r="H27" s="36"/>
+      <c r="I27" s="36"/>
+      <c r="J27" s="36"/>
+      <c r="K27" s="36"/>
+      <c r="L27" s="36"/>
+      <c r="M27" s="36"/>
+      <c r="N27" s="37"/>
+      <c r="S27" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="T27" s="33"/>
-      <c r="U27" s="33"/>
-      <c r="V27" s="33"/>
-      <c r="W27" s="33"/>
-      <c r="X27" s="33"/>
-      <c r="Y27" s="33"/>
-      <c r="Z27" s="33"/>
-      <c r="AA27" s="33"/>
-      <c r="AB27" s="34"/>
+      <c r="T27" s="36"/>
+      <c r="U27" s="36"/>
+      <c r="V27" s="36"/>
+      <c r="W27" s="36"/>
+      <c r="X27" s="36"/>
+      <c r="Y27" s="36"/>
+      <c r="Z27" s="36"/>
+      <c r="AA27" s="36"/>
+      <c r="AB27" s="37"/>
     </row>
     <row r="28" spans="5:36" x14ac:dyDescent="0.3">
-      <c r="E28" s="35"/>
-      <c r="F28" s="36"/>
-      <c r="G28" s="36"/>
-      <c r="H28" s="36"/>
-      <c r="I28" s="36"/>
-      <c r="J28" s="36"/>
-      <c r="K28" s="36"/>
-      <c r="L28" s="36"/>
-      <c r="M28" s="36"/>
-      <c r="N28" s="37"/>
-      <c r="S28" s="35"/>
-      <c r="T28" s="36"/>
-      <c r="U28" s="36"/>
-      <c r="V28" s="36"/>
-      <c r="W28" s="36"/>
-      <c r="X28" s="36"/>
-      <c r="Y28" s="36"/>
-      <c r="Z28" s="36"/>
-      <c r="AA28" s="36"/>
-      <c r="AB28" s="37"/>
+      <c r="E28" s="38"/>
+      <c r="F28" s="39"/>
+      <c r="G28" s="39"/>
+      <c r="H28" s="39"/>
+      <c r="I28" s="39"/>
+      <c r="J28" s="39"/>
+      <c r="K28" s="39"/>
+      <c r="L28" s="39"/>
+      <c r="M28" s="39"/>
+      <c r="N28" s="40"/>
+      <c r="S28" s="38"/>
+      <c r="T28" s="39"/>
+      <c r="U28" s="39"/>
+      <c r="V28" s="39"/>
+      <c r="W28" s="39"/>
+      <c r="X28" s="39"/>
+      <c r="Y28" s="39"/>
+      <c r="Z28" s="39"/>
+      <c r="AA28" s="39"/>
+      <c r="AB28" s="40"/>
     </row>
     <row r="29" spans="5:36" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E29" s="38"/>
-      <c r="F29" s="39"/>
-      <c r="G29" s="39"/>
-      <c r="H29" s="39"/>
-      <c r="I29" s="39"/>
-      <c r="J29" s="39"/>
-      <c r="K29" s="39"/>
-      <c r="L29" s="39"/>
-      <c r="M29" s="39"/>
-      <c r="N29" s="40"/>
-      <c r="S29" s="38"/>
-      <c r="T29" s="39"/>
-      <c r="U29" s="39"/>
-      <c r="V29" s="39"/>
-      <c r="W29" s="39"/>
-      <c r="X29" s="39"/>
-      <c r="Y29" s="39"/>
-      <c r="Z29" s="39"/>
-      <c r="AA29" s="39"/>
-      <c r="AB29" s="40"/>
+      <c r="E29" s="50"/>
+      <c r="F29" s="51"/>
+      <c r="G29" s="51"/>
+      <c r="H29" s="51"/>
+      <c r="I29" s="51"/>
+      <c r="J29" s="51"/>
+      <c r="K29" s="51"/>
+      <c r="L29" s="51"/>
+      <c r="M29" s="51"/>
+      <c r="N29" s="52"/>
+      <c r="S29" s="50"/>
+      <c r="T29" s="51"/>
+      <c r="U29" s="51"/>
+      <c r="V29" s="51"/>
+      <c r="W29" s="51"/>
+      <c r="X29" s="51"/>
+      <c r="Y29" s="51"/>
+      <c r="Z29" s="51"/>
+      <c r="AA29" s="51"/>
+      <c r="AB29" s="52"/>
     </row>
     <row r="30" spans="5:36" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E30" s="30" t="s">
+      <c r="E30" s="44" t="s">
         <v>44</v>
       </c>
-      <c r="F30" s="31"/>
+      <c r="F30" s="45"/>
       <c r="G30" s="24" t="s">
         <v>33</v>
       </c>
@@ -2597,10 +2565,10 @@
       <c r="N30" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="S30" s="30" t="s">
+      <c r="S30" s="44" t="s">
         <v>44</v>
       </c>
-      <c r="T30" s="31"/>
+      <c r="T30" s="45"/>
       <c r="U30" s="24" t="s">
         <v>33</v>
       </c>
@@ -2627,8 +2595,8 @@
       </c>
     </row>
     <row r="31" spans="5:36" x14ac:dyDescent="0.3">
-      <c r="E31" s="26"/>
-      <c r="F31" s="27"/>
+      <c r="E31" s="46"/>
+      <c r="F31" s="47"/>
       <c r="G31" s="23">
         <v>4</v>
       </c>
@@ -2653,8 +2621,8 @@
       <c r="N31" s="5">
         <v>479</v>
       </c>
-      <c r="S31" s="26"/>
-      <c r="T31" s="27"/>
+      <c r="S31" s="46"/>
+      <c r="T31" s="47"/>
       <c r="U31" s="23">
         <v>4</v>
       </c>
@@ -2681,8 +2649,8 @@
       </c>
     </row>
     <row r="32" spans="5:36" x14ac:dyDescent="0.3">
-      <c r="E32" s="26"/>
-      <c r="F32" s="27"/>
+      <c r="E32" s="46"/>
+      <c r="F32" s="47"/>
       <c r="G32" s="23">
         <v>4</v>
       </c>
@@ -2707,8 +2675,8 @@
       <c r="N32" s="5">
         <v>300</v>
       </c>
-      <c r="S32" s="26"/>
-      <c r="T32" s="27"/>
+      <c r="S32" s="46"/>
+      <c r="T32" s="47"/>
       <c r="U32" s="23">
         <v>4</v>
       </c>
@@ -2735,8 +2703,8 @@
       </c>
     </row>
     <row r="33" spans="5:30" x14ac:dyDescent="0.3">
-      <c r="E33" s="26"/>
-      <c r="F33" s="27"/>
+      <c r="E33" s="46"/>
+      <c r="F33" s="47"/>
       <c r="G33" s="23">
         <v>4</v>
       </c>
@@ -2761,8 +2729,8 @@
       <c r="N33" s="5">
         <v>276</v>
       </c>
-      <c r="S33" s="26"/>
-      <c r="T33" s="27"/>
+      <c r="S33" s="46"/>
+      <c r="T33" s="47"/>
       <c r="U33" s="23">
         <v>4</v>
       </c>
@@ -2789,8 +2757,8 @@
       </c>
     </row>
     <row r="34" spans="5:30" x14ac:dyDescent="0.3">
-      <c r="E34" s="26"/>
-      <c r="F34" s="27"/>
+      <c r="E34" s="46"/>
+      <c r="F34" s="47"/>
       <c r="G34" s="23">
         <v>4</v>
       </c>
@@ -2815,8 +2783,8 @@
       <c r="N34" s="5">
         <v>290</v>
       </c>
-      <c r="S34" s="26"/>
-      <c r="T34" s="27"/>
+      <c r="S34" s="46"/>
+      <c r="T34" s="47"/>
       <c r="U34" s="23">
         <v>4</v>
       </c>
@@ -2843,8 +2811,8 @@
       </c>
     </row>
     <row r="35" spans="5:30" x14ac:dyDescent="0.3">
-      <c r="E35" s="26"/>
-      <c r="F35" s="27"/>
+      <c r="E35" s="46"/>
+      <c r="F35" s="47"/>
       <c r="G35" s="23">
         <v>8</v>
       </c>
@@ -2869,8 +2837,8 @@
       <c r="N35" s="5">
         <v>320</v>
       </c>
-      <c r="S35" s="26"/>
-      <c r="T35" s="27"/>
+      <c r="S35" s="46"/>
+      <c r="T35" s="47"/>
       <c r="U35" s="23">
         <v>8</v>
       </c>
@@ -2897,8 +2865,8 @@
       </c>
     </row>
     <row r="36" spans="5:30" ht="20.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E36" s="26"/>
-      <c r="F36" s="27"/>
+      <c r="E36" s="46"/>
+      <c r="F36" s="47"/>
       <c r="G36" s="23">
         <v>8</v>
       </c>
@@ -2923,8 +2891,8 @@
       <c r="N36" s="5">
         <v>291</v>
       </c>
-      <c r="S36" s="26"/>
-      <c r="T36" s="27"/>
+      <c r="S36" s="46"/>
+      <c r="T36" s="47"/>
       <c r="U36" s="23">
         <v>8</v>
       </c>
@@ -2951,8 +2919,8 @@
       </c>
     </row>
     <row r="37" spans="5:30" ht="20.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E37" s="28"/>
-      <c r="F37" s="29"/>
+      <c r="E37" s="48"/>
+      <c r="F37" s="49"/>
       <c r="G37" s="25">
         <v>12</v>
       </c>
@@ -2978,8 +2946,8 @@
         <v>304</v>
       </c>
       <c r="Q37"/>
-      <c r="S37" s="28"/>
-      <c r="T37" s="29"/>
+      <c r="S37" s="48"/>
+      <c r="T37" s="49"/>
       <c r="U37" s="25">
         <v>12</v>
       </c>
@@ -2995,25 +2963,25 @@
       <c r="Y37" s="7">
         <v>4</v>
       </c>
-      <c r="Z37" s="72">
+      <c r="Z37" s="26">
         <v>242691</v>
       </c>
-      <c r="AA37" s="72">
+      <c r="AA37" s="26">
         <v>242553</v>
       </c>
       <c r="AB37" s="8">
         <v>304</v>
       </c>
-      <c r="AC37" s="73" t="s">
+      <c r="AC37" s="53" t="s">
         <v>48</v>
       </c>
-      <c r="AD37" s="74"/>
+      <c r="AD37" s="54"/>
     </row>
     <row r="38" spans="5:30" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E38" s="26" t="s">
+      <c r="E38" s="46" t="s">
         <v>47</v>
       </c>
-      <c r="F38" s="27"/>
+      <c r="F38" s="47"/>
       <c r="G38" s="24" t="s">
         <v>33</v>
       </c>
@@ -3045,10 +3013,10 @@
         <v>46</v>
       </c>
       <c r="Q38"/>
-      <c r="S38" s="26" t="s">
+      <c r="S38" s="46" t="s">
         <v>47</v>
       </c>
-      <c r="T38" s="27"/>
+      <c r="T38" s="47"/>
       <c r="U38" s="24" t="s">
         <v>33</v>
       </c>
@@ -3081,8 +3049,8 @@
       </c>
     </row>
     <row r="39" spans="5:30" x14ac:dyDescent="0.3">
-      <c r="E39" s="26"/>
-      <c r="F39" s="27"/>
+      <c r="E39" s="46"/>
+      <c r="F39" s="47"/>
       <c r="G39" s="23">
         <v>4</v>
       </c>
@@ -3116,8 +3084,8 @@
         <v>17.056856187290968</v>
       </c>
       <c r="Q39"/>
-      <c r="S39" s="26"/>
-      <c r="T39" s="27"/>
+      <c r="S39" s="46"/>
+      <c r="T39" s="47"/>
       <c r="U39" s="23">
         <v>4</v>
       </c>
@@ -3152,8 +3120,8 @@
       </c>
     </row>
     <row r="40" spans="5:30" x14ac:dyDescent="0.3">
-      <c r="E40" s="26"/>
-      <c r="F40" s="27"/>
+      <c r="E40" s="46"/>
+      <c r="F40" s="47"/>
       <c r="G40" s="23">
         <v>4</v>
       </c>
@@ -3187,8 +3155,8 @@
         <v>9.6440035016049013</v>
       </c>
       <c r="Q40"/>
-      <c r="S40" s="26"/>
-      <c r="T40" s="27"/>
+      <c r="S40" s="46"/>
+      <c r="T40" s="47"/>
       <c r="U40" s="23">
         <v>4</v>
       </c>
@@ -3223,8 +3191,8 @@
       </c>
     </row>
     <row r="41" spans="5:30" x14ac:dyDescent="0.3">
-      <c r="E41" s="26"/>
-      <c r="F41" s="27"/>
+      <c r="E41" s="46"/>
+      <c r="F41" s="47"/>
       <c r="G41" s="23">
         <v>4</v>
       </c>
@@ -3258,8 +3226,8 @@
         <v>9.1386861313868604</v>
       </c>
       <c r="Q41"/>
-      <c r="S41" s="26"/>
-      <c r="T41" s="27"/>
+      <c r="S41" s="46"/>
+      <c r="T41" s="47"/>
       <c r="U41" s="23">
         <v>4</v>
       </c>
@@ -3294,8 +3262,8 @@
       </c>
     </row>
     <row r="42" spans="5:30" x14ac:dyDescent="0.3">
-      <c r="E42" s="26"/>
-      <c r="F42" s="27"/>
+      <c r="E42" s="46"/>
+      <c r="F42" s="47"/>
       <c r="G42" s="23">
         <v>4</v>
       </c>
@@ -3328,8 +3296,8 @@
         <f t="shared" si="1"/>
         <v>0.54248248607867799</v>
       </c>
-      <c r="S42" s="26"/>
-      <c r="T42" s="27"/>
+      <c r="S42" s="46"/>
+      <c r="T42" s="47"/>
       <c r="U42" s="23">
         <v>4</v>
       </c>
@@ -3364,8 +3332,8 @@
       </c>
     </row>
     <row r="43" spans="5:30" x14ac:dyDescent="0.3">
-      <c r="E43" s="26"/>
-      <c r="F43" s="27"/>
+      <c r="E43" s="46"/>
+      <c r="F43" s="47"/>
       <c r="G43" s="23">
         <v>8</v>
       </c>
@@ -3398,8 +3366,8 @@
         <f t="shared" si="1"/>
         <v>0.28200185621474977</v>
       </c>
-      <c r="S43" s="26"/>
-      <c r="T43" s="27"/>
+      <c r="S43" s="46"/>
+      <c r="T43" s="47"/>
       <c r="U43" s="23">
         <v>8</v>
       </c>
@@ -3434,8 +3402,8 @@
       </c>
     </row>
     <row r="44" spans="5:30" x14ac:dyDescent="0.3">
-      <c r="E44" s="26"/>
-      <c r="F44" s="27"/>
+      <c r="E44" s="46"/>
+      <c r="F44" s="47"/>
       <c r="G44" s="23">
         <v>8</v>
       </c>
@@ -3468,8 +3436,8 @@
         <f t="shared" si="1"/>
         <v>-5.6277056277056277</v>
       </c>
-      <c r="S44" s="26"/>
-      <c r="T44" s="27"/>
+      <c r="S44" s="46"/>
+      <c r="T44" s="47"/>
       <c r="U44" s="23">
         <v>8</v>
       </c>
@@ -3504,8 +3472,8 @@
       </c>
     </row>
     <row r="45" spans="5:30" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E45" s="28"/>
-      <c r="F45" s="29"/>
+      <c r="E45" s="48"/>
+      <c r="F45" s="49"/>
       <c r="G45" s="25">
         <v>12</v>
       </c>
@@ -3538,8 +3506,8 @@
         <f t="shared" si="1"/>
         <v>-61.256930870796602</v>
       </c>
-      <c r="S45" s="28"/>
-      <c r="T45" s="29"/>
+      <c r="S45" s="48"/>
+      <c r="T45" s="49"/>
       <c r="U45" s="25">
         <v>12</v>
       </c>
@@ -3575,86 +3543,142 @@
     </row>
     <row r="47" spans="5:30" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="48" spans="5:30" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E48" s="32" t="s">
+      <c r="E48" s="35" t="s">
         <v>49</v>
       </c>
-      <c r="F48" s="33"/>
-      <c r="G48" s="33"/>
-      <c r="H48" s="33"/>
-      <c r="I48" s="33"/>
-      <c r="J48" s="33"/>
-      <c r="K48" s="34"/>
+      <c r="F48" s="36"/>
+      <c r="G48" s="36"/>
+      <c r="H48" s="36"/>
+      <c r="I48" s="36"/>
+      <c r="J48" s="36"/>
+      <c r="K48" s="37"/>
       <c r="L48"/>
       <c r="M48"/>
-      <c r="N48"/>
-    </row>
-    <row r="49" spans="5:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E49" s="35"/>
-      <c r="F49" s="36"/>
-      <c r="G49" s="36"/>
-      <c r="H49" s="36"/>
-      <c r="I49" s="36"/>
-      <c r="J49" s="36"/>
-      <c r="K49" s="37"/>
+      <c r="N48" s="35" t="s">
+        <v>51</v>
+      </c>
+      <c r="O48" s="36"/>
+      <c r="P48" s="36"/>
+      <c r="Q48" s="36"/>
+      <c r="R48" s="36"/>
+      <c r="S48" s="36"/>
+      <c r="T48" s="37"/>
+    </row>
+    <row r="49" spans="5:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E49" s="38"/>
+      <c r="F49" s="39"/>
+      <c r="G49" s="39"/>
+      <c r="H49" s="39"/>
+      <c r="I49" s="39"/>
+      <c r="J49" s="39"/>
+      <c r="K49" s="40"/>
       <c r="L49"/>
       <c r="M49"/>
-      <c r="N49"/>
-    </row>
-    <row r="50" spans="5:14" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E50" s="77"/>
-      <c r="F50" s="78"/>
-      <c r="G50" s="78"/>
-      <c r="H50" s="78"/>
-      <c r="I50" s="78"/>
-      <c r="J50" s="78"/>
-      <c r="K50" s="79"/>
+      <c r="N49" s="38"/>
+      <c r="O49" s="39"/>
+      <c r="P49" s="39"/>
+      <c r="Q49" s="39"/>
+      <c r="R49" s="39"/>
+      <c r="S49" s="39"/>
+      <c r="T49" s="40"/>
+    </row>
+    <row r="50" spans="5:20" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E50" s="41"/>
+      <c r="F50" s="42"/>
+      <c r="G50" s="42"/>
+      <c r="H50" s="42"/>
+      <c r="I50" s="42"/>
+      <c r="J50" s="42"/>
+      <c r="K50" s="43"/>
       <c r="L50"/>
       <c r="M50"/>
-      <c r="N50"/>
-    </row>
-    <row r="51" spans="5:14" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E51" s="30" t="s">
+      <c r="N50" s="41"/>
+      <c r="O50" s="42"/>
+      <c r="P50" s="42"/>
+      <c r="Q50" s="42"/>
+      <c r="R50" s="42"/>
+      <c r="S50" s="42"/>
+      <c r="T50" s="43"/>
+    </row>
+    <row r="51" spans="5:20" ht="20.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E51" s="44" t="s">
         <v>34</v>
       </c>
-      <c r="F51" s="31"/>
-      <c r="G51" s="86" t="s">
+      <c r="F51" s="45"/>
+      <c r="G51" s="32" t="s">
         <v>33</v>
       </c>
-      <c r="H51" s="87" t="s">
+      <c r="H51" s="33" t="s">
         <v>42</v>
       </c>
-      <c r="I51" s="87" t="s">
+      <c r="I51" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="J51" s="87" t="s">
+      <c r="J51" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="K51" s="88" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="52" spans="5:14" x14ac:dyDescent="0.3">
-      <c r="E52" s="26"/>
-      <c r="F52" s="27"/>
-      <c r="G52" s="4">
-        <v>2</v>
-      </c>
-      <c r="H52" s="2">
-        <v>4</v>
-      </c>
-      <c r="I52" s="2">
+      <c r="K51" s="34" t="s">
+        <v>2</v>
+      </c>
+      <c r="N51" s="44" t="s">
+        <v>52</v>
+      </c>
+      <c r="O51" s="45"/>
+      <c r="P51" s="32" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q51" s="33" t="s">
+        <v>42</v>
+      </c>
+      <c r="R51" s="33" t="s">
+        <v>0</v>
+      </c>
+      <c r="S51" s="33" t="s">
+        <v>1</v>
+      </c>
+      <c r="T51" s="34" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="52" spans="5:20" x14ac:dyDescent="0.3">
+      <c r="E52" s="46"/>
+      <c r="F52" s="47"/>
+      <c r="G52" s="86">
+        <v>2</v>
+      </c>
+      <c r="H52" s="27">
+        <v>4</v>
+      </c>
+      <c r="I52" s="27">
         <v>1616</v>
       </c>
-      <c r="J52" s="2">
+      <c r="J52" s="27">
         <v>2121</v>
       </c>
-      <c r="K52" s="5">
+      <c r="K52" s="28">
         <v>512</v>
       </c>
-    </row>
-    <row r="53" spans="5:14" x14ac:dyDescent="0.3">
-      <c r="E53" s="26"/>
-      <c r="F53" s="27"/>
+      <c r="N52" s="46"/>
+      <c r="O52" s="47"/>
+      <c r="P52" s="86">
+        <v>2</v>
+      </c>
+      <c r="Q52" s="27">
+        <v>4</v>
+      </c>
+      <c r="R52" s="27">
+        <v>124</v>
+      </c>
+      <c r="S52" s="27">
+        <v>113</v>
+      </c>
+      <c r="T52" s="28">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="53" spans="5:20" x14ac:dyDescent="0.3">
+      <c r="E53" s="46"/>
+      <c r="F53" s="47"/>
       <c r="G53" s="4">
         <v>2</v>
       </c>
@@ -3670,11 +3694,28 @@
       <c r="K53" s="5">
         <v>489</v>
       </c>
-    </row>
-    <row r="54" spans="5:14" x14ac:dyDescent="0.3">
-      <c r="E54" s="26"/>
-      <c r="F54" s="27"/>
-      <c r="G54" s="80">
+      <c r="N53" s="46"/>
+      <c r="O53" s="47"/>
+      <c r="P53" s="4">
+        <v>2</v>
+      </c>
+      <c r="Q53" s="2">
+        <v>8</v>
+      </c>
+      <c r="R53" s="2">
+        <v>257</v>
+      </c>
+      <c r="S53" s="2">
+        <v>226</v>
+      </c>
+      <c r="T53" s="5">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="54" spans="5:20" x14ac:dyDescent="0.3">
+      <c r="E54" s="46"/>
+      <c r="F54" s="47"/>
+      <c r="G54" s="29">
         <v>4</v>
       </c>
       <c r="H54" s="2">
@@ -3689,11 +3730,28 @@
       <c r="K54" s="5">
         <v>303</v>
       </c>
-    </row>
-    <row r="55" spans="5:14" x14ac:dyDescent="0.3">
-      <c r="E55" s="26"/>
-      <c r="F55" s="27"/>
-      <c r="G55" s="80">
+      <c r="N54" s="46"/>
+      <c r="O54" s="47"/>
+      <c r="P54" s="29">
+        <v>4</v>
+      </c>
+      <c r="Q54" s="2">
+        <v>4</v>
+      </c>
+      <c r="R54" s="2">
+        <v>663</v>
+      </c>
+      <c r="S54" s="2">
+        <v>453</v>
+      </c>
+      <c r="T54" s="5">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="55" spans="5:20" x14ac:dyDescent="0.3">
+      <c r="E55" s="46"/>
+      <c r="F55" s="47"/>
+      <c r="G55" s="29">
         <v>4</v>
       </c>
       <c r="H55" s="2">
@@ -3708,11 +3766,28 @@
       <c r="K55" s="5">
         <v>300</v>
       </c>
-    </row>
-    <row r="56" spans="5:14" x14ac:dyDescent="0.3">
-      <c r="E56" s="26"/>
-      <c r="F56" s="27"/>
-      <c r="G56" s="80">
+      <c r="N55" s="46"/>
+      <c r="O55" s="47"/>
+      <c r="P55" s="29">
+        <v>4</v>
+      </c>
+      <c r="Q55" s="2">
+        <v>8</v>
+      </c>
+      <c r="R55" s="2">
+        <v>1365</v>
+      </c>
+      <c r="S55" s="2">
+        <v>900</v>
+      </c>
+      <c r="T55" s="5">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="56" spans="5:20" x14ac:dyDescent="0.3">
+      <c r="E56" s="46"/>
+      <c r="F56" s="47"/>
+      <c r="G56" s="29">
         <v>8</v>
       </c>
       <c r="H56" s="2">
@@ -3727,11 +3802,28 @@
       <c r="K56" s="5">
         <v>329</v>
       </c>
-    </row>
-    <row r="57" spans="5:14" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E57" s="28"/>
-      <c r="F57" s="29"/>
-      <c r="G57" s="81">
+      <c r="N56" s="46"/>
+      <c r="O56" s="47"/>
+      <c r="P56" s="29">
+        <v>8</v>
+      </c>
+      <c r="Q56" s="2">
+        <v>4</v>
+      </c>
+      <c r="R56" s="2">
+        <v>3092</v>
+      </c>
+      <c r="S56" s="2">
+        <v>2690</v>
+      </c>
+      <c r="T56" s="5">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="57" spans="5:20" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E57" s="48"/>
+      <c r="F57" s="49"/>
+      <c r="G57" s="30">
         <v>8</v>
       </c>
       <c r="H57" s="7">
@@ -3746,31 +3838,67 @@
       <c r="K57" s="8">
         <v>329</v>
       </c>
-    </row>
-    <row r="58" spans="5:14" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E58" s="30" t="s">
+      <c r="N57" s="48"/>
+      <c r="O57" s="49"/>
+      <c r="P57" s="30">
+        <v>8</v>
+      </c>
+      <c r="Q57" s="7">
+        <v>8</v>
+      </c>
+      <c r="R57" s="7">
+        <v>6239</v>
+      </c>
+      <c r="S57" s="7">
+        <v>5378</v>
+      </c>
+      <c r="T57" s="8">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="58" spans="5:20" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E58" s="44" t="s">
         <v>50</v>
       </c>
-      <c r="F58" s="31"/>
-      <c r="G58" s="83" t="s">
+      <c r="F58" s="45"/>
+      <c r="G58" s="32" t="s">
         <v>33</v>
       </c>
-      <c r="H58" s="84" t="s">
+      <c r="H58" s="33" t="s">
         <v>42</v>
       </c>
-      <c r="I58" s="84" t="s">
+      <c r="I58" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="J58" s="84" t="s">
+      <c r="J58" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="K58" s="85" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="59" spans="5:14" x14ac:dyDescent="0.3">
-      <c r="E59" s="26"/>
-      <c r="F59" s="27"/>
+      <c r="K58" s="34" t="s">
+        <v>2</v>
+      </c>
+      <c r="N58" s="44" t="s">
+        <v>53</v>
+      </c>
+      <c r="O58" s="45"/>
+      <c r="P58" s="32" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q58" s="33" t="s">
+        <v>42</v>
+      </c>
+      <c r="R58" s="33" t="s">
+        <v>0</v>
+      </c>
+      <c r="S58" s="33" t="s">
+        <v>1</v>
+      </c>
+      <c r="T58" s="34" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="59" spans="5:20" x14ac:dyDescent="0.3">
+      <c r="E59" s="46"/>
+      <c r="F59" s="47"/>
       <c r="G59" s="21">
         <v>2</v>
       </c>
@@ -3786,10 +3914,27 @@
       <c r="K59" s="22">
         <v>492</v>
       </c>
-    </row>
-    <row r="60" spans="5:14" x14ac:dyDescent="0.3">
-      <c r="E60" s="26"/>
-      <c r="F60" s="27"/>
+      <c r="N59" s="46"/>
+      <c r="O59" s="47"/>
+      <c r="P59" s="86">
+        <v>2</v>
+      </c>
+      <c r="Q59" s="27">
+        <v>4</v>
+      </c>
+      <c r="R59" s="27">
+        <v>154</v>
+      </c>
+      <c r="S59" s="27">
+        <v>146</v>
+      </c>
+      <c r="T59" s="28">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="60" spans="5:20" x14ac:dyDescent="0.3">
+      <c r="E60" s="46"/>
+      <c r="F60" s="47"/>
       <c r="G60" s="4">
         <v>2</v>
       </c>
@@ -3805,30 +3950,64 @@
       <c r="K60" s="5">
         <v>489</v>
       </c>
-    </row>
-    <row r="61" spans="5:14" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E61" s="26"/>
-      <c r="F61" s="27"/>
-      <c r="G61" s="82">
-        <v>4</v>
-      </c>
-      <c r="H61" s="75">
-        <v>4</v>
-      </c>
-      <c r="I61" s="75">
+      <c r="N60" s="46"/>
+      <c r="O60" s="47"/>
+      <c r="P60" s="4">
+        <v>2</v>
+      </c>
+      <c r="Q60" s="2">
+        <v>8</v>
+      </c>
+      <c r="R60" s="2">
+        <v>313</v>
+      </c>
+      <c r="S60" s="2">
+        <v>289</v>
+      </c>
+      <c r="T60" s="5">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="61" spans="5:20" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E61" s="46"/>
+      <c r="F61" s="47"/>
+      <c r="G61" s="31">
+        <v>4</v>
+      </c>
+      <c r="H61" s="27">
+        <v>4</v>
+      </c>
+      <c r="I61" s="27">
         <v>5986</v>
       </c>
-      <c r="J61" s="75">
+      <c r="J61" s="27">
         <v>6798</v>
       </c>
-      <c r="K61" s="76">
+      <c r="K61" s="28">
         <v>307</v>
       </c>
-    </row>
-    <row r="62" spans="5:14" x14ac:dyDescent="0.3">
-      <c r="E62" s="26"/>
-      <c r="F62" s="27"/>
-      <c r="G62" s="80">
+      <c r="N61" s="46"/>
+      <c r="O61" s="47"/>
+      <c r="P61" s="29">
+        <v>4</v>
+      </c>
+      <c r="Q61" s="2">
+        <v>4</v>
+      </c>
+      <c r="R61" s="2">
+        <v>797</v>
+      </c>
+      <c r="S61" s="2">
+        <v>586</v>
+      </c>
+      <c r="T61" s="5">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="62" spans="5:20" x14ac:dyDescent="0.3">
+      <c r="E62" s="46"/>
+      <c r="F62" s="47"/>
+      <c r="G62" s="29">
         <v>4</v>
       </c>
       <c r="H62" s="2">
@@ -3843,11 +4022,28 @@
       <c r="K62" s="5">
         <v>298</v>
       </c>
-    </row>
-    <row r="63" spans="5:14" x14ac:dyDescent="0.3">
-      <c r="E63" s="26"/>
-      <c r="F63" s="27"/>
-      <c r="G63" s="80">
+      <c r="N62" s="46"/>
+      <c r="O62" s="47"/>
+      <c r="P62" s="29">
+        <v>4</v>
+      </c>
+      <c r="Q62" s="2">
+        <v>8</v>
+      </c>
+      <c r="R62" s="2">
+        <v>1683</v>
+      </c>
+      <c r="S62" s="2">
+        <v>1158</v>
+      </c>
+      <c r="T62" s="5">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="63" spans="5:20" x14ac:dyDescent="0.3">
+      <c r="E63" s="46"/>
+      <c r="F63" s="47"/>
+      <c r="G63" s="29">
         <v>8</v>
       </c>
       <c r="H63" s="2">
@@ -3862,11 +4058,28 @@
       <c r="K63" s="5">
         <v>357</v>
       </c>
-    </row>
-    <row r="64" spans="5:14" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E64" s="28"/>
-      <c r="F64" s="29"/>
-      <c r="G64" s="81">
+      <c r="N63" s="46"/>
+      <c r="O63" s="47"/>
+      <c r="P63" s="29">
+        <v>8</v>
+      </c>
+      <c r="Q63" s="2">
+        <v>4</v>
+      </c>
+      <c r="R63" s="2">
+        <v>3845</v>
+      </c>
+      <c r="S63" s="2">
+        <v>3460</v>
+      </c>
+      <c r="T63" s="5">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="64" spans="5:20" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E64" s="48"/>
+      <c r="F64" s="49"/>
+      <c r="G64" s="30">
         <v>8</v>
       </c>
       <c r="H64" s="7">
@@ -3881,27 +4094,46 @@
       <c r="K64" s="8">
         <v>341</v>
       </c>
+      <c r="N64" s="48"/>
+      <c r="O64" s="49"/>
+      <c r="P64" s="30">
+        <v>8</v>
+      </c>
+      <c r="Q64" s="7">
+        <v>8</v>
+      </c>
+      <c r="R64" s="7">
+        <v>7781</v>
+      </c>
+      <c r="S64" s="7">
+        <v>6925</v>
+      </c>
+      <c r="T64" s="8">
+        <v>409</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="50">
-    <mergeCell ref="E48:K50"/>
-    <mergeCell ref="E51:F57"/>
-    <mergeCell ref="E58:F64"/>
-    <mergeCell ref="S27:AB29"/>
-    <mergeCell ref="S30:T37"/>
-    <mergeCell ref="S38:T45"/>
-    <mergeCell ref="AC37:AD37"/>
-    <mergeCell ref="AA18:AC20"/>
-    <mergeCell ref="X21:Y24"/>
-    <mergeCell ref="AH18:AJ20"/>
-    <mergeCell ref="AE21:AF24"/>
-    <mergeCell ref="S18:U20"/>
-    <mergeCell ref="N13:P15"/>
-    <mergeCell ref="H17:J17"/>
-    <mergeCell ref="H18:J20"/>
-    <mergeCell ref="E21:F24"/>
-    <mergeCell ref="K17:M17"/>
-    <mergeCell ref="K18:M20"/>
+  <mergeCells count="53">
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="N48:T50"/>
+    <mergeCell ref="N51:O57"/>
+    <mergeCell ref="N58:O64"/>
+    <mergeCell ref="Q3:S3"/>
+    <mergeCell ref="W3:Y3"/>
+    <mergeCell ref="N3:P3"/>
+    <mergeCell ref="H11:P11"/>
+    <mergeCell ref="K3:M3"/>
+    <mergeCell ref="T3:V3"/>
+    <mergeCell ref="T4:V6"/>
+    <mergeCell ref="Q4:S6"/>
+    <mergeCell ref="K4:M6"/>
+    <mergeCell ref="N4:P6"/>
+    <mergeCell ref="AC3:AE3"/>
+    <mergeCell ref="AC4:AE6"/>
+    <mergeCell ref="Z3:AB3"/>
+    <mergeCell ref="Z4:AB6"/>
+    <mergeCell ref="W4:Y6"/>
     <mergeCell ref="D1:E1"/>
     <mergeCell ref="F1:I1"/>
     <mergeCell ref="D9:E9"/>
@@ -3913,27 +4145,28 @@
     <mergeCell ref="D7:E7"/>
     <mergeCell ref="F7:G7"/>
     <mergeCell ref="D8:E8"/>
-    <mergeCell ref="AC3:AE3"/>
-    <mergeCell ref="AC4:AE6"/>
-    <mergeCell ref="Z3:AB3"/>
-    <mergeCell ref="Z4:AB6"/>
-    <mergeCell ref="W4:Y6"/>
+    <mergeCell ref="S18:U20"/>
+    <mergeCell ref="N13:P15"/>
+    <mergeCell ref="H17:J17"/>
+    <mergeCell ref="H18:J20"/>
+    <mergeCell ref="E21:F24"/>
+    <mergeCell ref="K17:M17"/>
+    <mergeCell ref="K18:M20"/>
+    <mergeCell ref="O21:P24"/>
+    <mergeCell ref="AC37:AD37"/>
+    <mergeCell ref="AA18:AC20"/>
+    <mergeCell ref="X21:Y24"/>
+    <mergeCell ref="AH18:AJ20"/>
+    <mergeCell ref="AE21:AF24"/>
+    <mergeCell ref="E48:K50"/>
+    <mergeCell ref="E51:F57"/>
+    <mergeCell ref="E58:F64"/>
+    <mergeCell ref="S27:AB29"/>
+    <mergeCell ref="S30:T37"/>
+    <mergeCell ref="S38:T45"/>
     <mergeCell ref="E38:F45"/>
     <mergeCell ref="E30:F37"/>
     <mergeCell ref="E27:N29"/>
-    <mergeCell ref="Q3:S3"/>
-    <mergeCell ref="W3:Y3"/>
-    <mergeCell ref="N3:P3"/>
-    <mergeCell ref="H11:P11"/>
-    <mergeCell ref="K3:M3"/>
-    <mergeCell ref="T3:V3"/>
-    <mergeCell ref="T4:V6"/>
-    <mergeCell ref="Q4:S6"/>
-    <mergeCell ref="K4:M6"/>
-    <mergeCell ref="N4:P6"/>
-    <mergeCell ref="O21:P24"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="F10:G10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
add wp for make and modify table of comporasions
</commit_message>
<xml_diff>
--- a/module_library/comp_sum_select.xlsx
+++ b/module_library/comp_sum_select.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\LRMLD\module_library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA8207AC-ED92-43BA-ABC7-D60F99CCF1B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8061868E-8773-4B8C-84BB-DD4E0736B642}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="58">
   <si>
     <t>LUT</t>
   </si>
@@ -250,6 +250,18 @@
     <t xml:space="preserve">M_W = 10
  L_W = 8
 </t>
+  </si>
+  <si>
+    <t>LLR_W</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N </t>
+  </si>
+  <si>
+    <t>LABEL_W</t>
+  </si>
+  <si>
+    <t>make</t>
   </si>
 </sst>
 </file>
@@ -303,7 +315,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="55">
+  <borders count="57">
     <border>
       <left/>
       <right/>
@@ -1017,11 +1029,29 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="96">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1125,6 +1155,15 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1170,6 +1209,99 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1179,107 +1311,32 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1567,182 +1624,183 @@
     <col min="1" max="7" width="8.88671875" style="1"/>
     <col min="8" max="25" width="10.77734375" style="1" customWidth="1"/>
     <col min="26" max="27" width="12.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="28" max="35" width="10.77734375" style="1" customWidth="1"/>
+    <col min="28" max="28" width="13" style="1" customWidth="1"/>
+    <col min="29" max="35" width="10.77734375" style="1" customWidth="1"/>
     <col min="36" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="D1" s="57" t="s">
+      <c r="D1" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="57"/>
-      <c r="F1" s="57" t="s">
-        <v>8</v>
-      </c>
-      <c r="G1" s="57"/>
-      <c r="H1" s="57"/>
-      <c r="I1" s="57"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
+      <c r="I1" s="36"/>
     </row>
     <row r="2" spans="4:31" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="3" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="H3" s="61" t="s">
+      <c r="H3" s="81" t="s">
         <v>12</v>
       </c>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
-      <c r="K3" s="62" t="s">
+      <c r="I3" s="60"/>
+      <c r="J3" s="60"/>
+      <c r="K3" s="60" t="s">
         <v>12</v>
       </c>
-      <c r="L3" s="62"/>
-      <c r="M3" s="62"/>
-      <c r="N3" s="77" t="s">
+      <c r="L3" s="60"/>
+      <c r="M3" s="60"/>
+      <c r="N3" s="56" t="s">
         <v>14</v>
       </c>
-      <c r="O3" s="78"/>
-      <c r="P3" s="79"/>
-      <c r="Q3" s="74" t="s">
+      <c r="O3" s="57"/>
+      <c r="P3" s="58"/>
+      <c r="Q3" s="53" t="s">
         <v>13</v>
       </c>
-      <c r="R3" s="75"/>
-      <c r="S3" s="75"/>
-      <c r="T3" s="75" t="s">
+      <c r="R3" s="54"/>
+      <c r="S3" s="54"/>
+      <c r="T3" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="U3" s="75"/>
-      <c r="V3" s="81"/>
-      <c r="W3" s="76" t="s">
+      <c r="U3" s="54"/>
+      <c r="V3" s="61"/>
+      <c r="W3" s="55" t="s">
         <v>15</v>
       </c>
-      <c r="X3" s="75"/>
-      <c r="Y3" s="75"/>
-      <c r="Z3" s="63" t="s">
+      <c r="X3" s="54"/>
+      <c r="Y3" s="54"/>
+      <c r="Z3" s="68" t="s">
         <v>13</v>
       </c>
-      <c r="AA3" s="64"/>
-      <c r="AB3" s="65"/>
-      <c r="AC3" s="63" t="s">
+      <c r="AA3" s="69"/>
+      <c r="AB3" s="70"/>
+      <c r="AC3" s="68" t="s">
         <v>22</v>
       </c>
-      <c r="AD3" s="64"/>
-      <c r="AE3" s="65"/>
+      <c r="AD3" s="69"/>
+      <c r="AE3" s="70"/>
     </row>
     <row r="4" spans="4:31" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D4" s="57" t="s">
+      <c r="D4" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="57"/>
-      <c r="F4" s="57"/>
-      <c r="G4" s="58"/>
-      <c r="H4" s="59" t="s">
+      <c r="E4" s="36"/>
+      <c r="F4" s="36"/>
+      <c r="G4" s="37"/>
+      <c r="H4" s="80" t="s">
         <v>20</v>
       </c>
-      <c r="I4" s="60"/>
-      <c r="J4" s="60"/>
-      <c r="K4" s="60" t="s">
+      <c r="I4" s="65"/>
+      <c r="J4" s="65"/>
+      <c r="K4" s="65" t="s">
         <v>21</v>
       </c>
-      <c r="L4" s="60"/>
-      <c r="M4" s="60"/>
-      <c r="N4" s="84" t="s">
+      <c r="L4" s="65"/>
+      <c r="M4" s="65"/>
+      <c r="N4" s="66" t="s">
         <v>9</v>
       </c>
-      <c r="O4" s="55"/>
-      <c r="P4" s="85"/>
-      <c r="Q4" s="83" t="s">
+      <c r="O4" s="62"/>
+      <c r="P4" s="67"/>
+      <c r="Q4" s="64" t="s">
         <v>10</v>
       </c>
-      <c r="R4" s="57"/>
-      <c r="S4" s="57"/>
-      <c r="T4" s="55" t="s">
+      <c r="R4" s="36"/>
+      <c r="S4" s="36"/>
+      <c r="T4" s="62" t="s">
         <v>18</v>
       </c>
-      <c r="U4" s="55"/>
-      <c r="V4" s="82"/>
-      <c r="W4" s="73" t="s">
+      <c r="U4" s="62"/>
+      <c r="V4" s="63"/>
+      <c r="W4" s="79" t="s">
         <v>11</v>
       </c>
-      <c r="X4" s="57"/>
-      <c r="Y4" s="57"/>
-      <c r="Z4" s="66" t="s">
+      <c r="X4" s="36"/>
+      <c r="Y4" s="36"/>
+      <c r="Z4" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="AA4" s="67"/>
-      <c r="AB4" s="68"/>
-      <c r="AC4" s="66" t="s">
+      <c r="AA4" s="72"/>
+      <c r="AB4" s="73"/>
+      <c r="AC4" s="71" t="s">
         <v>23</v>
       </c>
-      <c r="AD4" s="67"/>
-      <c r="AE4" s="68"/>
+      <c r="AD4" s="72"/>
+      <c r="AE4" s="73"/>
     </row>
     <row r="5" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="D5" s="57"/>
-      <c r="E5" s="57"/>
-      <c r="F5" s="57"/>
-      <c r="G5" s="58"/>
-      <c r="H5" s="59"/>
-      <c r="I5" s="60"/>
-      <c r="J5" s="60"/>
-      <c r="K5" s="60"/>
-      <c r="L5" s="60"/>
-      <c r="M5" s="60"/>
-      <c r="N5" s="84"/>
-      <c r="O5" s="55"/>
-      <c r="P5" s="85"/>
-      <c r="Q5" s="83"/>
-      <c r="R5" s="57"/>
-      <c r="S5" s="57"/>
-      <c r="T5" s="55"/>
-      <c r="U5" s="55"/>
-      <c r="V5" s="82"/>
-      <c r="W5" s="73"/>
-      <c r="X5" s="57"/>
-      <c r="Y5" s="57"/>
-      <c r="Z5" s="69"/>
-      <c r="AA5" s="56"/>
-      <c r="AB5" s="47"/>
-      <c r="AC5" s="69"/>
-      <c r="AD5" s="56"/>
-      <c r="AE5" s="47"/>
+      <c r="D5" s="36"/>
+      <c r="E5" s="36"/>
+      <c r="F5" s="36"/>
+      <c r="G5" s="37"/>
+      <c r="H5" s="80"/>
+      <c r="I5" s="65"/>
+      <c r="J5" s="65"/>
+      <c r="K5" s="65"/>
+      <c r="L5" s="65"/>
+      <c r="M5" s="65"/>
+      <c r="N5" s="66"/>
+      <c r="O5" s="62"/>
+      <c r="P5" s="67"/>
+      <c r="Q5" s="64"/>
+      <c r="R5" s="36"/>
+      <c r="S5" s="36"/>
+      <c r="T5" s="62"/>
+      <c r="U5" s="62"/>
+      <c r="V5" s="63"/>
+      <c r="W5" s="79"/>
+      <c r="X5" s="36"/>
+      <c r="Y5" s="36"/>
+      <c r="Z5" s="74"/>
+      <c r="AA5" s="75"/>
+      <c r="AB5" s="50"/>
+      <c r="AC5" s="74"/>
+      <c r="AD5" s="75"/>
+      <c r="AE5" s="50"/>
     </row>
     <row r="6" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="D6" s="57"/>
-      <c r="E6" s="57"/>
-      <c r="F6" s="57"/>
-      <c r="G6" s="58"/>
-      <c r="H6" s="59"/>
-      <c r="I6" s="60"/>
-      <c r="J6" s="60"/>
-      <c r="K6" s="60"/>
-      <c r="L6" s="60"/>
-      <c r="M6" s="60"/>
-      <c r="N6" s="84"/>
-      <c r="O6" s="55"/>
-      <c r="P6" s="85"/>
-      <c r="Q6" s="83"/>
-      <c r="R6" s="57"/>
-      <c r="S6" s="57"/>
-      <c r="T6" s="55"/>
-      <c r="U6" s="55"/>
-      <c r="V6" s="82"/>
-      <c r="W6" s="73"/>
-      <c r="X6" s="57"/>
-      <c r="Y6" s="57"/>
-      <c r="Z6" s="70"/>
-      <c r="AA6" s="71"/>
-      <c r="AB6" s="72"/>
-      <c r="AC6" s="70"/>
-      <c r="AD6" s="71"/>
-      <c r="AE6" s="72"/>
+      <c r="D6" s="36"/>
+      <c r="E6" s="36"/>
+      <c r="F6" s="36"/>
+      <c r="G6" s="37"/>
+      <c r="H6" s="80"/>
+      <c r="I6" s="65"/>
+      <c r="J6" s="65"/>
+      <c r="K6" s="65"/>
+      <c r="L6" s="65"/>
+      <c r="M6" s="65"/>
+      <c r="N6" s="66"/>
+      <c r="O6" s="62"/>
+      <c r="P6" s="67"/>
+      <c r="Q6" s="64"/>
+      <c r="R6" s="36"/>
+      <c r="S6" s="36"/>
+      <c r="T6" s="62"/>
+      <c r="U6" s="62"/>
+      <c r="V6" s="63"/>
+      <c r="W6" s="79"/>
+      <c r="X6" s="36"/>
+      <c r="Y6" s="36"/>
+      <c r="Z6" s="76"/>
+      <c r="AA6" s="77"/>
+      <c r="AB6" s="78"/>
+      <c r="AC6" s="76"/>
+      <c r="AD6" s="77"/>
+      <c r="AE6" s="78"/>
     </row>
     <row r="7" spans="4:31" ht="20.399999999999999" x14ac:dyDescent="0.3">
-      <c r="D7" s="57" t="s">
-        <v>4</v>
-      </c>
-      <c r="E7" s="57"/>
-      <c r="F7" s="57" t="s">
+      <c r="D7" s="36" t="s">
+        <v>4</v>
+      </c>
+      <c r="E7" s="36"/>
+      <c r="F7" s="36" t="s">
         <v>5</v>
       </c>
-      <c r="G7" s="58"/>
+      <c r="G7" s="37"/>
       <c r="H7" s="11" t="s">
         <v>0</v>
       </c>
@@ -1817,14 +1875,14 @@
       </c>
     </row>
     <row r="8" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="D8" s="57">
-        <v>8</v>
-      </c>
-      <c r="E8" s="57"/>
-      <c r="F8" s="57">
-        <v>8</v>
-      </c>
-      <c r="G8" s="58"/>
+      <c r="D8" s="36">
+        <v>8</v>
+      </c>
+      <c r="E8" s="36"/>
+      <c r="F8" s="36">
+        <v>8</v>
+      </c>
+      <c r="G8" s="37"/>
       <c r="H8" s="11">
         <v>331</v>
       </c>
@@ -1899,14 +1957,14 @@
       </c>
     </row>
     <row r="9" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="D9" s="57">
+      <c r="D9" s="36">
         <v>10</v>
       </c>
-      <c r="E9" s="57"/>
-      <c r="F9" s="57">
+      <c r="E9" s="36"/>
+      <c r="F9" s="36">
         <v>16</v>
       </c>
-      <c r="G9" s="58"/>
+      <c r="G9" s="37"/>
       <c r="H9" s="11">
         <v>504</v>
       </c>
@@ -1981,14 +2039,14 @@
       </c>
     </row>
     <row r="10" spans="4:31" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D10" s="57">
+      <c r="D10" s="36">
         <v>10</v>
       </c>
-      <c r="E10" s="57"/>
-      <c r="F10" s="57">
+      <c r="E10" s="36"/>
+      <c r="F10" s="36">
         <v>32</v>
       </c>
-      <c r="G10" s="58"/>
+      <c r="G10" s="37"/>
       <c r="H10" s="13">
         <v>761</v>
       </c>
@@ -2063,17 +2121,17 @@
       </c>
     </row>
     <row r="11" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="H11" s="80" t="s">
+      <c r="H11" s="59" t="s">
         <v>24</v>
       </c>
-      <c r="I11" s="80"/>
-      <c r="J11" s="80"/>
-      <c r="K11" s="80"/>
-      <c r="L11" s="80"/>
-      <c r="M11" s="80"/>
-      <c r="N11" s="80"/>
-      <c r="O11" s="80"/>
-      <c r="P11" s="80"/>
+      <c r="I11" s="59"/>
+      <c r="J11" s="59"/>
+      <c r="K11" s="59"/>
+      <c r="L11" s="59"/>
+      <c r="M11" s="59"/>
+      <c r="N11" s="59"/>
+      <c r="O11" s="59"/>
+      <c r="P11" s="59"/>
     </row>
     <row r="12" spans="4:31" ht="23.4" x14ac:dyDescent="0.3">
       <c r="O12" s="19" t="s">
@@ -2081,103 +2139,103 @@
       </c>
     </row>
     <row r="13" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="N13" s="56" t="s">
+      <c r="N13" s="75" t="s">
         <v>19</v>
       </c>
-      <c r="O13" s="56"/>
-      <c r="P13" s="56"/>
+      <c r="O13" s="75"/>
+      <c r="P13" s="75"/>
     </row>
     <row r="14" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="N14" s="56"/>
-      <c r="O14" s="56"/>
-      <c r="P14" s="56"/>
+      <c r="N14" s="75"/>
+      <c r="O14" s="75"/>
+      <c r="P14" s="75"/>
     </row>
     <row r="15" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="N15" s="56"/>
-      <c r="O15" s="56"/>
-      <c r="P15" s="56"/>
+      <c r="N15" s="75"/>
+      <c r="O15" s="75"/>
+      <c r="P15" s="75"/>
     </row>
     <row r="17" spans="5:36" x14ac:dyDescent="0.3">
-      <c r="H17" s="57" t="s">
+      <c r="H17" s="36" t="s">
         <v>26</v>
       </c>
-      <c r="I17" s="57"/>
-      <c r="J17" s="57"/>
-      <c r="K17" s="57" t="s">
+      <c r="I17" s="36"/>
+      <c r="J17" s="36"/>
+      <c r="K17" s="36" t="s">
         <v>26</v>
       </c>
-      <c r="L17" s="57"/>
-      <c r="M17" s="57"/>
+      <c r="L17" s="36"/>
+      <c r="M17" s="36"/>
       <c r="S17"/>
       <c r="T17"/>
       <c r="U17"/>
     </row>
     <row r="18" spans="5:36" x14ac:dyDescent="0.3">
-      <c r="H18" s="55" t="s">
+      <c r="H18" s="62" t="s">
         <v>28</v>
       </c>
-      <c r="I18" s="55"/>
-      <c r="J18" s="55"/>
-      <c r="K18" s="55" t="s">
+      <c r="I18" s="62"/>
+      <c r="J18" s="62"/>
+      <c r="K18" s="62" t="s">
         <v>29</v>
       </c>
-      <c r="L18" s="55"/>
-      <c r="M18" s="55"/>
-      <c r="S18" s="55" t="s">
+      <c r="L18" s="62"/>
+      <c r="M18" s="62"/>
+      <c r="S18" s="62" t="s">
         <v>32</v>
       </c>
-      <c r="T18" s="55"/>
-      <c r="U18" s="55"/>
-      <c r="AA18" s="55" t="s">
+      <c r="T18" s="62"/>
+      <c r="U18" s="62"/>
+      <c r="AA18" s="62" t="s">
         <v>35</v>
       </c>
-      <c r="AB18" s="55"/>
-      <c r="AC18" s="55"/>
-      <c r="AH18" s="55" t="s">
+      <c r="AB18" s="62"/>
+      <c r="AC18" s="62"/>
+      <c r="AH18" s="62" t="s">
         <v>36</v>
       </c>
-      <c r="AI18" s="55"/>
-      <c r="AJ18" s="55"/>
+      <c r="AI18" s="62"/>
+      <c r="AJ18" s="62"/>
     </row>
     <row r="19" spans="5:36" x14ac:dyDescent="0.3">
-      <c r="H19" s="55"/>
-      <c r="I19" s="55"/>
-      <c r="J19" s="55"/>
-      <c r="K19" s="55"/>
-      <c r="L19" s="55"/>
-      <c r="M19" s="55"/>
-      <c r="S19" s="55"/>
-      <c r="T19" s="55"/>
-      <c r="U19" s="55"/>
-      <c r="AA19" s="55"/>
-      <c r="AB19" s="55"/>
-      <c r="AC19" s="55"/>
-      <c r="AH19" s="55"/>
-      <c r="AI19" s="55"/>
-      <c r="AJ19" s="55"/>
+      <c r="H19" s="62"/>
+      <c r="I19" s="62"/>
+      <c r="J19" s="62"/>
+      <c r="K19" s="62"/>
+      <c r="L19" s="62"/>
+      <c r="M19" s="62"/>
+      <c r="S19" s="62"/>
+      <c r="T19" s="62"/>
+      <c r="U19" s="62"/>
+      <c r="AA19" s="62"/>
+      <c r="AB19" s="62"/>
+      <c r="AC19" s="62"/>
+      <c r="AH19" s="62"/>
+      <c r="AI19" s="62"/>
+      <c r="AJ19" s="62"/>
     </row>
     <row r="20" spans="5:36" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H20" s="55"/>
-      <c r="I20" s="55"/>
-      <c r="J20" s="55"/>
-      <c r="K20" s="55"/>
-      <c r="L20" s="55"/>
-      <c r="M20" s="55"/>
-      <c r="S20" s="55"/>
-      <c r="T20" s="55"/>
-      <c r="U20" s="55"/>
-      <c r="AA20" s="55"/>
-      <c r="AB20" s="55"/>
-      <c r="AC20" s="55"/>
-      <c r="AH20" s="55"/>
-      <c r="AI20" s="55"/>
-      <c r="AJ20" s="55"/>
+      <c r="H20" s="62"/>
+      <c r="I20" s="62"/>
+      <c r="J20" s="62"/>
+      <c r="K20" s="62"/>
+      <c r="L20" s="62"/>
+      <c r="M20" s="62"/>
+      <c r="S20" s="62"/>
+      <c r="T20" s="62"/>
+      <c r="U20" s="62"/>
+      <c r="AA20" s="62"/>
+      <c r="AB20" s="62"/>
+      <c r="AC20" s="62"/>
+      <c r="AH20" s="62"/>
+      <c r="AI20" s="62"/>
+      <c r="AJ20" s="62"/>
     </row>
     <row r="21" spans="5:36" ht="20.399999999999999" x14ac:dyDescent="0.3">
-      <c r="E21" s="55" t="s">
+      <c r="E21" s="62" t="s">
         <v>30</v>
       </c>
-      <c r="F21" s="55"/>
+      <c r="F21" s="62"/>
       <c r="G21" s="2" t="s">
         <v>27</v>
       </c>
@@ -2199,10 +2257,10 @@
       <c r="M21" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="O21" s="55" t="s">
+      <c r="O21" s="62" t="s">
         <v>34</v>
       </c>
-      <c r="P21" s="55"/>
+      <c r="P21" s="62"/>
       <c r="Q21" s="18" t="s">
         <v>33</v>
       </c>
@@ -2219,10 +2277,10 @@
         <v>2</v>
       </c>
       <c r="W21"/>
-      <c r="X21" s="55" t="s">
+      <c r="X21" s="62" t="s">
         <v>34</v>
       </c>
-      <c r="Y21" s="55"/>
+      <c r="Y21" s="62"/>
       <c r="Z21" s="2" t="s">
         <v>31</v>
       </c>
@@ -2235,10 +2293,10 @@
       <c r="AC21" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="AE21" s="55" t="s">
+      <c r="AE21" s="62" t="s">
         <v>37</v>
       </c>
-      <c r="AF21" s="55"/>
+      <c r="AF21" s="62"/>
       <c r="AG21" s="18" t="s">
         <v>38</v>
       </c>
@@ -2253,8 +2311,8 @@
       </c>
     </row>
     <row r="22" spans="5:36" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E22" s="55"/>
-      <c r="F22" s="55"/>
+      <c r="E22" s="62"/>
+      <c r="F22" s="62"/>
       <c r="G22" s="2">
         <v>4</v>
       </c>
@@ -2276,8 +2334,8 @@
       <c r="M22" s="2">
         <v>578</v>
       </c>
-      <c r="O22" s="55"/>
-      <c r="P22" s="55"/>
+      <c r="O22" s="62"/>
+      <c r="P22" s="62"/>
       <c r="Q22" s="18">
         <v>8</v>
       </c>
@@ -2294,8 +2352,8 @@
         <v>455</v>
       </c>
       <c r="W22"/>
-      <c r="X22" s="55"/>
-      <c r="Y22" s="55"/>
+      <c r="X22" s="62"/>
+      <c r="Y22" s="62"/>
       <c r="Z22" s="2">
         <v>4</v>
       </c>
@@ -2308,8 +2366,8 @@
       <c r="AC22" s="2">
         <v>555</v>
       </c>
-      <c r="AE22" s="55"/>
-      <c r="AF22" s="55"/>
+      <c r="AE22" s="62"/>
+      <c r="AF22" s="62"/>
       <c r="AG22" s="2">
         <v>2</v>
       </c>
@@ -2324,8 +2382,8 @@
       </c>
     </row>
     <row r="23" spans="5:36" x14ac:dyDescent="0.3">
-      <c r="E23" s="55"/>
-      <c r="F23" s="55"/>
+      <c r="E23" s="62"/>
+      <c r="F23" s="62"/>
       <c r="G23" s="2">
         <v>8</v>
       </c>
@@ -2347,8 +2405,8 @@
       <c r="M23" s="2">
         <v>476</v>
       </c>
-      <c r="O23" s="55"/>
-      <c r="P23" s="55"/>
+      <c r="O23" s="62"/>
+      <c r="P23" s="62"/>
       <c r="Q23" s="18">
         <v>12</v>
       </c>
@@ -2365,8 +2423,8 @@
         <v>462</v>
       </c>
       <c r="W23"/>
-      <c r="X23" s="55"/>
-      <c r="Y23" s="55"/>
+      <c r="X23" s="62"/>
+      <c r="Y23" s="62"/>
       <c r="Z23" s="2">
         <v>8</v>
       </c>
@@ -2379,8 +2437,8 @@
       <c r="AC23" s="2">
         <v>542</v>
       </c>
-      <c r="AE23" s="55"/>
-      <c r="AF23" s="55"/>
+      <c r="AE23" s="62"/>
+      <c r="AF23" s="62"/>
       <c r="AG23" s="2">
         <v>4</v>
       </c>
@@ -2395,8 +2453,8 @@
       </c>
     </row>
     <row r="24" spans="5:36" x14ac:dyDescent="0.3">
-      <c r="E24" s="55"/>
-      <c r="F24" s="55"/>
+      <c r="E24" s="62"/>
+      <c r="F24" s="62"/>
       <c r="G24" s="2">
         <v>16</v>
       </c>
@@ -2418,8 +2476,8 @@
       <c r="M24" s="2">
         <v>387</v>
       </c>
-      <c r="O24" s="55"/>
-      <c r="P24" s="55"/>
+      <c r="O24" s="62"/>
+      <c r="P24" s="62"/>
       <c r="Q24" s="18">
         <v>16</v>
       </c>
@@ -2436,8 +2494,8 @@
         <v>390</v>
       </c>
       <c r="W24"/>
-      <c r="X24" s="55"/>
-      <c r="Y24" s="55"/>
+      <c r="X24" s="62"/>
+      <c r="Y24" s="62"/>
       <c r="Z24" s="2">
         <v>16</v>
       </c>
@@ -2450,8 +2508,8 @@
       <c r="AC24" s="2">
         <v>493</v>
       </c>
-      <c r="AE24" s="55"/>
-      <c r="AF24" s="55"/>
+      <c r="AE24" s="62"/>
+      <c r="AF24" s="62"/>
       <c r="AG24" s="2">
         <v>8</v>
       </c>
@@ -2467,80 +2525,80 @@
     </row>
     <row r="26" spans="5:36" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="27" spans="5:36" x14ac:dyDescent="0.3">
-      <c r="E27" s="35" t="s">
+      <c r="E27" s="38" t="s">
         <v>39</v>
       </c>
-      <c r="F27" s="36"/>
-      <c r="G27" s="36"/>
-      <c r="H27" s="36"/>
-      <c r="I27" s="36"/>
-      <c r="J27" s="36"/>
-      <c r="K27" s="36"/>
-      <c r="L27" s="36"/>
-      <c r="M27" s="36"/>
-      <c r="N27" s="37"/>
-      <c r="S27" s="35" t="s">
+      <c r="F27" s="39"/>
+      <c r="G27" s="39"/>
+      <c r="H27" s="39"/>
+      <c r="I27" s="39"/>
+      <c r="J27" s="39"/>
+      <c r="K27" s="39"/>
+      <c r="L27" s="39"/>
+      <c r="M27" s="39"/>
+      <c r="N27" s="40"/>
+      <c r="S27" s="38" t="s">
         <v>39</v>
       </c>
-      <c r="T27" s="36"/>
-      <c r="U27" s="36"/>
-      <c r="V27" s="36"/>
-      <c r="W27" s="36"/>
-      <c r="X27" s="36"/>
-      <c r="Y27" s="36"/>
-      <c r="Z27" s="36"/>
-      <c r="AA27" s="36"/>
-      <c r="AB27" s="37"/>
+      <c r="T27" s="39"/>
+      <c r="U27" s="39"/>
+      <c r="V27" s="39"/>
+      <c r="W27" s="39"/>
+      <c r="X27" s="39"/>
+      <c r="Y27" s="39"/>
+      <c r="Z27" s="39"/>
+      <c r="AA27" s="39"/>
+      <c r="AB27" s="40"/>
     </row>
     <row r="28" spans="5:36" x14ac:dyDescent="0.3">
-      <c r="E28" s="38"/>
-      <c r="F28" s="39"/>
-      <c r="G28" s="39"/>
-      <c r="H28" s="39"/>
-      <c r="I28" s="39"/>
-      <c r="J28" s="39"/>
-      <c r="K28" s="39"/>
-      <c r="L28" s="39"/>
-      <c r="M28" s="39"/>
-      <c r="N28" s="40"/>
-      <c r="S28" s="38"/>
-      <c r="T28" s="39"/>
-      <c r="U28" s="39"/>
-      <c r="V28" s="39"/>
-      <c r="W28" s="39"/>
-      <c r="X28" s="39"/>
-      <c r="Y28" s="39"/>
-      <c r="Z28" s="39"/>
-      <c r="AA28" s="39"/>
-      <c r="AB28" s="40"/>
+      <c r="E28" s="41"/>
+      <c r="F28" s="42"/>
+      <c r="G28" s="42"/>
+      <c r="H28" s="42"/>
+      <c r="I28" s="42"/>
+      <c r="J28" s="42"/>
+      <c r="K28" s="42"/>
+      <c r="L28" s="42"/>
+      <c r="M28" s="42"/>
+      <c r="N28" s="43"/>
+      <c r="S28" s="41"/>
+      <c r="T28" s="42"/>
+      <c r="U28" s="42"/>
+      <c r="V28" s="42"/>
+      <c r="W28" s="42"/>
+      <c r="X28" s="42"/>
+      <c r="Y28" s="42"/>
+      <c r="Z28" s="42"/>
+      <c r="AA28" s="42"/>
+      <c r="AB28" s="43"/>
     </row>
     <row r="29" spans="5:36" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E29" s="50"/>
-      <c r="F29" s="51"/>
-      <c r="G29" s="51"/>
-      <c r="H29" s="51"/>
-      <c r="I29" s="51"/>
-      <c r="J29" s="51"/>
-      <c r="K29" s="51"/>
-      <c r="L29" s="51"/>
-      <c r="M29" s="51"/>
-      <c r="N29" s="52"/>
-      <c r="S29" s="50"/>
-      <c r="T29" s="51"/>
-      <c r="U29" s="51"/>
-      <c r="V29" s="51"/>
-      <c r="W29" s="51"/>
-      <c r="X29" s="51"/>
-      <c r="Y29" s="51"/>
-      <c r="Z29" s="51"/>
-      <c r="AA29" s="51"/>
-      <c r="AB29" s="52"/>
+      <c r="E29" s="84"/>
+      <c r="F29" s="85"/>
+      <c r="G29" s="85"/>
+      <c r="H29" s="85"/>
+      <c r="I29" s="85"/>
+      <c r="J29" s="85"/>
+      <c r="K29" s="85"/>
+      <c r="L29" s="85"/>
+      <c r="M29" s="85"/>
+      <c r="N29" s="86"/>
+      <c r="S29" s="84"/>
+      <c r="T29" s="85"/>
+      <c r="U29" s="85"/>
+      <c r="V29" s="85"/>
+      <c r="W29" s="85"/>
+      <c r="X29" s="85"/>
+      <c r="Y29" s="85"/>
+      <c r="Z29" s="85"/>
+      <c r="AA29" s="85"/>
+      <c r="AB29" s="86"/>
     </row>
     <row r="30" spans="5:36" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E30" s="44" t="s">
+      <c r="E30" s="47" t="s">
         <v>44</v>
       </c>
-      <c r="F30" s="45"/>
+      <c r="F30" s="48"/>
       <c r="G30" s="24" t="s">
         <v>33</v>
       </c>
@@ -2565,10 +2623,10 @@
       <c r="N30" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="S30" s="44" t="s">
+      <c r="S30" s="47" t="s">
         <v>44</v>
       </c>
-      <c r="T30" s="45"/>
+      <c r="T30" s="48"/>
       <c r="U30" s="24" t="s">
         <v>33</v>
       </c>
@@ -2595,8 +2653,8 @@
       </c>
     </row>
     <row r="31" spans="5:36" x14ac:dyDescent="0.3">
-      <c r="E31" s="46"/>
-      <c r="F31" s="47"/>
+      <c r="E31" s="49"/>
+      <c r="F31" s="50"/>
       <c r="G31" s="23">
         <v>4</v>
       </c>
@@ -2621,8 +2679,8 @@
       <c r="N31" s="5">
         <v>479</v>
       </c>
-      <c r="S31" s="46"/>
-      <c r="T31" s="47"/>
+      <c r="S31" s="49"/>
+      <c r="T31" s="50"/>
       <c r="U31" s="23">
         <v>4</v>
       </c>
@@ -2649,8 +2707,8 @@
       </c>
     </row>
     <row r="32" spans="5:36" x14ac:dyDescent="0.3">
-      <c r="E32" s="46"/>
-      <c r="F32" s="47"/>
+      <c r="E32" s="49"/>
+      <c r="F32" s="50"/>
       <c r="G32" s="23">
         <v>4</v>
       </c>
@@ -2675,8 +2733,8 @@
       <c r="N32" s="5">
         <v>300</v>
       </c>
-      <c r="S32" s="46"/>
-      <c r="T32" s="47"/>
+      <c r="S32" s="49"/>
+      <c r="T32" s="50"/>
       <c r="U32" s="23">
         <v>4</v>
       </c>
@@ -2702,9 +2760,9 @@
         <v>315</v>
       </c>
     </row>
-    <row r="33" spans="5:30" x14ac:dyDescent="0.3">
-      <c r="E33" s="46"/>
-      <c r="F33" s="47"/>
+    <row r="33" spans="5:31" x14ac:dyDescent="0.3">
+      <c r="E33" s="49"/>
+      <c r="F33" s="50"/>
       <c r="G33" s="23">
         <v>4</v>
       </c>
@@ -2729,8 +2787,8 @@
       <c r="N33" s="5">
         <v>276</v>
       </c>
-      <c r="S33" s="46"/>
-      <c r="T33" s="47"/>
+      <c r="S33" s="49"/>
+      <c r="T33" s="50"/>
       <c r="U33" s="23">
         <v>4</v>
       </c>
@@ -2756,9 +2814,9 @@
         <v>305</v>
       </c>
     </row>
-    <row r="34" spans="5:30" x14ac:dyDescent="0.3">
-      <c r="E34" s="46"/>
-      <c r="F34" s="47"/>
+    <row r="34" spans="5:31" x14ac:dyDescent="0.3">
+      <c r="E34" s="49"/>
+      <c r="F34" s="50"/>
       <c r="G34" s="23">
         <v>4</v>
       </c>
@@ -2783,8 +2841,8 @@
       <c r="N34" s="5">
         <v>290</v>
       </c>
-      <c r="S34" s="46"/>
-      <c r="T34" s="47"/>
+      <c r="S34" s="49"/>
+      <c r="T34" s="50"/>
       <c r="U34" s="23">
         <v>4</v>
       </c>
@@ -2810,9 +2868,9 @@
         <v>304</v>
       </c>
     </row>
-    <row r="35" spans="5:30" x14ac:dyDescent="0.3">
-      <c r="E35" s="46"/>
-      <c r="F35" s="47"/>
+    <row r="35" spans="5:31" x14ac:dyDescent="0.3">
+      <c r="E35" s="49"/>
+      <c r="F35" s="50"/>
       <c r="G35" s="23">
         <v>8</v>
       </c>
@@ -2837,8 +2895,8 @@
       <c r="N35" s="5">
         <v>320</v>
       </c>
-      <c r="S35" s="46"/>
-      <c r="T35" s="47"/>
+      <c r="S35" s="49"/>
+      <c r="T35" s="50"/>
       <c r="U35" s="23">
         <v>8</v>
       </c>
@@ -2864,9 +2922,9 @@
         <v>320</v>
       </c>
     </row>
-    <row r="36" spans="5:30" ht="20.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E36" s="46"/>
-      <c r="F36" s="47"/>
+    <row r="36" spans="5:31" ht="20.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E36" s="49"/>
+      <c r="F36" s="50"/>
       <c r="G36" s="23">
         <v>8</v>
       </c>
@@ -2891,8 +2949,8 @@
       <c r="N36" s="5">
         <v>291</v>
       </c>
-      <c r="S36" s="46"/>
-      <c r="T36" s="47"/>
+      <c r="S36" s="49"/>
+      <c r="T36" s="50"/>
       <c r="U36" s="23">
         <v>8</v>
       </c>
@@ -2918,9 +2976,9 @@
         <v>297</v>
       </c>
     </row>
-    <row r="37" spans="5:30" ht="20.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E37" s="48"/>
-      <c r="F37" s="49"/>
+    <row r="37" spans="5:31" ht="20.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E37" s="51"/>
+      <c r="F37" s="52"/>
       <c r="G37" s="25">
         <v>12</v>
       </c>
@@ -2946,8 +3004,8 @@
         <v>304</v>
       </c>
       <c r="Q37"/>
-      <c r="S37" s="48"/>
-      <c r="T37" s="49"/>
+      <c r="S37" s="51"/>
+      <c r="T37" s="52"/>
       <c r="U37" s="25">
         <v>12</v>
       </c>
@@ -2972,16 +3030,16 @@
       <c r="AB37" s="8">
         <v>304</v>
       </c>
-      <c r="AC37" s="53" t="s">
+      <c r="AC37" s="82" t="s">
         <v>48</v>
       </c>
-      <c r="AD37" s="54"/>
-    </row>
-    <row r="38" spans="5:30" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E38" s="46" t="s">
+      <c r="AD37" s="83"/>
+    </row>
+    <row r="38" spans="5:31" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E38" s="49" t="s">
         <v>47</v>
       </c>
-      <c r="F38" s="47"/>
+      <c r="F38" s="50"/>
       <c r="G38" s="24" t="s">
         <v>33</v>
       </c>
@@ -3013,10 +3071,10 @@
         <v>46</v>
       </c>
       <c r="Q38"/>
-      <c r="S38" s="46" t="s">
+      <c r="S38" s="49" t="s">
         <v>47</v>
       </c>
-      <c r="T38" s="47"/>
+      <c r="T38" s="50"/>
       <c r="U38" s="24" t="s">
         <v>33</v>
       </c>
@@ -3048,9 +3106,9 @@
         <v>46</v>
       </c>
     </row>
-    <row r="39" spans="5:30" x14ac:dyDescent="0.3">
-      <c r="E39" s="46"/>
-      <c r="F39" s="47"/>
+    <row r="39" spans="5:31" x14ac:dyDescent="0.3">
+      <c r="E39" s="49"/>
+      <c r="F39" s="50"/>
       <c r="G39" s="23">
         <v>4</v>
       </c>
@@ -3084,8 +3142,8 @@
         <v>17.056856187290968</v>
       </c>
       <c r="Q39"/>
-      <c r="S39" s="46"/>
-      <c r="T39" s="47"/>
+      <c r="S39" s="49"/>
+      <c r="T39" s="50"/>
       <c r="U39" s="23">
         <v>4</v>
       </c>
@@ -3119,9 +3177,9 @@
         <v>17.056856187290968</v>
       </c>
     </row>
-    <row r="40" spans="5:30" x14ac:dyDescent="0.3">
-      <c r="E40" s="46"/>
-      <c r="F40" s="47"/>
+    <row r="40" spans="5:31" x14ac:dyDescent="0.3">
+      <c r="E40" s="49"/>
+      <c r="F40" s="50"/>
       <c r="G40" s="23">
         <v>4</v>
       </c>
@@ -3155,8 +3213,8 @@
         <v>9.6440035016049013</v>
       </c>
       <c r="Q40"/>
-      <c r="S40" s="46"/>
-      <c r="T40" s="47"/>
+      <c r="S40" s="49"/>
+      <c r="T40" s="50"/>
       <c r="U40" s="23">
         <v>4</v>
       </c>
@@ -3190,9 +3248,9 @@
         <v>9.6440035016049013</v>
       </c>
     </row>
-    <row r="41" spans="5:30" x14ac:dyDescent="0.3">
-      <c r="E41" s="46"/>
-      <c r="F41" s="47"/>
+    <row r="41" spans="5:31" x14ac:dyDescent="0.3">
+      <c r="E41" s="49"/>
+      <c r="F41" s="50"/>
       <c r="G41" s="23">
         <v>4</v>
       </c>
@@ -3226,8 +3284,8 @@
         <v>9.1386861313868604</v>
       </c>
       <c r="Q41"/>
-      <c r="S41" s="46"/>
-      <c r="T41" s="47"/>
+      <c r="S41" s="49"/>
+      <c r="T41" s="50"/>
       <c r="U41" s="23">
         <v>4</v>
       </c>
@@ -3261,9 +3319,9 @@
         <v>9.1386861313868604</v>
       </c>
     </row>
-    <row r="42" spans="5:30" x14ac:dyDescent="0.3">
-      <c r="E42" s="46"/>
-      <c r="F42" s="47"/>
+    <row r="42" spans="5:31" x14ac:dyDescent="0.3">
+      <c r="E42" s="49"/>
+      <c r="F42" s="50"/>
       <c r="G42" s="23">
         <v>4</v>
       </c>
@@ -3296,8 +3354,8 @@
         <f t="shared" si="1"/>
         <v>0.54248248607867799</v>
       </c>
-      <c r="S42" s="46"/>
-      <c r="T42" s="47"/>
+      <c r="S42" s="49"/>
+      <c r="T42" s="50"/>
       <c r="U42" s="23">
         <v>4</v>
       </c>
@@ -3331,9 +3389,9 @@
         <v>0.54248248607867799</v>
       </c>
     </row>
-    <row r="43" spans="5:30" x14ac:dyDescent="0.3">
-      <c r="E43" s="46"/>
-      <c r="F43" s="47"/>
+    <row r="43" spans="5:31" x14ac:dyDescent="0.3">
+      <c r="E43" s="49"/>
+      <c r="F43" s="50"/>
       <c r="G43" s="23">
         <v>8</v>
       </c>
@@ -3366,8 +3424,8 @@
         <f t="shared" si="1"/>
         <v>0.28200185621474977</v>
       </c>
-      <c r="S43" s="46"/>
-      <c r="T43" s="47"/>
+      <c r="S43" s="49"/>
+      <c r="T43" s="50"/>
       <c r="U43" s="23">
         <v>8</v>
       </c>
@@ -3401,9 +3459,9 @@
         <v>0.28200185621474977</v>
       </c>
     </row>
-    <row r="44" spans="5:30" x14ac:dyDescent="0.3">
-      <c r="E44" s="46"/>
-      <c r="F44" s="47"/>
+    <row r="44" spans="5:31" x14ac:dyDescent="0.3">
+      <c r="E44" s="49"/>
+      <c r="F44" s="50"/>
       <c r="G44" s="23">
         <v>8</v>
       </c>
@@ -3436,8 +3494,8 @@
         <f t="shared" si="1"/>
         <v>-5.6277056277056277</v>
       </c>
-      <c r="S44" s="46"/>
-      <c r="T44" s="47"/>
+      <c r="S44" s="49"/>
+      <c r="T44" s="50"/>
       <c r="U44" s="23">
         <v>8</v>
       </c>
@@ -3471,9 +3529,9 @@
         <v>-5.6277056277056277</v>
       </c>
     </row>
-    <row r="45" spans="5:30" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E45" s="48"/>
-      <c r="F45" s="49"/>
+    <row r="45" spans="5:31" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E45" s="51"/>
+      <c r="F45" s="52"/>
       <c r="G45" s="25">
         <v>12</v>
       </c>
@@ -3506,8 +3564,8 @@
         <f t="shared" si="1"/>
         <v>-61.256930870796602</v>
       </c>
-      <c r="S45" s="48"/>
-      <c r="T45" s="49"/>
+      <c r="S45" s="51"/>
+      <c r="T45" s="52"/>
       <c r="U45" s="25">
         <v>12</v>
       </c>
@@ -3541,70 +3599,99 @@
         <v>-61.256930870796602</v>
       </c>
     </row>
-    <row r="47" spans="5:30" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="48" spans="5:30" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E48" s="35" t="s">
+    <row r="47" spans="5:31" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="48" spans="5:31" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E48" s="38" t="s">
         <v>49</v>
       </c>
-      <c r="F48" s="36"/>
-      <c r="G48" s="36"/>
-      <c r="H48" s="36"/>
-      <c r="I48" s="36"/>
-      <c r="J48" s="36"/>
-      <c r="K48" s="37"/>
+      <c r="F48" s="39"/>
+      <c r="G48" s="39"/>
+      <c r="H48" s="39"/>
+      <c r="I48" s="39"/>
+      <c r="J48" s="39"/>
+      <c r="K48" s="40"/>
       <c r="L48"/>
       <c r="M48"/>
-      <c r="N48" s="35" t="s">
+      <c r="N48" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="O48" s="36"/>
-      <c r="P48" s="36"/>
-      <c r="Q48" s="36"/>
-      <c r="R48" s="36"/>
-      <c r="S48" s="36"/>
-      <c r="T48" s="37"/>
-    </row>
-    <row r="49" spans="5:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E49" s="38"/>
-      <c r="F49" s="39"/>
-      <c r="G49" s="39"/>
-      <c r="H49" s="39"/>
-      <c r="I49" s="39"/>
-      <c r="J49" s="39"/>
-      <c r="K49" s="40"/>
+      <c r="O48" s="39"/>
+      <c r="P48" s="39"/>
+      <c r="Q48" s="39"/>
+      <c r="R48" s="39"/>
+      <c r="S48" s="39"/>
+      <c r="T48" s="40"/>
+      <c r="W48" s="91" t="s">
+        <v>57</v>
+      </c>
+      <c r="X48" s="92"/>
+      <c r="Y48" s="92"/>
+      <c r="Z48" s="92"/>
+      <c r="AA48" s="92"/>
+      <c r="AB48" s="92"/>
+      <c r="AC48" s="92"/>
+      <c r="AD48" s="92"/>
+      <c r="AE48" s="93"/>
+    </row>
+    <row r="49" spans="5:31" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E49" s="41"/>
+      <c r="F49" s="42"/>
+      <c r="G49" s="42"/>
+      <c r="H49" s="42"/>
+      <c r="I49" s="42"/>
+      <c r="J49" s="42"/>
+      <c r="K49" s="43"/>
       <c r="L49"/>
       <c r="M49"/>
-      <c r="N49" s="38"/>
-      <c r="O49" s="39"/>
-      <c r="P49" s="39"/>
-      <c r="Q49" s="39"/>
-      <c r="R49" s="39"/>
-      <c r="S49" s="39"/>
-      <c r="T49" s="40"/>
-    </row>
-    <row r="50" spans="5:20" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E50" s="41"/>
-      <c r="F50" s="42"/>
-      <c r="G50" s="42"/>
-      <c r="H50" s="42"/>
-      <c r="I50" s="42"/>
-      <c r="J50" s="42"/>
-      <c r="K50" s="43"/>
+      <c r="N49" s="41"/>
+      <c r="O49" s="42"/>
+      <c r="P49" s="42"/>
+      <c r="Q49" s="42"/>
+      <c r="R49" s="42"/>
+      <c r="S49" s="42"/>
+      <c r="T49" s="43"/>
+      <c r="W49" s="87"/>
+      <c r="X49" s="88"/>
+      <c r="Y49" s="88"/>
+      <c r="Z49" s="88"/>
+      <c r="AA49" s="88"/>
+      <c r="AB49" s="88"/>
+      <c r="AC49" s="88"/>
+      <c r="AD49" s="88"/>
+      <c r="AE49" s="94"/>
+    </row>
+    <row r="50" spans="5:31" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E50" s="44"/>
+      <c r="F50" s="45"/>
+      <c r="G50" s="45"/>
+      <c r="H50" s="45"/>
+      <c r="I50" s="45"/>
+      <c r="J50" s="45"/>
+      <c r="K50" s="46"/>
       <c r="L50"/>
       <c r="M50"/>
-      <c r="N50" s="41"/>
-      <c r="O50" s="42"/>
-      <c r="P50" s="42"/>
-      <c r="Q50" s="42"/>
-      <c r="R50" s="42"/>
-      <c r="S50" s="42"/>
-      <c r="T50" s="43"/>
-    </row>
-    <row r="51" spans="5:20" ht="20.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E51" s="44" t="s">
+      <c r="N50" s="44"/>
+      <c r="O50" s="45"/>
+      <c r="P50" s="45"/>
+      <c r="Q50" s="45"/>
+      <c r="R50" s="45"/>
+      <c r="S50" s="45"/>
+      <c r="T50" s="46"/>
+      <c r="W50" s="89"/>
+      <c r="X50" s="90"/>
+      <c r="Y50" s="90"/>
+      <c r="Z50" s="90"/>
+      <c r="AA50" s="90"/>
+      <c r="AB50" s="90"/>
+      <c r="AC50" s="90"/>
+      <c r="AD50" s="90"/>
+      <c r="AE50" s="95"/>
+    </row>
+    <row r="51" spans="5:31" ht="20.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E51" s="47" t="s">
         <v>34</v>
       </c>
-      <c r="F51" s="45"/>
+      <c r="F51" s="48"/>
       <c r="G51" s="32" t="s">
         <v>33</v>
       </c>
@@ -3620,10 +3707,10 @@
       <c r="K51" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="N51" s="44" t="s">
+      <c r="N51" s="47" t="s">
         <v>52</v>
       </c>
-      <c r="O51" s="45"/>
+      <c r="O51" s="48"/>
       <c r="P51" s="32" t="s">
         <v>33</v>
       </c>
@@ -3639,11 +3726,36 @@
       <c r="T51" s="34" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="52" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E52" s="46"/>
-      <c r="F52" s="47"/>
-      <c r="G52" s="86">
+      <c r="W51" s="47" t="s">
+        <v>52</v>
+      </c>
+      <c r="X51" s="48"/>
+      <c r="Y51" s="32" t="s">
+        <v>54</v>
+      </c>
+      <c r="Z51" s="33" t="s">
+        <v>42</v>
+      </c>
+      <c r="AA51" s="33" t="s">
+        <v>55</v>
+      </c>
+      <c r="AB51" s="33" t="s">
+        <v>56</v>
+      </c>
+      <c r="AC51" s="33" t="s">
+        <v>0</v>
+      </c>
+      <c r="AD51" s="33" t="s">
+        <v>1</v>
+      </c>
+      <c r="AE51" s="34" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="52" spans="5:31" x14ac:dyDescent="0.3">
+      <c r="E52" s="49"/>
+      <c r="F52" s="50"/>
+      <c r="G52" s="35">
         <v>2</v>
       </c>
       <c r="H52" s="27">
@@ -3658,9 +3770,9 @@
       <c r="K52" s="28">
         <v>512</v>
       </c>
-      <c r="N52" s="46"/>
-      <c r="O52" s="47"/>
-      <c r="P52" s="86">
+      <c r="N52" s="49"/>
+      <c r="O52" s="50"/>
+      <c r="P52" s="35">
         <v>2</v>
       </c>
       <c r="Q52" s="27">
@@ -3675,10 +3787,33 @@
       <c r="T52" s="28">
         <v>578</v>
       </c>
-    </row>
-    <row r="53" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E53" s="46"/>
-      <c r="F53" s="47"/>
+      <c r="W52" s="49"/>
+      <c r="X52" s="50"/>
+      <c r="Y52" s="35">
+        <v>6</v>
+      </c>
+      <c r="Z52" s="27">
+        <v>4</v>
+      </c>
+      <c r="AA52" s="27">
+        <v>2</v>
+      </c>
+      <c r="AB52" s="27">
+        <v>4</v>
+      </c>
+      <c r="AC52" s="27">
+        <v>264</v>
+      </c>
+      <c r="AD52" s="27">
+        <v>317</v>
+      </c>
+      <c r="AE52" s="28">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="53" spans="5:31" x14ac:dyDescent="0.3">
+      <c r="E53" s="49"/>
+      <c r="F53" s="50"/>
       <c r="G53" s="4">
         <v>2</v>
       </c>
@@ -3694,8 +3829,8 @@
       <c r="K53" s="5">
         <v>489</v>
       </c>
-      <c r="N53" s="46"/>
-      <c r="O53" s="47"/>
+      <c r="N53" s="49"/>
+      <c r="O53" s="50"/>
       <c r="P53" s="4">
         <v>2</v>
       </c>
@@ -3711,10 +3846,33 @@
       <c r="T53" s="5">
         <v>587</v>
       </c>
-    </row>
-    <row r="54" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E54" s="46"/>
-      <c r="F54" s="47"/>
+      <c r="W53" s="49"/>
+      <c r="X53" s="50"/>
+      <c r="Y53" s="4">
+        <v>6</v>
+      </c>
+      <c r="Z53" s="2">
+        <v>8</v>
+      </c>
+      <c r="AA53" s="2">
+        <v>2</v>
+      </c>
+      <c r="AB53" s="2">
+        <v>4</v>
+      </c>
+      <c r="AC53" s="2">
+        <v>497</v>
+      </c>
+      <c r="AD53" s="2">
+        <v>562</v>
+      </c>
+      <c r="AE53" s="5">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="54" spans="5:31" x14ac:dyDescent="0.3">
+      <c r="E54" s="49"/>
+      <c r="F54" s="50"/>
       <c r="G54" s="29">
         <v>4</v>
       </c>
@@ -3730,8 +3888,8 @@
       <c r="K54" s="5">
         <v>303</v>
       </c>
-      <c r="N54" s="46"/>
-      <c r="O54" s="47"/>
+      <c r="N54" s="49"/>
+      <c r="O54" s="50"/>
       <c r="P54" s="29">
         <v>4</v>
       </c>
@@ -3747,10 +3905,33 @@
       <c r="T54" s="5">
         <v>327</v>
       </c>
-    </row>
-    <row r="55" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E55" s="46"/>
-      <c r="F55" s="47"/>
+      <c r="W54" s="49"/>
+      <c r="X54" s="50"/>
+      <c r="Y54" s="29">
+        <v>8</v>
+      </c>
+      <c r="Z54" s="2">
+        <v>4</v>
+      </c>
+      <c r="AA54" s="2">
+        <v>2</v>
+      </c>
+      <c r="AB54" s="2">
+        <v>4</v>
+      </c>
+      <c r="AC54" s="2">
+        <v>348</v>
+      </c>
+      <c r="AD54" s="2">
+        <v>404</v>
+      </c>
+      <c r="AE54" s="5">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="55" spans="5:31" x14ac:dyDescent="0.3">
+      <c r="E55" s="49"/>
+      <c r="F55" s="50"/>
       <c r="G55" s="29">
         <v>4</v>
       </c>
@@ -3766,8 +3947,8 @@
       <c r="K55" s="5">
         <v>300</v>
       </c>
-      <c r="N55" s="46"/>
-      <c r="O55" s="47"/>
+      <c r="N55" s="49"/>
+      <c r="O55" s="50"/>
       <c r="P55" s="29">
         <v>4</v>
       </c>
@@ -3783,10 +3964,33 @@
       <c r="T55" s="5">
         <v>314</v>
       </c>
-    </row>
-    <row r="56" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E56" s="46"/>
-      <c r="F56" s="47"/>
+      <c r="W55" s="49"/>
+      <c r="X55" s="50"/>
+      <c r="Y55" s="29">
+        <v>8</v>
+      </c>
+      <c r="Z55" s="2">
+        <v>8</v>
+      </c>
+      <c r="AA55" s="2">
+        <v>2</v>
+      </c>
+      <c r="AB55" s="2">
+        <v>4</v>
+      </c>
+      <c r="AC55" s="2">
+        <v>651</v>
+      </c>
+      <c r="AD55" s="2">
+        <v>713</v>
+      </c>
+      <c r="AE55" s="5">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="56" spans="5:31" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E56" s="49"/>
+      <c r="F56" s="50"/>
       <c r="G56" s="29">
         <v>8</v>
       </c>
@@ -3802,8 +4006,8 @@
       <c r="K56" s="5">
         <v>329</v>
       </c>
-      <c r="N56" s="46"/>
-      <c r="O56" s="47"/>
+      <c r="N56" s="49"/>
+      <c r="O56" s="50"/>
       <c r="P56" s="29">
         <v>8</v>
       </c>
@@ -3819,10 +4023,27 @@
       <c r="T56" s="5">
         <v>543</v>
       </c>
-    </row>
-    <row r="57" spans="5:20" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E57" s="48"/>
-      <c r="F57" s="49"/>
+      <c r="W56" s="51"/>
+      <c r="X56" s="52"/>
+      <c r="Y56" s="30">
+        <v>8</v>
+      </c>
+      <c r="Z56" s="7">
+        <v>8</v>
+      </c>
+      <c r="AA56" s="7">
+        <v>4</v>
+      </c>
+      <c r="AB56" s="7">
+        <v>8</v>
+      </c>
+      <c r="AC56" s="7"/>
+      <c r="AD56" s="7"/>
+      <c r="AE56" s="8"/>
+    </row>
+    <row r="57" spans="5:31" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E57" s="51"/>
+      <c r="F57" s="52"/>
       <c r="G57" s="30">
         <v>8</v>
       </c>
@@ -3838,8 +4059,8 @@
       <c r="K57" s="8">
         <v>329</v>
       </c>
-      <c r="N57" s="48"/>
-      <c r="O57" s="49"/>
+      <c r="N57" s="51"/>
+      <c r="O57" s="52"/>
       <c r="P57" s="30">
         <v>8</v>
       </c>
@@ -3855,12 +4076,21 @@
       <c r="T57" s="8">
         <v>398</v>
       </c>
-    </row>
-    <row r="58" spans="5:20" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E58" s="44" t="s">
+      <c r="W57"/>
+      <c r="X57"/>
+      <c r="Y57"/>
+      <c r="Z57"/>
+      <c r="AA57"/>
+      <c r="AB57"/>
+      <c r="AC57"/>
+      <c r="AD57"/>
+      <c r="AE57"/>
+    </row>
+    <row r="58" spans="5:31" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E58" s="47" t="s">
         <v>50</v>
       </c>
-      <c r="F58" s="45"/>
+      <c r="F58" s="48"/>
       <c r="G58" s="32" t="s">
         <v>33</v>
       </c>
@@ -3876,10 +4106,10 @@
       <c r="K58" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="N58" s="44" t="s">
+      <c r="N58" s="47" t="s">
         <v>53</v>
       </c>
-      <c r="O58" s="45"/>
+      <c r="O58" s="48"/>
       <c r="P58" s="32" t="s">
         <v>33</v>
       </c>
@@ -3896,9 +4126,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="59" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E59" s="46"/>
-      <c r="F59" s="47"/>
+    <row r="59" spans="5:31" x14ac:dyDescent="0.3">
+      <c r="E59" s="49"/>
+      <c r="F59" s="50"/>
       <c r="G59" s="21">
         <v>2</v>
       </c>
@@ -3914,9 +4144,9 @@
       <c r="K59" s="22">
         <v>492</v>
       </c>
-      <c r="N59" s="46"/>
-      <c r="O59" s="47"/>
-      <c r="P59" s="86">
+      <c r="N59" s="49"/>
+      <c r="O59" s="50"/>
+      <c r="P59" s="35">
         <v>2</v>
       </c>
       <c r="Q59" s="27">
@@ -3932,9 +4162,9 @@
         <v>629</v>
       </c>
     </row>
-    <row r="60" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E60" s="46"/>
-      <c r="F60" s="47"/>
+    <row r="60" spans="5:31" x14ac:dyDescent="0.3">
+      <c r="E60" s="49"/>
+      <c r="F60" s="50"/>
       <c r="G60" s="4">
         <v>2</v>
       </c>
@@ -3950,8 +4180,8 @@
       <c r="K60" s="5">
         <v>489</v>
       </c>
-      <c r="N60" s="46"/>
-      <c r="O60" s="47"/>
+      <c r="N60" s="49"/>
+      <c r="O60" s="50"/>
       <c r="P60" s="4">
         <v>2</v>
       </c>
@@ -3968,9 +4198,9 @@
         <v>605</v>
       </c>
     </row>
-    <row r="61" spans="5:20" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E61" s="46"/>
-      <c r="F61" s="47"/>
+    <row r="61" spans="5:31" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E61" s="49"/>
+      <c r="F61" s="50"/>
       <c r="G61" s="31">
         <v>4</v>
       </c>
@@ -3986,8 +4216,8 @@
       <c r="K61" s="28">
         <v>307</v>
       </c>
-      <c r="N61" s="46"/>
-      <c r="O61" s="47"/>
+      <c r="N61" s="49"/>
+      <c r="O61" s="50"/>
       <c r="P61" s="29">
         <v>4</v>
       </c>
@@ -4004,9 +4234,9 @@
         <v>322</v>
       </c>
     </row>
-    <row r="62" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E62" s="46"/>
-      <c r="F62" s="47"/>
+    <row r="62" spans="5:31" x14ac:dyDescent="0.3">
+      <c r="E62" s="49"/>
+      <c r="F62" s="50"/>
       <c r="G62" s="29">
         <v>4</v>
       </c>
@@ -4022,8 +4252,8 @@
       <c r="K62" s="5">
         <v>298</v>
       </c>
-      <c r="N62" s="46"/>
-      <c r="O62" s="47"/>
+      <c r="N62" s="49"/>
+      <c r="O62" s="50"/>
       <c r="P62" s="29">
         <v>4</v>
       </c>
@@ -4040,9 +4270,9 @@
         <v>318</v>
       </c>
     </row>
-    <row r="63" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E63" s="46"/>
-      <c r="F63" s="47"/>
+    <row r="63" spans="5:31" x14ac:dyDescent="0.3">
+      <c r="E63" s="49"/>
+      <c r="F63" s="50"/>
       <c r="G63" s="29">
         <v>8</v>
       </c>
@@ -4058,8 +4288,8 @@
       <c r="K63" s="5">
         <v>357</v>
       </c>
-      <c r="N63" s="46"/>
-      <c r="O63" s="47"/>
+      <c r="N63" s="49"/>
+      <c r="O63" s="50"/>
       <c r="P63" s="29">
         <v>8</v>
       </c>
@@ -4076,9 +4306,9 @@
         <v>510</v>
       </c>
     </row>
-    <row r="64" spans="5:20" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E64" s="48"/>
-      <c r="F64" s="49"/>
+    <row r="64" spans="5:31" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E64" s="51"/>
+      <c r="F64" s="52"/>
       <c r="G64" s="30">
         <v>8</v>
       </c>
@@ -4094,8 +4324,8 @@
       <c r="K64" s="8">
         <v>341</v>
       </c>
-      <c r="N64" s="48"/>
-      <c r="O64" s="49"/>
+      <c r="N64" s="51"/>
+      <c r="O64" s="52"/>
       <c r="P64" s="30">
         <v>8</v>
       </c>
@@ -4113,27 +4343,20 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="53">
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="N48:T50"/>
-    <mergeCell ref="N51:O57"/>
-    <mergeCell ref="N58:O64"/>
-    <mergeCell ref="Q3:S3"/>
-    <mergeCell ref="W3:Y3"/>
-    <mergeCell ref="N3:P3"/>
-    <mergeCell ref="H11:P11"/>
-    <mergeCell ref="K3:M3"/>
-    <mergeCell ref="T3:V3"/>
-    <mergeCell ref="T4:V6"/>
-    <mergeCell ref="Q4:S6"/>
-    <mergeCell ref="K4:M6"/>
-    <mergeCell ref="N4:P6"/>
-    <mergeCell ref="AC3:AE3"/>
-    <mergeCell ref="AC4:AE6"/>
-    <mergeCell ref="Z3:AB3"/>
-    <mergeCell ref="Z4:AB6"/>
-    <mergeCell ref="W4:Y6"/>
+  <mergeCells count="55">
+    <mergeCell ref="W51:X56"/>
+    <mergeCell ref="W48:AE50"/>
+    <mergeCell ref="S38:T45"/>
+    <mergeCell ref="E38:F45"/>
+    <mergeCell ref="E30:F37"/>
+    <mergeCell ref="E27:N29"/>
+    <mergeCell ref="AC37:AD37"/>
+    <mergeCell ref="AA18:AC20"/>
+    <mergeCell ref="X21:Y24"/>
+    <mergeCell ref="AH18:AJ20"/>
+    <mergeCell ref="AE21:AF24"/>
+    <mergeCell ref="S27:AB29"/>
+    <mergeCell ref="S30:T37"/>
     <mergeCell ref="D1:E1"/>
     <mergeCell ref="F1:I1"/>
     <mergeCell ref="D9:E9"/>
@@ -4145,6 +4368,26 @@
     <mergeCell ref="D7:E7"/>
     <mergeCell ref="F7:G7"/>
     <mergeCell ref="D8:E8"/>
+    <mergeCell ref="AC3:AE3"/>
+    <mergeCell ref="AC4:AE6"/>
+    <mergeCell ref="Z3:AB3"/>
+    <mergeCell ref="Z4:AB6"/>
+    <mergeCell ref="W4:Y6"/>
+    <mergeCell ref="Q3:S3"/>
+    <mergeCell ref="W3:Y3"/>
+    <mergeCell ref="N3:P3"/>
+    <mergeCell ref="H11:P11"/>
+    <mergeCell ref="K3:M3"/>
+    <mergeCell ref="T3:V3"/>
+    <mergeCell ref="T4:V6"/>
+    <mergeCell ref="Q4:S6"/>
+    <mergeCell ref="K4:M6"/>
+    <mergeCell ref="N4:P6"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="N48:T50"/>
+    <mergeCell ref="N51:O57"/>
+    <mergeCell ref="N58:O64"/>
     <mergeCell ref="S18:U20"/>
     <mergeCell ref="N13:P15"/>
     <mergeCell ref="H17:J17"/>
@@ -4153,20 +4396,9 @@
     <mergeCell ref="K17:M17"/>
     <mergeCell ref="K18:M20"/>
     <mergeCell ref="O21:P24"/>
-    <mergeCell ref="AC37:AD37"/>
-    <mergeCell ref="AA18:AC20"/>
-    <mergeCell ref="X21:Y24"/>
-    <mergeCell ref="AH18:AJ20"/>
-    <mergeCell ref="AE21:AF24"/>
     <mergeCell ref="E48:K50"/>
     <mergeCell ref="E51:F57"/>
     <mergeCell ref="E58:F64"/>
-    <mergeCell ref="S27:AB29"/>
-    <mergeCell ref="S30:T37"/>
-    <mergeCell ref="S38:T45"/>
-    <mergeCell ref="E38:F45"/>
-    <mergeCell ref="E30:F37"/>
-    <mergeCell ref="E27:N29"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
add folder for working decoders projects and first one for RM(16,11), modified table of comporasions
</commit_message>
<xml_diff>
--- a/module_library/comp_sum_select.xlsx
+++ b/module_library/comp_sum_select.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\LRMLD\module_library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8061868E-8773-4B8C-84BB-DD4E0736B642}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFDB8E80-4F41-4A87-AAF0-5CA64B10B186}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="62">
   <si>
     <t>LUT</t>
   </si>
@@ -262,6 +262,20 @@
   </si>
   <si>
     <t>make</t>
+  </si>
+  <si>
+    <t>RM(16,11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IS_FSM = 0
+</t>
+  </si>
+  <si>
+    <t>LAT, cls</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IS_FSM = 1
+</t>
   </si>
 </sst>
 </file>
@@ -315,7 +329,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="57">
+  <borders count="59">
     <border>
       <left/>
       <right/>
@@ -1047,11 +1061,37 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="101">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1158,28 +1198,178 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1191,151 +1381,16 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1618,7 +1673,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="D1:AJ64"/>
+  <dimension ref="D1:AJ74"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="7" width="8.88671875" style="1"/>
@@ -1630,177 +1685,177 @@
   </cols>
   <sheetData>
     <row r="1" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="D1" s="36" t="s">
+      <c r="D1" s="64" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36" t="s">
-        <v>8</v>
-      </c>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="36"/>
+      <c r="E1" s="64"/>
+      <c r="F1" s="64" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" s="64"/>
+      <c r="H1" s="64"/>
+      <c r="I1" s="64"/>
     </row>
     <row r="2" spans="4:31" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="3" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="H3" s="81" t="s">
+      <c r="H3" s="68" t="s">
         <v>12</v>
       </c>
-      <c r="I3" s="60"/>
-      <c r="J3" s="60"/>
-      <c r="K3" s="60" t="s">
+      <c r="I3" s="69"/>
+      <c r="J3" s="69"/>
+      <c r="K3" s="69" t="s">
         <v>12</v>
       </c>
-      <c r="L3" s="60"/>
-      <c r="M3" s="60"/>
-      <c r="N3" s="56" t="s">
+      <c r="L3" s="69"/>
+      <c r="M3" s="69"/>
+      <c r="N3" s="85" t="s">
         <v>14</v>
       </c>
-      <c r="O3" s="57"/>
-      <c r="P3" s="58"/>
-      <c r="Q3" s="53" t="s">
+      <c r="O3" s="86"/>
+      <c r="P3" s="87"/>
+      <c r="Q3" s="82" t="s">
         <v>13</v>
       </c>
-      <c r="R3" s="54"/>
-      <c r="S3" s="54"/>
-      <c r="T3" s="54" t="s">
+      <c r="R3" s="83"/>
+      <c r="S3" s="83"/>
+      <c r="T3" s="83" t="s">
         <v>17</v>
       </c>
-      <c r="U3" s="54"/>
-      <c r="V3" s="61"/>
-      <c r="W3" s="55" t="s">
+      <c r="U3" s="83"/>
+      <c r="V3" s="89"/>
+      <c r="W3" s="84" t="s">
         <v>15</v>
       </c>
-      <c r="X3" s="54"/>
-      <c r="Y3" s="54"/>
-      <c r="Z3" s="68" t="s">
+      <c r="X3" s="83"/>
+      <c r="Y3" s="83"/>
+      <c r="Z3" s="70" t="s">
         <v>13</v>
       </c>
-      <c r="AA3" s="69"/>
-      <c r="AB3" s="70"/>
-      <c r="AC3" s="68" t="s">
+      <c r="AA3" s="71"/>
+      <c r="AB3" s="72"/>
+      <c r="AC3" s="70" t="s">
         <v>22</v>
       </c>
-      <c r="AD3" s="69"/>
-      <c r="AE3" s="70"/>
+      <c r="AD3" s="71"/>
+      <c r="AE3" s="72"/>
     </row>
     <row r="4" spans="4:31" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D4" s="36" t="s">
+      <c r="D4" s="64" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="36"/>
-      <c r="F4" s="36"/>
-      <c r="G4" s="37"/>
-      <c r="H4" s="80" t="s">
+      <c r="E4" s="64"/>
+      <c r="F4" s="64"/>
+      <c r="G4" s="65"/>
+      <c r="H4" s="66" t="s">
         <v>20</v>
       </c>
-      <c r="I4" s="65"/>
-      <c r="J4" s="65"/>
-      <c r="K4" s="65" t="s">
+      <c r="I4" s="67"/>
+      <c r="J4" s="67"/>
+      <c r="K4" s="67" t="s">
         <v>21</v>
       </c>
-      <c r="L4" s="65"/>
-      <c r="M4" s="65"/>
-      <c r="N4" s="66" t="s">
+      <c r="L4" s="67"/>
+      <c r="M4" s="67"/>
+      <c r="N4" s="92" t="s">
         <v>9</v>
       </c>
-      <c r="O4" s="62"/>
-      <c r="P4" s="67"/>
-      <c r="Q4" s="64" t="s">
+      <c r="O4" s="63"/>
+      <c r="P4" s="93"/>
+      <c r="Q4" s="91" t="s">
         <v>10</v>
       </c>
-      <c r="R4" s="36"/>
-      <c r="S4" s="36"/>
-      <c r="T4" s="62" t="s">
+      <c r="R4" s="64"/>
+      <c r="S4" s="64"/>
+      <c r="T4" s="63" t="s">
         <v>18</v>
       </c>
-      <c r="U4" s="62"/>
-      <c r="V4" s="63"/>
-      <c r="W4" s="79" t="s">
+      <c r="U4" s="63"/>
+      <c r="V4" s="90"/>
+      <c r="W4" s="81" t="s">
         <v>11</v>
       </c>
-      <c r="X4" s="36"/>
-      <c r="Y4" s="36"/>
-      <c r="Z4" s="71" t="s">
+      <c r="X4" s="64"/>
+      <c r="Y4" s="64"/>
+      <c r="Z4" s="73" t="s">
         <v>16</v>
       </c>
-      <c r="AA4" s="72"/>
-      <c r="AB4" s="73"/>
-      <c r="AC4" s="71" t="s">
+      <c r="AA4" s="74"/>
+      <c r="AB4" s="75"/>
+      <c r="AC4" s="73" t="s">
         <v>23</v>
       </c>
-      <c r="AD4" s="72"/>
-      <c r="AE4" s="73"/>
+      <c r="AD4" s="74"/>
+      <c r="AE4" s="75"/>
     </row>
     <row r="5" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="D5" s="36"/>
-      <c r="E5" s="36"/>
-      <c r="F5" s="36"/>
-      <c r="G5" s="37"/>
-      <c r="H5" s="80"/>
-      <c r="I5" s="65"/>
-      <c r="J5" s="65"/>
-      <c r="K5" s="65"/>
-      <c r="L5" s="65"/>
-      <c r="M5" s="65"/>
-      <c r="N5" s="66"/>
-      <c r="O5" s="62"/>
-      <c r="P5" s="67"/>
-      <c r="Q5" s="64"/>
-      <c r="R5" s="36"/>
-      <c r="S5" s="36"/>
-      <c r="T5" s="62"/>
-      <c r="U5" s="62"/>
-      <c r="V5" s="63"/>
-      <c r="W5" s="79"/>
-      <c r="X5" s="36"/>
-      <c r="Y5" s="36"/>
-      <c r="Z5" s="74"/>
-      <c r="AA5" s="75"/>
-      <c r="AB5" s="50"/>
-      <c r="AC5" s="74"/>
-      <c r="AD5" s="75"/>
-      <c r="AE5" s="50"/>
+      <c r="D5" s="64"/>
+      <c r="E5" s="64"/>
+      <c r="F5" s="64"/>
+      <c r="G5" s="65"/>
+      <c r="H5" s="66"/>
+      <c r="I5" s="67"/>
+      <c r="J5" s="67"/>
+      <c r="K5" s="67"/>
+      <c r="L5" s="67"/>
+      <c r="M5" s="67"/>
+      <c r="N5" s="92"/>
+      <c r="O5" s="63"/>
+      <c r="P5" s="93"/>
+      <c r="Q5" s="91"/>
+      <c r="R5" s="64"/>
+      <c r="S5" s="64"/>
+      <c r="T5" s="63"/>
+      <c r="U5" s="63"/>
+      <c r="V5" s="90"/>
+      <c r="W5" s="81"/>
+      <c r="X5" s="64"/>
+      <c r="Y5" s="64"/>
+      <c r="Z5" s="76"/>
+      <c r="AA5" s="77"/>
+      <c r="AB5" s="40"/>
+      <c r="AC5" s="76"/>
+      <c r="AD5" s="77"/>
+      <c r="AE5" s="40"/>
     </row>
     <row r="6" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="D6" s="36"/>
-      <c r="E6" s="36"/>
-      <c r="F6" s="36"/>
-      <c r="G6" s="37"/>
-      <c r="H6" s="80"/>
-      <c r="I6" s="65"/>
-      <c r="J6" s="65"/>
-      <c r="K6" s="65"/>
-      <c r="L6" s="65"/>
-      <c r="M6" s="65"/>
-      <c r="N6" s="66"/>
-      <c r="O6" s="62"/>
-      <c r="P6" s="67"/>
-      <c r="Q6" s="64"/>
-      <c r="R6" s="36"/>
-      <c r="S6" s="36"/>
-      <c r="T6" s="62"/>
-      <c r="U6" s="62"/>
-      <c r="V6" s="63"/>
-      <c r="W6" s="79"/>
-      <c r="X6" s="36"/>
-      <c r="Y6" s="36"/>
-      <c r="Z6" s="76"/>
-      <c r="AA6" s="77"/>
-      <c r="AB6" s="78"/>
-      <c r="AC6" s="76"/>
-      <c r="AD6" s="77"/>
-      <c r="AE6" s="78"/>
+      <c r="D6" s="64"/>
+      <c r="E6" s="64"/>
+      <c r="F6" s="64"/>
+      <c r="G6" s="65"/>
+      <c r="H6" s="66"/>
+      <c r="I6" s="67"/>
+      <c r="J6" s="67"/>
+      <c r="K6" s="67"/>
+      <c r="L6" s="67"/>
+      <c r="M6" s="67"/>
+      <c r="N6" s="92"/>
+      <c r="O6" s="63"/>
+      <c r="P6" s="93"/>
+      <c r="Q6" s="91"/>
+      <c r="R6" s="64"/>
+      <c r="S6" s="64"/>
+      <c r="T6" s="63"/>
+      <c r="U6" s="63"/>
+      <c r="V6" s="90"/>
+      <c r="W6" s="81"/>
+      <c r="X6" s="64"/>
+      <c r="Y6" s="64"/>
+      <c r="Z6" s="78"/>
+      <c r="AA6" s="79"/>
+      <c r="AB6" s="80"/>
+      <c r="AC6" s="78"/>
+      <c r="AD6" s="79"/>
+      <c r="AE6" s="80"/>
     </row>
     <row r="7" spans="4:31" ht="20.399999999999999" x14ac:dyDescent="0.3">
-      <c r="D7" s="36" t="s">
-        <v>4</v>
-      </c>
-      <c r="E7" s="36"/>
-      <c r="F7" s="36" t="s">
+      <c r="D7" s="64" t="s">
+        <v>4</v>
+      </c>
+      <c r="E7" s="64"/>
+      <c r="F7" s="64" t="s">
         <v>5</v>
       </c>
-      <c r="G7" s="37"/>
+      <c r="G7" s="65"/>
       <c r="H7" s="11" t="s">
         <v>0</v>
       </c>
@@ -1875,14 +1930,14 @@
       </c>
     </row>
     <row r="8" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="D8" s="36">
-        <v>8</v>
-      </c>
-      <c r="E8" s="36"/>
-      <c r="F8" s="36">
-        <v>8</v>
-      </c>
-      <c r="G8" s="37"/>
+      <c r="D8" s="64">
+        <v>8</v>
+      </c>
+      <c r="E8" s="64"/>
+      <c r="F8" s="64">
+        <v>8</v>
+      </c>
+      <c r="G8" s="65"/>
       <c r="H8" s="11">
         <v>331</v>
       </c>
@@ -1957,14 +2012,14 @@
       </c>
     </row>
     <row r="9" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="D9" s="36">
+      <c r="D9" s="64">
         <v>10</v>
       </c>
-      <c r="E9" s="36"/>
-      <c r="F9" s="36">
+      <c r="E9" s="64"/>
+      <c r="F9" s="64">
         <v>16</v>
       </c>
-      <c r="G9" s="37"/>
+      <c r="G9" s="65"/>
       <c r="H9" s="11">
         <v>504</v>
       </c>
@@ -2039,14 +2094,14 @@
       </c>
     </row>
     <row r="10" spans="4:31" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D10" s="36">
+      <c r="D10" s="64">
         <v>10</v>
       </c>
-      <c r="E10" s="36"/>
-      <c r="F10" s="36">
+      <c r="E10" s="64"/>
+      <c r="F10" s="64">
         <v>32</v>
       </c>
-      <c r="G10" s="37"/>
+      <c r="G10" s="65"/>
       <c r="H10" s="13">
         <v>761</v>
       </c>
@@ -2121,17 +2176,17 @@
       </c>
     </row>
     <row r="11" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="H11" s="59" t="s">
+      <c r="H11" s="88" t="s">
         <v>24</v>
       </c>
-      <c r="I11" s="59"/>
-      <c r="J11" s="59"/>
-      <c r="K11" s="59"/>
-      <c r="L11" s="59"/>
-      <c r="M11" s="59"/>
-      <c r="N11" s="59"/>
-      <c r="O11" s="59"/>
-      <c r="P11" s="59"/>
+      <c r="I11" s="88"/>
+      <c r="J11" s="88"/>
+      <c r="K11" s="88"/>
+      <c r="L11" s="88"/>
+      <c r="M11" s="88"/>
+      <c r="N11" s="88"/>
+      <c r="O11" s="88"/>
+      <c r="P11" s="88"/>
     </row>
     <row r="12" spans="4:31" ht="23.4" x14ac:dyDescent="0.3">
       <c r="O12" s="19" t="s">
@@ -2139,103 +2194,103 @@
       </c>
     </row>
     <row r="13" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="N13" s="75" t="s">
+      <c r="N13" s="77" t="s">
         <v>19</v>
       </c>
-      <c r="O13" s="75"/>
-      <c r="P13" s="75"/>
+      <c r="O13" s="77"/>
+      <c r="P13" s="77"/>
     </row>
     <row r="14" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="N14" s="75"/>
-      <c r="O14" s="75"/>
-      <c r="P14" s="75"/>
+      <c r="N14" s="77"/>
+      <c r="O14" s="77"/>
+      <c r="P14" s="77"/>
     </row>
     <row r="15" spans="4:31" x14ac:dyDescent="0.3">
-      <c r="N15" s="75"/>
-      <c r="O15" s="75"/>
-      <c r="P15" s="75"/>
+      <c r="N15" s="77"/>
+      <c r="O15" s="77"/>
+      <c r="P15" s="77"/>
     </row>
     <row r="17" spans="5:36" x14ac:dyDescent="0.3">
-      <c r="H17" s="36" t="s">
+      <c r="H17" s="64" t="s">
         <v>26</v>
       </c>
-      <c r="I17" s="36"/>
-      <c r="J17" s="36"/>
-      <c r="K17" s="36" t="s">
+      <c r="I17" s="64"/>
+      <c r="J17" s="64"/>
+      <c r="K17" s="64" t="s">
         <v>26</v>
       </c>
-      <c r="L17" s="36"/>
-      <c r="M17" s="36"/>
+      <c r="L17" s="64"/>
+      <c r="M17" s="64"/>
       <c r="S17"/>
       <c r="T17"/>
       <c r="U17"/>
     </row>
     <row r="18" spans="5:36" x14ac:dyDescent="0.3">
-      <c r="H18" s="62" t="s">
+      <c r="H18" s="63" t="s">
         <v>28</v>
       </c>
-      <c r="I18" s="62"/>
-      <c r="J18" s="62"/>
-      <c r="K18" s="62" t="s">
+      <c r="I18" s="63"/>
+      <c r="J18" s="63"/>
+      <c r="K18" s="63" t="s">
         <v>29</v>
       </c>
-      <c r="L18" s="62"/>
-      <c r="M18" s="62"/>
-      <c r="S18" s="62" t="s">
+      <c r="L18" s="63"/>
+      <c r="M18" s="63"/>
+      <c r="S18" s="63" t="s">
         <v>32</v>
       </c>
-      <c r="T18" s="62"/>
-      <c r="U18" s="62"/>
-      <c r="AA18" s="62" t="s">
+      <c r="T18" s="63"/>
+      <c r="U18" s="63"/>
+      <c r="AA18" s="63" t="s">
         <v>35</v>
       </c>
-      <c r="AB18" s="62"/>
-      <c r="AC18" s="62"/>
-      <c r="AH18" s="62" t="s">
+      <c r="AB18" s="63"/>
+      <c r="AC18" s="63"/>
+      <c r="AH18" s="63" t="s">
         <v>36</v>
       </c>
-      <c r="AI18" s="62"/>
-      <c r="AJ18" s="62"/>
+      <c r="AI18" s="63"/>
+      <c r="AJ18" s="63"/>
     </row>
     <row r="19" spans="5:36" x14ac:dyDescent="0.3">
-      <c r="H19" s="62"/>
-      <c r="I19" s="62"/>
-      <c r="J19" s="62"/>
-      <c r="K19" s="62"/>
-      <c r="L19" s="62"/>
-      <c r="M19" s="62"/>
-      <c r="S19" s="62"/>
-      <c r="T19" s="62"/>
-      <c r="U19" s="62"/>
-      <c r="AA19" s="62"/>
-      <c r="AB19" s="62"/>
-      <c r="AC19" s="62"/>
-      <c r="AH19" s="62"/>
-      <c r="AI19" s="62"/>
-      <c r="AJ19" s="62"/>
+      <c r="H19" s="63"/>
+      <c r="I19" s="63"/>
+      <c r="J19" s="63"/>
+      <c r="K19" s="63"/>
+      <c r="L19" s="63"/>
+      <c r="M19" s="63"/>
+      <c r="S19" s="63"/>
+      <c r="T19" s="63"/>
+      <c r="U19" s="63"/>
+      <c r="AA19" s="63"/>
+      <c r="AB19" s="63"/>
+      <c r="AC19" s="63"/>
+      <c r="AH19" s="63"/>
+      <c r="AI19" s="63"/>
+      <c r="AJ19" s="63"/>
     </row>
     <row r="20" spans="5:36" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H20" s="62"/>
-      <c r="I20" s="62"/>
-      <c r="J20" s="62"/>
-      <c r="K20" s="62"/>
-      <c r="L20" s="62"/>
-      <c r="M20" s="62"/>
-      <c r="S20" s="62"/>
-      <c r="T20" s="62"/>
-      <c r="U20" s="62"/>
-      <c r="AA20" s="62"/>
-      <c r="AB20" s="62"/>
-      <c r="AC20" s="62"/>
-      <c r="AH20" s="62"/>
-      <c r="AI20" s="62"/>
-      <c r="AJ20" s="62"/>
+      <c r="H20" s="63"/>
+      <c r="I20" s="63"/>
+      <c r="J20" s="63"/>
+      <c r="K20" s="63"/>
+      <c r="L20" s="63"/>
+      <c r="M20" s="63"/>
+      <c r="S20" s="63"/>
+      <c r="T20" s="63"/>
+      <c r="U20" s="63"/>
+      <c r="AA20" s="63"/>
+      <c r="AB20" s="63"/>
+      <c r="AC20" s="63"/>
+      <c r="AH20" s="63"/>
+      <c r="AI20" s="63"/>
+      <c r="AJ20" s="63"/>
     </row>
     <row r="21" spans="5:36" ht="20.399999999999999" x14ac:dyDescent="0.3">
-      <c r="E21" s="62" t="s">
+      <c r="E21" s="63" t="s">
         <v>30</v>
       </c>
-      <c r="F21" s="62"/>
+      <c r="F21" s="63"/>
       <c r="G21" s="2" t="s">
         <v>27</v>
       </c>
@@ -2257,10 +2312,10 @@
       <c r="M21" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="O21" s="62" t="s">
+      <c r="O21" s="63" t="s">
         <v>34</v>
       </c>
-      <c r="P21" s="62"/>
+      <c r="P21" s="63"/>
       <c r="Q21" s="18" t="s">
         <v>33</v>
       </c>
@@ -2277,10 +2332,10 @@
         <v>2</v>
       </c>
       <c r="W21"/>
-      <c r="X21" s="62" t="s">
+      <c r="X21" s="63" t="s">
         <v>34</v>
       </c>
-      <c r="Y21" s="62"/>
+      <c r="Y21" s="63"/>
       <c r="Z21" s="2" t="s">
         <v>31</v>
       </c>
@@ -2293,10 +2348,10 @@
       <c r="AC21" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="AE21" s="62" t="s">
+      <c r="AE21" s="63" t="s">
         <v>37</v>
       </c>
-      <c r="AF21" s="62"/>
+      <c r="AF21" s="63"/>
       <c r="AG21" s="18" t="s">
         <v>38</v>
       </c>
@@ -2311,8 +2366,8 @@
       </c>
     </row>
     <row r="22" spans="5:36" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E22" s="62"/>
-      <c r="F22" s="62"/>
+      <c r="E22" s="63"/>
+      <c r="F22" s="63"/>
       <c r="G22" s="2">
         <v>4</v>
       </c>
@@ -2334,8 +2389,8 @@
       <c r="M22" s="2">
         <v>578</v>
       </c>
-      <c r="O22" s="62"/>
-      <c r="P22" s="62"/>
+      <c r="O22" s="63"/>
+      <c r="P22" s="63"/>
       <c r="Q22" s="18">
         <v>8</v>
       </c>
@@ -2352,8 +2407,8 @@
         <v>455</v>
       </c>
       <c r="W22"/>
-      <c r="X22" s="62"/>
-      <c r="Y22" s="62"/>
+      <c r="X22" s="63"/>
+      <c r="Y22" s="63"/>
       <c r="Z22" s="2">
         <v>4</v>
       </c>
@@ -2366,8 +2421,8 @@
       <c r="AC22" s="2">
         <v>555</v>
       </c>
-      <c r="AE22" s="62"/>
-      <c r="AF22" s="62"/>
+      <c r="AE22" s="63"/>
+      <c r="AF22" s="63"/>
       <c r="AG22" s="2">
         <v>2</v>
       </c>
@@ -2382,8 +2437,8 @@
       </c>
     </row>
     <row r="23" spans="5:36" x14ac:dyDescent="0.3">
-      <c r="E23" s="62"/>
-      <c r="F23" s="62"/>
+      <c r="E23" s="63"/>
+      <c r="F23" s="63"/>
       <c r="G23" s="2">
         <v>8</v>
       </c>
@@ -2405,8 +2460,8 @@
       <c r="M23" s="2">
         <v>476</v>
       </c>
-      <c r="O23" s="62"/>
-      <c r="P23" s="62"/>
+      <c r="O23" s="63"/>
+      <c r="P23" s="63"/>
       <c r="Q23" s="18">
         <v>12</v>
       </c>
@@ -2423,8 +2478,8 @@
         <v>462</v>
       </c>
       <c r="W23"/>
-      <c r="X23" s="62"/>
-      <c r="Y23" s="62"/>
+      <c r="X23" s="63"/>
+      <c r="Y23" s="63"/>
       <c r="Z23" s="2">
         <v>8</v>
       </c>
@@ -2437,8 +2492,8 @@
       <c r="AC23" s="2">
         <v>542</v>
       </c>
-      <c r="AE23" s="62"/>
-      <c r="AF23" s="62"/>
+      <c r="AE23" s="63"/>
+      <c r="AF23" s="63"/>
       <c r="AG23" s="2">
         <v>4</v>
       </c>
@@ -2453,8 +2508,8 @@
       </c>
     </row>
     <row r="24" spans="5:36" x14ac:dyDescent="0.3">
-      <c r="E24" s="62"/>
-      <c r="F24" s="62"/>
+      <c r="E24" s="63"/>
+      <c r="F24" s="63"/>
       <c r="G24" s="2">
         <v>16</v>
       </c>
@@ -2476,8 +2531,8 @@
       <c r="M24" s="2">
         <v>387</v>
       </c>
-      <c r="O24" s="62"/>
-      <c r="P24" s="62"/>
+      <c r="O24" s="63"/>
+      <c r="P24" s="63"/>
       <c r="Q24" s="18">
         <v>16</v>
       </c>
@@ -2494,8 +2549,8 @@
         <v>390</v>
       </c>
       <c r="W24"/>
-      <c r="X24" s="62"/>
-      <c r="Y24" s="62"/>
+      <c r="X24" s="63"/>
+      <c r="Y24" s="63"/>
       <c r="Z24" s="2">
         <v>16</v>
       </c>
@@ -2508,8 +2563,8 @@
       <c r="AC24" s="2">
         <v>493</v>
       </c>
-      <c r="AE24" s="62"/>
-      <c r="AF24" s="62"/>
+      <c r="AE24" s="63"/>
+      <c r="AF24" s="63"/>
       <c r="AG24" s="2">
         <v>8</v>
       </c>
@@ -2525,80 +2580,80 @@
     </row>
     <row r="26" spans="5:36" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="27" spans="5:36" x14ac:dyDescent="0.3">
-      <c r="E27" s="38" t="s">
+      <c r="E27" s="52" t="s">
         <v>39</v>
       </c>
-      <c r="F27" s="39"/>
-      <c r="G27" s="39"/>
-      <c r="H27" s="39"/>
-      <c r="I27" s="39"/>
-      <c r="J27" s="39"/>
-      <c r="K27" s="39"/>
-      <c r="L27" s="39"/>
-      <c r="M27" s="39"/>
-      <c r="N27" s="40"/>
-      <c r="S27" s="38" t="s">
+      <c r="F27" s="53"/>
+      <c r="G27" s="53"/>
+      <c r="H27" s="53"/>
+      <c r="I27" s="53"/>
+      <c r="J27" s="53"/>
+      <c r="K27" s="53"/>
+      <c r="L27" s="53"/>
+      <c r="M27" s="53"/>
+      <c r="N27" s="54"/>
+      <c r="S27" s="52" t="s">
         <v>39</v>
       </c>
-      <c r="T27" s="39"/>
-      <c r="U27" s="39"/>
-      <c r="V27" s="39"/>
-      <c r="W27" s="39"/>
-      <c r="X27" s="39"/>
-      <c r="Y27" s="39"/>
-      <c r="Z27" s="39"/>
-      <c r="AA27" s="39"/>
-      <c r="AB27" s="40"/>
+      <c r="T27" s="53"/>
+      <c r="U27" s="53"/>
+      <c r="V27" s="53"/>
+      <c r="W27" s="53"/>
+      <c r="X27" s="53"/>
+      <c r="Y27" s="53"/>
+      <c r="Z27" s="53"/>
+      <c r="AA27" s="53"/>
+      <c r="AB27" s="54"/>
     </row>
     <row r="28" spans="5:36" x14ac:dyDescent="0.3">
-      <c r="E28" s="41"/>
-      <c r="F28" s="42"/>
-      <c r="G28" s="42"/>
-      <c r="H28" s="42"/>
-      <c r="I28" s="42"/>
-      <c r="J28" s="42"/>
-      <c r="K28" s="42"/>
-      <c r="L28" s="42"/>
-      <c r="M28" s="42"/>
-      <c r="N28" s="43"/>
-      <c r="S28" s="41"/>
-      <c r="T28" s="42"/>
-      <c r="U28" s="42"/>
-      <c r="V28" s="42"/>
-      <c r="W28" s="42"/>
-      <c r="X28" s="42"/>
-      <c r="Y28" s="42"/>
-      <c r="Z28" s="42"/>
-      <c r="AA28" s="42"/>
-      <c r="AB28" s="43"/>
+      <c r="E28" s="55"/>
+      <c r="F28" s="56"/>
+      <c r="G28" s="56"/>
+      <c r="H28" s="56"/>
+      <c r="I28" s="56"/>
+      <c r="J28" s="56"/>
+      <c r="K28" s="56"/>
+      <c r="L28" s="56"/>
+      <c r="M28" s="56"/>
+      <c r="N28" s="57"/>
+      <c r="S28" s="55"/>
+      <c r="T28" s="56"/>
+      <c r="U28" s="56"/>
+      <c r="V28" s="56"/>
+      <c r="W28" s="56"/>
+      <c r="X28" s="56"/>
+      <c r="Y28" s="56"/>
+      <c r="Z28" s="56"/>
+      <c r="AA28" s="56"/>
+      <c r="AB28" s="57"/>
     </row>
     <row r="29" spans="5:36" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E29" s="84"/>
-      <c r="F29" s="85"/>
-      <c r="G29" s="85"/>
-      <c r="H29" s="85"/>
-      <c r="I29" s="85"/>
-      <c r="J29" s="85"/>
-      <c r="K29" s="85"/>
-      <c r="L29" s="85"/>
-      <c r="M29" s="85"/>
-      <c r="N29" s="86"/>
-      <c r="S29" s="84"/>
-      <c r="T29" s="85"/>
-      <c r="U29" s="85"/>
-      <c r="V29" s="85"/>
-      <c r="W29" s="85"/>
-      <c r="X29" s="85"/>
-      <c r="Y29" s="85"/>
-      <c r="Z29" s="85"/>
-      <c r="AA29" s="85"/>
-      <c r="AB29" s="86"/>
+      <c r="E29" s="58"/>
+      <c r="F29" s="59"/>
+      <c r="G29" s="59"/>
+      <c r="H29" s="59"/>
+      <c r="I29" s="59"/>
+      <c r="J29" s="59"/>
+      <c r="K29" s="59"/>
+      <c r="L29" s="59"/>
+      <c r="M29" s="59"/>
+      <c r="N29" s="60"/>
+      <c r="S29" s="58"/>
+      <c r="T29" s="59"/>
+      <c r="U29" s="59"/>
+      <c r="V29" s="59"/>
+      <c r="W29" s="59"/>
+      <c r="X29" s="59"/>
+      <c r="Y29" s="59"/>
+      <c r="Z29" s="59"/>
+      <c r="AA29" s="59"/>
+      <c r="AB29" s="60"/>
     </row>
     <row r="30" spans="5:36" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E30" s="47" t="s">
+      <c r="E30" s="37" t="s">
         <v>44</v>
       </c>
-      <c r="F30" s="48"/>
+      <c r="F30" s="38"/>
       <c r="G30" s="24" t="s">
         <v>33</v>
       </c>
@@ -2623,10 +2678,10 @@
       <c r="N30" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="S30" s="47" t="s">
+      <c r="S30" s="37" t="s">
         <v>44</v>
       </c>
-      <c r="T30" s="48"/>
+      <c r="T30" s="38"/>
       <c r="U30" s="24" t="s">
         <v>33</v>
       </c>
@@ -2653,8 +2708,8 @@
       </c>
     </row>
     <row r="31" spans="5:36" x14ac:dyDescent="0.3">
-      <c r="E31" s="49"/>
-      <c r="F31" s="50"/>
+      <c r="E31" s="39"/>
+      <c r="F31" s="40"/>
       <c r="G31" s="23">
         <v>4</v>
       </c>
@@ -2679,8 +2734,8 @@
       <c r="N31" s="5">
         <v>479</v>
       </c>
-      <c r="S31" s="49"/>
-      <c r="T31" s="50"/>
+      <c r="S31" s="39"/>
+      <c r="T31" s="40"/>
       <c r="U31" s="23">
         <v>4</v>
       </c>
@@ -2707,8 +2762,8 @@
       </c>
     </row>
     <row r="32" spans="5:36" x14ac:dyDescent="0.3">
-      <c r="E32" s="49"/>
-      <c r="F32" s="50"/>
+      <c r="E32" s="39"/>
+      <c r="F32" s="40"/>
       <c r="G32" s="23">
         <v>4</v>
       </c>
@@ -2733,8 +2788,8 @@
       <c r="N32" s="5">
         <v>300</v>
       </c>
-      <c r="S32" s="49"/>
-      <c r="T32" s="50"/>
+      <c r="S32" s="39"/>
+      <c r="T32" s="40"/>
       <c r="U32" s="23">
         <v>4</v>
       </c>
@@ -2761,8 +2816,8 @@
       </c>
     </row>
     <row r="33" spans="5:31" x14ac:dyDescent="0.3">
-      <c r="E33" s="49"/>
-      <c r="F33" s="50"/>
+      <c r="E33" s="39"/>
+      <c r="F33" s="40"/>
       <c r="G33" s="23">
         <v>4</v>
       </c>
@@ -2787,8 +2842,8 @@
       <c r="N33" s="5">
         <v>276</v>
       </c>
-      <c r="S33" s="49"/>
-      <c r="T33" s="50"/>
+      <c r="S33" s="39"/>
+      <c r="T33" s="40"/>
       <c r="U33" s="23">
         <v>4</v>
       </c>
@@ -2815,8 +2870,8 @@
       </c>
     </row>
     <row r="34" spans="5:31" x14ac:dyDescent="0.3">
-      <c r="E34" s="49"/>
-      <c r="F34" s="50"/>
+      <c r="E34" s="39"/>
+      <c r="F34" s="40"/>
       <c r="G34" s="23">
         <v>4</v>
       </c>
@@ -2841,8 +2896,8 @@
       <c r="N34" s="5">
         <v>290</v>
       </c>
-      <c r="S34" s="49"/>
-      <c r="T34" s="50"/>
+      <c r="S34" s="39"/>
+      <c r="T34" s="40"/>
       <c r="U34" s="23">
         <v>4</v>
       </c>
@@ -2869,8 +2924,8 @@
       </c>
     </row>
     <row r="35" spans="5:31" x14ac:dyDescent="0.3">
-      <c r="E35" s="49"/>
-      <c r="F35" s="50"/>
+      <c r="E35" s="39"/>
+      <c r="F35" s="40"/>
       <c r="G35" s="23">
         <v>8</v>
       </c>
@@ -2895,8 +2950,8 @@
       <c r="N35" s="5">
         <v>320</v>
       </c>
-      <c r="S35" s="49"/>
-      <c r="T35" s="50"/>
+      <c r="S35" s="39"/>
+      <c r="T35" s="40"/>
       <c r="U35" s="23">
         <v>8</v>
       </c>
@@ -2923,8 +2978,8 @@
       </c>
     </row>
     <row r="36" spans="5:31" ht="20.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E36" s="49"/>
-      <c r="F36" s="50"/>
+      <c r="E36" s="39"/>
+      <c r="F36" s="40"/>
       <c r="G36" s="23">
         <v>8</v>
       </c>
@@ -2949,8 +3004,8 @@
       <c r="N36" s="5">
         <v>291</v>
       </c>
-      <c r="S36" s="49"/>
-      <c r="T36" s="50"/>
+      <c r="S36" s="39"/>
+      <c r="T36" s="40"/>
       <c r="U36" s="23">
         <v>8</v>
       </c>
@@ -2977,8 +3032,8 @@
       </c>
     </row>
     <row r="37" spans="5:31" ht="20.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E37" s="51"/>
-      <c r="F37" s="52"/>
+      <c r="E37" s="41"/>
+      <c r="F37" s="42"/>
       <c r="G37" s="25">
         <v>12</v>
       </c>
@@ -3004,8 +3059,8 @@
         <v>304</v>
       </c>
       <c r="Q37"/>
-      <c r="S37" s="51"/>
-      <c r="T37" s="52"/>
+      <c r="S37" s="41"/>
+      <c r="T37" s="42"/>
       <c r="U37" s="25">
         <v>12</v>
       </c>
@@ -3030,16 +3085,16 @@
       <c r="AB37" s="8">
         <v>304</v>
       </c>
-      <c r="AC37" s="82" t="s">
+      <c r="AC37" s="61" t="s">
         <v>48</v>
       </c>
-      <c r="AD37" s="83"/>
+      <c r="AD37" s="62"/>
     </row>
     <row r="38" spans="5:31" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E38" s="49" t="s">
+      <c r="E38" s="39" t="s">
         <v>47</v>
       </c>
-      <c r="F38" s="50"/>
+      <c r="F38" s="40"/>
       <c r="G38" s="24" t="s">
         <v>33</v>
       </c>
@@ -3071,10 +3126,10 @@
         <v>46</v>
       </c>
       <c r="Q38"/>
-      <c r="S38" s="49" t="s">
+      <c r="S38" s="39" t="s">
         <v>47</v>
       </c>
-      <c r="T38" s="50"/>
+      <c r="T38" s="40"/>
       <c r="U38" s="24" t="s">
         <v>33</v>
       </c>
@@ -3107,8 +3162,8 @@
       </c>
     </row>
     <row r="39" spans="5:31" x14ac:dyDescent="0.3">
-      <c r="E39" s="49"/>
-      <c r="F39" s="50"/>
+      <c r="E39" s="39"/>
+      <c r="F39" s="40"/>
       <c r="G39" s="23">
         <v>4</v>
       </c>
@@ -3142,8 +3197,8 @@
         <v>17.056856187290968</v>
       </c>
       <c r="Q39"/>
-      <c r="S39" s="49"/>
-      <c r="T39" s="50"/>
+      <c r="S39" s="39"/>
+      <c r="T39" s="40"/>
       <c r="U39" s="23">
         <v>4</v>
       </c>
@@ -3178,8 +3233,8 @@
       </c>
     </row>
     <row r="40" spans="5:31" x14ac:dyDescent="0.3">
-      <c r="E40" s="49"/>
-      <c r="F40" s="50"/>
+      <c r="E40" s="39"/>
+      <c r="F40" s="40"/>
       <c r="G40" s="23">
         <v>4</v>
       </c>
@@ -3213,8 +3268,8 @@
         <v>9.6440035016049013</v>
       </c>
       <c r="Q40"/>
-      <c r="S40" s="49"/>
-      <c r="T40" s="50"/>
+      <c r="S40" s="39"/>
+      <c r="T40" s="40"/>
       <c r="U40" s="23">
         <v>4</v>
       </c>
@@ -3249,8 +3304,8 @@
       </c>
     </row>
     <row r="41" spans="5:31" x14ac:dyDescent="0.3">
-      <c r="E41" s="49"/>
-      <c r="F41" s="50"/>
+      <c r="E41" s="39"/>
+      <c r="F41" s="40"/>
       <c r="G41" s="23">
         <v>4</v>
       </c>
@@ -3284,8 +3339,8 @@
         <v>9.1386861313868604</v>
       </c>
       <c r="Q41"/>
-      <c r="S41" s="49"/>
-      <c r="T41" s="50"/>
+      <c r="S41" s="39"/>
+      <c r="T41" s="40"/>
       <c r="U41" s="23">
         <v>4</v>
       </c>
@@ -3320,8 +3375,8 @@
       </c>
     </row>
     <row r="42" spans="5:31" x14ac:dyDescent="0.3">
-      <c r="E42" s="49"/>
-      <c r="F42" s="50"/>
+      <c r="E42" s="39"/>
+      <c r="F42" s="40"/>
       <c r="G42" s="23">
         <v>4</v>
       </c>
@@ -3354,8 +3409,8 @@
         <f t="shared" si="1"/>
         <v>0.54248248607867799</v>
       </c>
-      <c r="S42" s="49"/>
-      <c r="T42" s="50"/>
+      <c r="S42" s="39"/>
+      <c r="T42" s="40"/>
       <c r="U42" s="23">
         <v>4</v>
       </c>
@@ -3390,8 +3445,8 @@
       </c>
     </row>
     <row r="43" spans="5:31" x14ac:dyDescent="0.3">
-      <c r="E43" s="49"/>
-      <c r="F43" s="50"/>
+      <c r="E43" s="39"/>
+      <c r="F43" s="40"/>
       <c r="G43" s="23">
         <v>8</v>
       </c>
@@ -3424,8 +3479,8 @@
         <f t="shared" si="1"/>
         <v>0.28200185621474977</v>
       </c>
-      <c r="S43" s="49"/>
-      <c r="T43" s="50"/>
+      <c r="S43" s="39"/>
+      <c r="T43" s="40"/>
       <c r="U43" s="23">
         <v>8</v>
       </c>
@@ -3460,8 +3515,8 @@
       </c>
     </row>
     <row r="44" spans="5:31" x14ac:dyDescent="0.3">
-      <c r="E44" s="49"/>
-      <c r="F44" s="50"/>
+      <c r="E44" s="39"/>
+      <c r="F44" s="40"/>
       <c r="G44" s="23">
         <v>8</v>
       </c>
@@ -3494,8 +3549,8 @@
         <f t="shared" si="1"/>
         <v>-5.6277056277056277</v>
       </c>
-      <c r="S44" s="49"/>
-      <c r="T44" s="50"/>
+      <c r="S44" s="39"/>
+      <c r="T44" s="40"/>
       <c r="U44" s="23">
         <v>8</v>
       </c>
@@ -3530,8 +3585,8 @@
       </c>
     </row>
     <row r="45" spans="5:31" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E45" s="51"/>
-      <c r="F45" s="52"/>
+      <c r="E45" s="41"/>
+      <c r="F45" s="42"/>
       <c r="G45" s="25">
         <v>12</v>
       </c>
@@ -3564,8 +3619,8 @@
         <f t="shared" si="1"/>
         <v>-61.256930870796602</v>
       </c>
-      <c r="S45" s="51"/>
-      <c r="T45" s="52"/>
+      <c r="S45" s="41"/>
+      <c r="T45" s="42"/>
       <c r="U45" s="25">
         <v>12</v>
       </c>
@@ -3601,97 +3656,97 @@
     </row>
     <row r="47" spans="5:31" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="48" spans="5:31" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E48" s="38" t="s">
+      <c r="E48" s="52" t="s">
         <v>49</v>
       </c>
-      <c r="F48" s="39"/>
-      <c r="G48" s="39"/>
-      <c r="H48" s="39"/>
-      <c r="I48" s="39"/>
-      <c r="J48" s="39"/>
-      <c r="K48" s="40"/>
+      <c r="F48" s="53"/>
+      <c r="G48" s="53"/>
+      <c r="H48" s="53"/>
+      <c r="I48" s="53"/>
+      <c r="J48" s="53"/>
+      <c r="K48" s="54"/>
       <c r="L48"/>
       <c r="M48"/>
-      <c r="N48" s="38" t="s">
+      <c r="N48" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="O48" s="39"/>
-      <c r="P48" s="39"/>
-      <c r="Q48" s="39"/>
-      <c r="R48" s="39"/>
-      <c r="S48" s="39"/>
-      <c r="T48" s="40"/>
-      <c r="W48" s="91" t="s">
+      <c r="O48" s="53"/>
+      <c r="P48" s="53"/>
+      <c r="Q48" s="53"/>
+      <c r="R48" s="53"/>
+      <c r="S48" s="53"/>
+      <c r="T48" s="54"/>
+      <c r="W48" s="43" t="s">
         <v>57</v>
       </c>
-      <c r="X48" s="92"/>
-      <c r="Y48" s="92"/>
-      <c r="Z48" s="92"/>
-      <c r="AA48" s="92"/>
-      <c r="AB48" s="92"/>
-      <c r="AC48" s="92"/>
-      <c r="AD48" s="92"/>
-      <c r="AE48" s="93"/>
+      <c r="X48" s="44"/>
+      <c r="Y48" s="44"/>
+      <c r="Z48" s="44"/>
+      <c r="AA48" s="44"/>
+      <c r="AB48" s="44"/>
+      <c r="AC48" s="44"/>
+      <c r="AD48" s="44"/>
+      <c r="AE48" s="45"/>
     </row>
     <row r="49" spans="5:31" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E49" s="41"/>
-      <c r="F49" s="42"/>
-      <c r="G49" s="42"/>
-      <c r="H49" s="42"/>
-      <c r="I49" s="42"/>
-      <c r="J49" s="42"/>
-      <c r="K49" s="43"/>
+      <c r="E49" s="55"/>
+      <c r="F49" s="56"/>
+      <c r="G49" s="56"/>
+      <c r="H49" s="56"/>
+      <c r="I49" s="56"/>
+      <c r="J49" s="56"/>
+      <c r="K49" s="57"/>
       <c r="L49"/>
       <c r="M49"/>
-      <c r="N49" s="41"/>
-      <c r="O49" s="42"/>
-      <c r="P49" s="42"/>
-      <c r="Q49" s="42"/>
-      <c r="R49" s="42"/>
-      <c r="S49" s="42"/>
-      <c r="T49" s="43"/>
-      <c r="W49" s="87"/>
-      <c r="X49" s="88"/>
-      <c r="Y49" s="88"/>
-      <c r="Z49" s="88"/>
-      <c r="AA49" s="88"/>
-      <c r="AB49" s="88"/>
-      <c r="AC49" s="88"/>
-      <c r="AD49" s="88"/>
-      <c r="AE49" s="94"/>
+      <c r="N49" s="55"/>
+      <c r="O49" s="56"/>
+      <c r="P49" s="56"/>
+      <c r="Q49" s="56"/>
+      <c r="R49" s="56"/>
+      <c r="S49" s="56"/>
+      <c r="T49" s="57"/>
+      <c r="W49" s="46"/>
+      <c r="X49" s="47"/>
+      <c r="Y49" s="47"/>
+      <c r="Z49" s="47"/>
+      <c r="AA49" s="47"/>
+      <c r="AB49" s="47"/>
+      <c r="AC49" s="47"/>
+      <c r="AD49" s="47"/>
+      <c r="AE49" s="48"/>
     </row>
     <row r="50" spans="5:31" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E50" s="44"/>
-      <c r="F50" s="45"/>
-      <c r="G50" s="45"/>
-      <c r="H50" s="45"/>
-      <c r="I50" s="45"/>
-      <c r="J50" s="45"/>
-      <c r="K50" s="46"/>
+      <c r="E50" s="94"/>
+      <c r="F50" s="95"/>
+      <c r="G50" s="95"/>
+      <c r="H50" s="95"/>
+      <c r="I50" s="95"/>
+      <c r="J50" s="95"/>
+      <c r="K50" s="96"/>
       <c r="L50"/>
       <c r="M50"/>
-      <c r="N50" s="44"/>
-      <c r="O50" s="45"/>
-      <c r="P50" s="45"/>
-      <c r="Q50" s="45"/>
-      <c r="R50" s="45"/>
-      <c r="S50" s="45"/>
-      <c r="T50" s="46"/>
-      <c r="W50" s="89"/>
-      <c r="X50" s="90"/>
-      <c r="Y50" s="90"/>
-      <c r="Z50" s="90"/>
-      <c r="AA50" s="90"/>
-      <c r="AB50" s="90"/>
-      <c r="AC50" s="90"/>
-      <c r="AD50" s="90"/>
-      <c r="AE50" s="95"/>
+      <c r="N50" s="94"/>
+      <c r="O50" s="95"/>
+      <c r="P50" s="95"/>
+      <c r="Q50" s="95"/>
+      <c r="R50" s="95"/>
+      <c r="S50" s="95"/>
+      <c r="T50" s="96"/>
+      <c r="W50" s="49"/>
+      <c r="X50" s="50"/>
+      <c r="Y50" s="50"/>
+      <c r="Z50" s="50"/>
+      <c r="AA50" s="50"/>
+      <c r="AB50" s="50"/>
+      <c r="AC50" s="50"/>
+      <c r="AD50" s="50"/>
+      <c r="AE50" s="51"/>
     </row>
     <row r="51" spans="5:31" ht="20.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E51" s="47" t="s">
+      <c r="E51" s="37" t="s">
         <v>34</v>
       </c>
-      <c r="F51" s="48"/>
+      <c r="F51" s="38"/>
       <c r="G51" s="32" t="s">
         <v>33</v>
       </c>
@@ -3707,10 +3762,10 @@
       <c r="K51" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="N51" s="47" t="s">
+      <c r="N51" s="37" t="s">
         <v>52</v>
       </c>
-      <c r="O51" s="48"/>
+      <c r="O51" s="38"/>
       <c r="P51" s="32" t="s">
         <v>33</v>
       </c>
@@ -3726,10 +3781,10 @@
       <c r="T51" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="W51" s="47" t="s">
+      <c r="W51" s="37" t="s">
         <v>52</v>
       </c>
-      <c r="X51" s="48"/>
+      <c r="X51" s="38"/>
       <c r="Y51" s="32" t="s">
         <v>54</v>
       </c>
@@ -3753,8 +3808,8 @@
       </c>
     </row>
     <row r="52" spans="5:31" x14ac:dyDescent="0.3">
-      <c r="E52" s="49"/>
-      <c r="F52" s="50"/>
+      <c r="E52" s="39"/>
+      <c r="F52" s="40"/>
       <c r="G52" s="35">
         <v>2</v>
       </c>
@@ -3770,8 +3825,8 @@
       <c r="K52" s="28">
         <v>512</v>
       </c>
-      <c r="N52" s="49"/>
-      <c r="O52" s="50"/>
+      <c r="N52" s="39"/>
+      <c r="O52" s="40"/>
       <c r="P52" s="35">
         <v>2</v>
       </c>
@@ -3787,8 +3842,8 @@
       <c r="T52" s="28">
         <v>578</v>
       </c>
-      <c r="W52" s="49"/>
-      <c r="X52" s="50"/>
+      <c r="W52" s="39"/>
+      <c r="X52" s="40"/>
       <c r="Y52" s="35">
         <v>6</v>
       </c>
@@ -3812,8 +3867,8 @@
       </c>
     </row>
     <row r="53" spans="5:31" x14ac:dyDescent="0.3">
-      <c r="E53" s="49"/>
-      <c r="F53" s="50"/>
+      <c r="E53" s="39"/>
+      <c r="F53" s="40"/>
       <c r="G53" s="4">
         <v>2</v>
       </c>
@@ -3829,8 +3884,8 @@
       <c r="K53" s="5">
         <v>489</v>
       </c>
-      <c r="N53" s="49"/>
-      <c r="O53" s="50"/>
+      <c r="N53" s="39"/>
+      <c r="O53" s="40"/>
       <c r="P53" s="4">
         <v>2</v>
       </c>
@@ -3846,8 +3901,8 @@
       <c r="T53" s="5">
         <v>587</v>
       </c>
-      <c r="W53" s="49"/>
-      <c r="X53" s="50"/>
+      <c r="W53" s="39"/>
+      <c r="X53" s="40"/>
       <c r="Y53" s="4">
         <v>6</v>
       </c>
@@ -3871,8 +3926,8 @@
       </c>
     </row>
     <row r="54" spans="5:31" x14ac:dyDescent="0.3">
-      <c r="E54" s="49"/>
-      <c r="F54" s="50"/>
+      <c r="E54" s="39"/>
+      <c r="F54" s="40"/>
       <c r="G54" s="29">
         <v>4</v>
       </c>
@@ -3888,8 +3943,8 @@
       <c r="K54" s="5">
         <v>303</v>
       </c>
-      <c r="N54" s="49"/>
-      <c r="O54" s="50"/>
+      <c r="N54" s="39"/>
+      <c r="O54" s="40"/>
       <c r="P54" s="29">
         <v>4</v>
       </c>
@@ -3905,8 +3960,8 @@
       <c r="T54" s="5">
         <v>327</v>
       </c>
-      <c r="W54" s="49"/>
-      <c r="X54" s="50"/>
+      <c r="W54" s="39"/>
+      <c r="X54" s="40"/>
       <c r="Y54" s="29">
         <v>8</v>
       </c>
@@ -3930,8 +3985,8 @@
       </c>
     </row>
     <row r="55" spans="5:31" x14ac:dyDescent="0.3">
-      <c r="E55" s="49"/>
-      <c r="F55" s="50"/>
+      <c r="E55" s="39"/>
+      <c r="F55" s="40"/>
       <c r="G55" s="29">
         <v>4</v>
       </c>
@@ -3947,8 +4002,8 @@
       <c r="K55" s="5">
         <v>300</v>
       </c>
-      <c r="N55" s="49"/>
-      <c r="O55" s="50"/>
+      <c r="N55" s="39"/>
+      <c r="O55" s="40"/>
       <c r="P55" s="29">
         <v>4</v>
       </c>
@@ -3964,8 +4019,8 @@
       <c r="T55" s="5">
         <v>314</v>
       </c>
-      <c r="W55" s="49"/>
-      <c r="X55" s="50"/>
+      <c r="W55" s="39"/>
+      <c r="X55" s="40"/>
       <c r="Y55" s="29">
         <v>8</v>
       </c>
@@ -3989,8 +4044,8 @@
       </c>
     </row>
     <row r="56" spans="5:31" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E56" s="49"/>
-      <c r="F56" s="50"/>
+      <c r="E56" s="39"/>
+      <c r="F56" s="40"/>
       <c r="G56" s="29">
         <v>8</v>
       </c>
@@ -4006,8 +4061,8 @@
       <c r="K56" s="5">
         <v>329</v>
       </c>
-      <c r="N56" s="49"/>
-      <c r="O56" s="50"/>
+      <c r="N56" s="39"/>
+      <c r="O56" s="40"/>
       <c r="P56" s="29">
         <v>8</v>
       </c>
@@ -4023,8 +4078,8 @@
       <c r="T56" s="5">
         <v>543</v>
       </c>
-      <c r="W56" s="51"/>
-      <c r="X56" s="52"/>
+      <c r="W56" s="41"/>
+      <c r="X56" s="42"/>
       <c r="Y56" s="30">
         <v>8</v>
       </c>
@@ -4037,13 +4092,19 @@
       <c r="AB56" s="7">
         <v>8</v>
       </c>
-      <c r="AC56" s="7"/>
-      <c r="AD56" s="7"/>
-      <c r="AE56" s="8"/>
+      <c r="AC56" s="7">
+        <v>3225</v>
+      </c>
+      <c r="AD56" s="7">
+        <v>3064</v>
+      </c>
+      <c r="AE56" s="8">
+        <v>313</v>
+      </c>
     </row>
     <row r="57" spans="5:31" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E57" s="51"/>
-      <c r="F57" s="52"/>
+      <c r="E57" s="41"/>
+      <c r="F57" s="42"/>
       <c r="G57" s="30">
         <v>8</v>
       </c>
@@ -4059,8 +4120,8 @@
       <c r="K57" s="8">
         <v>329</v>
       </c>
-      <c r="N57" s="51"/>
-      <c r="O57" s="52"/>
+      <c r="N57" s="41"/>
+      <c r="O57" s="42"/>
       <c r="P57" s="30">
         <v>8</v>
       </c>
@@ -4087,10 +4148,10 @@
       <c r="AE57"/>
     </row>
     <row r="58" spans="5:31" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E58" s="47" t="s">
+      <c r="E58" s="37" t="s">
         <v>50</v>
       </c>
-      <c r="F58" s="48"/>
+      <c r="F58" s="38"/>
       <c r="G58" s="32" t="s">
         <v>33</v>
       </c>
@@ -4106,10 +4167,10 @@
       <c r="K58" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="N58" s="47" t="s">
+      <c r="N58" s="37" t="s">
         <v>53</v>
       </c>
-      <c r="O58" s="48"/>
+      <c r="O58" s="38"/>
       <c r="P58" s="32" t="s">
         <v>33</v>
       </c>
@@ -4126,9 +4187,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="59" spans="5:31" x14ac:dyDescent="0.3">
-      <c r="E59" s="49"/>
-      <c r="F59" s="50"/>
+    <row r="59" spans="5:31" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E59" s="39"/>
+      <c r="F59" s="40"/>
       <c r="G59" s="21">
         <v>2</v>
       </c>
@@ -4144,8 +4205,8 @@
       <c r="K59" s="22">
         <v>492</v>
       </c>
-      <c r="N59" s="49"/>
-      <c r="O59" s="50"/>
+      <c r="N59" s="39"/>
+      <c r="O59" s="40"/>
       <c r="P59" s="35">
         <v>2</v>
       </c>
@@ -4162,9 +4223,9 @@
         <v>629</v>
       </c>
     </row>
-    <row r="60" spans="5:31" x14ac:dyDescent="0.3">
-      <c r="E60" s="49"/>
-      <c r="F60" s="50"/>
+    <row r="60" spans="5:31" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E60" s="39"/>
+      <c r="F60" s="40"/>
       <c r="G60" s="4">
         <v>2</v>
       </c>
@@ -4180,8 +4241,8 @@
       <c r="K60" s="5">
         <v>489</v>
       </c>
-      <c r="N60" s="49"/>
-      <c r="O60" s="50"/>
+      <c r="N60" s="39"/>
+      <c r="O60" s="40"/>
       <c r="P60" s="4">
         <v>2</v>
       </c>
@@ -4197,10 +4258,21 @@
       <c r="T60" s="5">
         <v>605</v>
       </c>
+      <c r="W60" s="43" t="s">
+        <v>58</v>
+      </c>
+      <c r="X60" s="44"/>
+      <c r="Y60" s="44"/>
+      <c r="Z60" s="44"/>
+      <c r="AA60" s="44"/>
+      <c r="AB60" s="44"/>
+      <c r="AC60" s="44"/>
+      <c r="AD60" s="45"/>
+      <c r="AE60"/>
     </row>
     <row r="61" spans="5:31" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E61" s="49"/>
-      <c r="F61" s="50"/>
+      <c r="E61" s="39"/>
+      <c r="F61" s="40"/>
       <c r="G61" s="31">
         <v>4</v>
       </c>
@@ -4216,8 +4288,8 @@
       <c r="K61" s="28">
         <v>307</v>
       </c>
-      <c r="N61" s="49"/>
-      <c r="O61" s="50"/>
+      <c r="N61" s="39"/>
+      <c r="O61" s="40"/>
       <c r="P61" s="29">
         <v>4</v>
       </c>
@@ -4233,10 +4305,19 @@
       <c r="T61" s="5">
         <v>322</v>
       </c>
-    </row>
-    <row r="62" spans="5:31" x14ac:dyDescent="0.3">
-      <c r="E62" s="49"/>
-      <c r="F62" s="50"/>
+      <c r="W61" s="46"/>
+      <c r="X61" s="100"/>
+      <c r="Y61" s="100"/>
+      <c r="Z61" s="100"/>
+      <c r="AA61" s="100"/>
+      <c r="AB61" s="100"/>
+      <c r="AC61" s="100"/>
+      <c r="AD61" s="48"/>
+      <c r="AE61"/>
+    </row>
+    <row r="62" spans="5:31" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E62" s="39"/>
+      <c r="F62" s="40"/>
       <c r="G62" s="29">
         <v>4</v>
       </c>
@@ -4252,8 +4333,8 @@
       <c r="K62" s="5">
         <v>298</v>
       </c>
-      <c r="N62" s="49"/>
-      <c r="O62" s="50"/>
+      <c r="N62" s="39"/>
+      <c r="O62" s="40"/>
       <c r="P62" s="29">
         <v>4</v>
       </c>
@@ -4269,10 +4350,19 @@
       <c r="T62" s="5">
         <v>318</v>
       </c>
-    </row>
-    <row r="63" spans="5:31" x14ac:dyDescent="0.3">
-      <c r="E63" s="49"/>
-      <c r="F63" s="50"/>
+      <c r="W62" s="49"/>
+      <c r="X62" s="50"/>
+      <c r="Y62" s="50"/>
+      <c r="Z62" s="50"/>
+      <c r="AA62" s="50"/>
+      <c r="AB62" s="50"/>
+      <c r="AC62" s="50"/>
+      <c r="AD62" s="51"/>
+      <c r="AE62"/>
+    </row>
+    <row r="63" spans="5:31" ht="21" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E63" s="39"/>
+      <c r="F63" s="40"/>
       <c r="G63" s="29">
         <v>8</v>
       </c>
@@ -4288,8 +4378,8 @@
       <c r="K63" s="5">
         <v>357</v>
       </c>
-      <c r="N63" s="49"/>
-      <c r="O63" s="50"/>
+      <c r="N63" s="39"/>
+      <c r="O63" s="40"/>
       <c r="P63" s="29">
         <v>8</v>
       </c>
@@ -4305,10 +4395,32 @@
       <c r="T63" s="5">
         <v>510</v>
       </c>
+      <c r="W63" s="39" t="s">
+        <v>59</v>
+      </c>
+      <c r="X63" s="40"/>
+      <c r="Y63" s="32" t="s">
+        <v>33</v>
+      </c>
+      <c r="Z63" s="32" t="s">
+        <v>54</v>
+      </c>
+      <c r="AA63" s="33" t="s">
+        <v>0</v>
+      </c>
+      <c r="AB63" s="33" t="s">
+        <v>1</v>
+      </c>
+      <c r="AC63" s="97" t="s">
+        <v>2</v>
+      </c>
+      <c r="AD63" s="34" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="64" spans="5:31" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E64" s="51"/>
-      <c r="F64" s="52"/>
+      <c r="E64" s="41"/>
+      <c r="F64" s="42"/>
       <c r="G64" s="30">
         <v>8</v>
       </c>
@@ -4324,8 +4436,8 @@
       <c r="K64" s="8">
         <v>341</v>
       </c>
-      <c r="N64" s="51"/>
-      <c r="O64" s="52"/>
+      <c r="N64" s="41"/>
+      <c r="O64" s="42"/>
       <c r="P64" s="30">
         <v>8</v>
       </c>
@@ -4341,48 +4453,150 @@
       <c r="T64" s="8">
         <v>409</v>
       </c>
+      <c r="W64" s="39"/>
+      <c r="X64" s="40"/>
+      <c r="Y64" s="35">
+        <v>2</v>
+      </c>
+      <c r="Z64" s="27">
+        <v>6</v>
+      </c>
+      <c r="AA64" s="27">
+        <v>18809</v>
+      </c>
+      <c r="AB64" s="27">
+        <v>17887</v>
+      </c>
+      <c r="AC64" s="98">
+        <v>417</v>
+      </c>
+      <c r="AD64" s="28">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="65" spans="23:30" x14ac:dyDescent="0.3">
+      <c r="W65" s="39"/>
+      <c r="X65" s="40"/>
+      <c r="Y65" s="4"/>
+      <c r="Z65" s="2"/>
+      <c r="AA65" s="2"/>
+      <c r="AB65" s="2"/>
+      <c r="AC65" s="36"/>
+      <c r="AD65" s="5"/>
+    </row>
+    <row r="66" spans="23:30" x14ac:dyDescent="0.3">
+      <c r="W66" s="39"/>
+      <c r="X66" s="40"/>
+      <c r="Y66" s="29"/>
+      <c r="Z66" s="2"/>
+      <c r="AA66" s="2"/>
+      <c r="AB66" s="2"/>
+      <c r="AC66" s="36"/>
+      <c r="AD66" s="5"/>
+    </row>
+    <row r="67" spans="23:30" x14ac:dyDescent="0.3">
+      <c r="W67" s="39"/>
+      <c r="X67" s="40"/>
+      <c r="Y67" s="29"/>
+      <c r="Z67" s="2"/>
+      <c r="AA67" s="2"/>
+      <c r="AB67" s="2"/>
+      <c r="AC67" s="36"/>
+      <c r="AD67" s="5"/>
+    </row>
+    <row r="68" spans="23:30" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="W68" s="41"/>
+      <c r="X68" s="42"/>
+      <c r="Y68" s="30"/>
+      <c r="Z68" s="7"/>
+      <c r="AA68" s="7"/>
+      <c r="AB68" s="7"/>
+      <c r="AC68" s="99"/>
+      <c r="AD68" s="8"/>
+    </row>
+    <row r="69" spans="23:30" ht="21" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="W69" s="39" t="s">
+        <v>61</v>
+      </c>
+      <c r="X69" s="40"/>
+      <c r="Y69" s="32" t="s">
+        <v>33</v>
+      </c>
+      <c r="Z69" s="32" t="s">
+        <v>54</v>
+      </c>
+      <c r="AA69" s="33" t="s">
+        <v>0</v>
+      </c>
+      <c r="AB69" s="33" t="s">
+        <v>1</v>
+      </c>
+      <c r="AC69" s="97" t="s">
+        <v>2</v>
+      </c>
+      <c r="AD69" s="34" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="70" spans="23:30" x14ac:dyDescent="0.3">
+      <c r="W70" s="39"/>
+      <c r="X70" s="40"/>
+      <c r="Y70" s="35">
+        <v>2</v>
+      </c>
+      <c r="Z70" s="27">
+        <v>6</v>
+      </c>
+      <c r="AA70" s="27"/>
+      <c r="AB70" s="27"/>
+      <c r="AC70" s="98"/>
+      <c r="AD70" s="28"/>
+    </row>
+    <row r="71" spans="23:30" x14ac:dyDescent="0.3">
+      <c r="W71" s="39"/>
+      <c r="X71" s="40"/>
+      <c r="Y71" s="4"/>
+      <c r="Z71" s="2"/>
+      <c r="AA71" s="2"/>
+      <c r="AB71" s="2"/>
+      <c r="AC71" s="36"/>
+      <c r="AD71" s="5"/>
+    </row>
+    <row r="72" spans="23:30" x14ac:dyDescent="0.3">
+      <c r="W72" s="39"/>
+      <c r="X72" s="40"/>
+      <c r="Y72" s="29"/>
+      <c r="Z72" s="2"/>
+      <c r="AA72" s="2"/>
+      <c r="AB72" s="2"/>
+      <c r="AC72" s="36"/>
+      <c r="AD72" s="5"/>
+    </row>
+    <row r="73" spans="23:30" x14ac:dyDescent="0.3">
+      <c r="W73" s="39"/>
+      <c r="X73" s="40"/>
+      <c r="Y73" s="29"/>
+      <c r="Z73" s="2"/>
+      <c r="AA73" s="2"/>
+      <c r="AB73" s="2"/>
+      <c r="AC73" s="36"/>
+      <c r="AD73" s="5"/>
+    </row>
+    <row r="74" spans="23:30" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="W74" s="41"/>
+      <c r="X74" s="42"/>
+      <c r="Y74" s="30"/>
+      <c r="Z74" s="7"/>
+      <c r="AA74" s="7"/>
+      <c r="AB74" s="7"/>
+      <c r="AC74" s="99"/>
+      <c r="AD74" s="8"/>
     </row>
   </sheetData>
-  <mergeCells count="55">
-    <mergeCell ref="W51:X56"/>
-    <mergeCell ref="W48:AE50"/>
-    <mergeCell ref="S38:T45"/>
-    <mergeCell ref="E38:F45"/>
-    <mergeCell ref="E30:F37"/>
-    <mergeCell ref="E27:N29"/>
-    <mergeCell ref="AC37:AD37"/>
-    <mergeCell ref="AA18:AC20"/>
-    <mergeCell ref="X21:Y24"/>
-    <mergeCell ref="AH18:AJ20"/>
-    <mergeCell ref="AE21:AF24"/>
-    <mergeCell ref="S27:AB29"/>
-    <mergeCell ref="S30:T37"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="F1:I1"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="H4:J6"/>
-    <mergeCell ref="H3:J3"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="D4:G6"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="AC3:AE3"/>
-    <mergeCell ref="AC4:AE6"/>
-    <mergeCell ref="Z3:AB3"/>
-    <mergeCell ref="Z4:AB6"/>
-    <mergeCell ref="W4:Y6"/>
-    <mergeCell ref="Q3:S3"/>
-    <mergeCell ref="W3:Y3"/>
-    <mergeCell ref="N3:P3"/>
-    <mergeCell ref="H11:P11"/>
-    <mergeCell ref="K3:M3"/>
-    <mergeCell ref="T3:V3"/>
-    <mergeCell ref="T4:V6"/>
-    <mergeCell ref="Q4:S6"/>
-    <mergeCell ref="K4:M6"/>
-    <mergeCell ref="N4:P6"/>
+  <mergeCells count="58">
+    <mergeCell ref="W63:X68"/>
+    <mergeCell ref="W60:AD62"/>
+    <mergeCell ref="W69:X74"/>
     <mergeCell ref="D10:E10"/>
     <mergeCell ref="F10:G10"/>
     <mergeCell ref="N48:T50"/>
@@ -4399,6 +4613,45 @@
     <mergeCell ref="E48:K50"/>
     <mergeCell ref="E51:F57"/>
     <mergeCell ref="E58:F64"/>
+    <mergeCell ref="Q3:S3"/>
+    <mergeCell ref="W3:Y3"/>
+    <mergeCell ref="N3:P3"/>
+    <mergeCell ref="H11:P11"/>
+    <mergeCell ref="K3:M3"/>
+    <mergeCell ref="T3:V3"/>
+    <mergeCell ref="T4:V6"/>
+    <mergeCell ref="Q4:S6"/>
+    <mergeCell ref="K4:M6"/>
+    <mergeCell ref="N4:P6"/>
+    <mergeCell ref="AC3:AE3"/>
+    <mergeCell ref="AC4:AE6"/>
+    <mergeCell ref="Z3:AB3"/>
+    <mergeCell ref="Z4:AB6"/>
+    <mergeCell ref="W4:Y6"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="F1:I1"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="H4:J6"/>
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="D4:G6"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="E27:N29"/>
+    <mergeCell ref="AC37:AD37"/>
+    <mergeCell ref="AA18:AC20"/>
+    <mergeCell ref="X21:Y24"/>
+    <mergeCell ref="AH18:AJ20"/>
+    <mergeCell ref="AE21:AF24"/>
+    <mergeCell ref="S27:AB29"/>
+    <mergeCell ref="S30:T37"/>
+    <mergeCell ref="W51:X56"/>
+    <mergeCell ref="W48:AE50"/>
+    <mergeCell ref="S38:T45"/>
+    <mergeCell ref="E38:F45"/>
+    <mergeCell ref="E30:F37"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>